<commit_message>
docs: fix user flow master structure
</commit_message>
<xml_diff>
--- a/docs/product/user-flow/user-flow-master.xlsx
+++ b/docs/product/user-flow/user-flow-master.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="R667c5249c3d0433f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_利用動線" sheetId="2" r:id="R57118db70efd4fd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定同意" sheetId="3" r:id="R9f59800e1eee442d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ケース一覧" sheetId="4" r:id="R0cb167197a4b4a9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_運営チェック" sheetId="5" r:id="R2f46c07db1304b17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_実装対応" sheetId="6" r:id="R818638a8c8814737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="R58243710d7024acd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_利用動線" sheetId="2" r:id="R86e095bca6d244cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定同意" sheetId="3" r:id="R3c0f70032b4141c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ケース一覧" sheetId="4" r:id="R44fd16095399437f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_運営チェック" sheetId="5" r:id="R3836304b6ca64cfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_実装対応" sheetId="6" r:id="Rec3e7c3b368e43a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -82,7 +82,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -119,6 +119,16 @@
         <x:fgColor rgb="FFEEF4F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF315B5B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF4F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -141,7 +151,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="44">
+  <x:cellXfs count="51">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -232,11 +242,58 @@
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="6">
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:color rgb="FF8A5A00"/>
@@ -491,13 +548,13 @@
       <x:c r="C3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="37" t="str">
+      <x:c r="A4" s="47" t="str">
         <x:v>シート</x:v>
       </x:c>
-      <x:c r="B4" s="37" t="str">
+      <x:c r="B4" s="47" t="str">
         <x:v>役割</x:v>
       </x:c>
-      <x:c r="C4" s="37" t="str">
+      <x:c r="C4" s="47" t="str">
         <x:v>ポイント</x:v>
       </x:c>
     </x:row>
@@ -562,13 +619,13 @@
       <x:c r="C10" s="41"/>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
-      <x:c r="A11" s="42" t="str">
+      <x:c r="A11" s="50" t="str">
         <x:v>更新ルール</x:v>
       </x:c>
-      <x:c r="B11" s="42" t="str">
+      <x:c r="B11" s="50" t="str">
         <x:v>同名ファイルを更新</x:v>
       </x:c>
-      <x:c r="C11" s="42" t="str">
+      <x:c r="C11" s="50" t="str">
         <x:v>別バージョンのExcelを増やさず、変更理由と履歴はGitで管理する。</x:v>
       </x:c>
     </x:row>
@@ -694,76 +751,76 @@
       <x:c r="X3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="37" t="str">
+      <x:c r="A4" s="47" t="str">
         <x:v>Flow ID</x:v>
       </x:c>
-      <x:c r="B4" s="37" t="str">
+      <x:c r="B4" s="47" t="str">
         <x:v>Case</x:v>
       </x:c>
-      <x:c r="C4" s="37" t="str">
+      <x:c r="C4" s="47" t="str">
         <x:v>Subcase</x:v>
       </x:c>
-      <x:c r="D4" s="37" t="str">
+      <x:c r="D4" s="47" t="str">
         <x:v>Step</x:v>
       </x:c>
-      <x:c r="E4" s="37" t="str">
+      <x:c r="E4" s="47" t="str">
         <x:v>ユーザー行動</x:v>
       </x:c>
-      <x:c r="F4" s="37" t="str">
-        <x:v>次に見せること</x:v>
-      </x:c>
-      <x:c r="G4" s="37" t="str">
+      <x:c r="F4" s="47" t="str">
+        <x:v>ユーザーへの説明</x:v>
+      </x:c>
+      <x:c r="G4" s="47" t="str">
         <x:v>利用中Account</x:v>
       </x:c>
-      <x:c r="H4" s="37" t="str">
-        <x:v>操作者</x:v>
-      </x:c>
-      <x:c r="I4" s="37" t="str">
-        <x:v>語る人</x:v>
-      </x:c>
-      <x:c r="J4" s="37" t="str">
+      <x:c r="H4" s="47" t="str">
+        <x:v>このStepの操作者</x:v>
+      </x:c>
+      <x:c r="I4" s="47" t="str">
+        <x:v>このStepで語る人</x:v>
+      </x:c>
+      <x:c r="J4" s="47" t="str">
         <x:v>Person</x:v>
       </x:c>
-      <x:c r="K4" s="37" t="str">
+      <x:c r="K4" s="47" t="str">
         <x:v>Payer</x:v>
       </x:c>
-      <x:c r="L4" s="37" t="str">
+      <x:c r="L4" s="47" t="str">
         <x:v>Supporter</x:v>
       </x:c>
-      <x:c r="M4" s="37" t="str">
+      <x:c r="M4" s="47" t="str">
         <x:v>Device</x:v>
       </x:c>
-      <x:c r="N4" s="37" t="str">
+      <x:c r="N4" s="47" t="str">
         <x:v>現在状態</x:v>
       </x:c>
-      <x:c r="O4" s="37" t="str">
+      <x:c r="O4" s="47" t="str">
         <x:v>分岐条件</x:v>
       </x:c>
-      <x:c r="P4" s="37" t="str">
+      <x:c r="P4" s="47" t="str">
         <x:v>次の状態</x:v>
       </x:c>
-      <x:c r="Q4" s="37" t="str">
+      <x:c r="Q4" s="47" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="R4" s="37" t="str">
+      <x:c r="R4" s="47" t="str">
         <x:v>購入</x:v>
       </x:c>
-      <x:c r="S4" s="37" t="str">
+      <x:c r="S4" s="47" t="str">
         <x:v>本人認証</x:v>
       </x:c>
-      <x:c r="T4" s="37" t="str">
+      <x:c r="T4" s="47" t="str">
         <x:v>設定・同意</x:v>
       </x:c>
-      <x:c r="U4" s="37" t="str">
+      <x:c r="U4" s="47" t="str">
         <x:v>内容共有</x:v>
       </x:c>
-      <x:c r="V4" s="37" t="str">
+      <x:c r="V4" s="47" t="str">
         <x:v>進捗共有</x:v>
       </x:c>
-      <x:c r="W4" s="37" t="str">
+      <x:c r="W4" s="47" t="str">
         <x:v>内部メモ</x:v>
       </x:c>
-      <x:c r="X4" s="37" t="str">
+      <x:c r="X4" s="47" t="str">
         <x:v>確定度</x:v>
       </x:c>
     </x:row>
@@ -784,7 +841,7 @@
         <x:v>HP→無料3問→自分の物語</x:v>
       </x:c>
       <x:c r="F5" s="40" t="str">
-        <x:v>Account登録</x:v>
+        <x:v>まず3問、無料で試せます。3問後に続けるか決められます。</x:v>
       </x:c>
       <x:c r="G5" s="40" t="str">
         <x:v>なし</x:v>
@@ -858,7 +915,7 @@
         <x:v>Account登録→幼い頃の3問を語る</x:v>
       </x:c>
       <x:c r="F6" s="40" t="str">
-        <x:v>3問後に内容・料金</x:v>
+        <x:v>ここまで無料です。続ける場合は内容と料金をご確認ください。</x:v>
       </x:c>
       <x:c r="G6" s="40" t="str">
         <x:v>本人</x:v>
@@ -932,7 +989,7 @@
         <x:v>本人が購入</x:v>
       </x:c>
       <x:c r="F7" s="40" t="str">
-        <x:v>はじまりの章</x:v>
+        <x:v>購入後、「はじまりの章」から本編を始められます。</x:v>
       </x:c>
       <x:c r="G7" s="40" t="str">
         <x:v>本人</x:v>
@@ -1006,7 +1063,7 @@
         <x:v>はじまりの章→本編をはじめる</x:v>
       </x:c>
       <x:c r="F8" s="40" t="str">
-        <x:v>9テーマ</x:v>
+        <x:v>本編を開始すると、9つのテーマを順番に辿れます。</x:v>
       </x:c>
       <x:c r="G8" s="40" t="str">
         <x:v>本人</x:v>
@@ -1080,7 +1137,7 @@
         <x:v>HP→内容・料金→縦糸横糸をはじめる</x:v>
       </x:c>
       <x:c r="F9" s="40" t="str">
-        <x:v>Account登録→購入</x:v>
+        <x:v>無料体験をせず、そのまま購入して始められます。</x:v>
       </x:c>
       <x:c r="G9" s="40" t="str">
         <x:v>なし→本人</x:v>
@@ -1154,7 +1211,7 @@
         <x:v>はじまりの章→本編をはじめる</x:v>
       </x:c>
       <x:c r="F10" s="40" t="str">
-        <x:v>9テーマ</x:v>
+        <x:v>本編を開始すると、9つのテーマを順番に辿れます。</x:v>
       </x:c>
       <x:c r="G10" s="40" t="str">
         <x:v>本人</x:v>
@@ -1228,7 +1285,7 @@
         <x:v>HP→大切な人の物語→一緒に試す</x:v>
       </x:c>
       <x:c r="F11" s="40" t="str">
-        <x:v>子Account登録</x:v>
+        <x:v>このスマホで一緒に3問試せます。続ける場合は、あとから本人のスマホでも使えます。</x:v>
       </x:c>
       <x:c r="G11" s="40" t="str">
         <x:v>なし</x:v>
@@ -1302,7 +1359,7 @@
         <x:v>子Accountで親の姓名を登録</x:v>
       </x:c>
       <x:c r="F12" s="40" t="str">
-        <x:v>この端末で3問</x:v>
+        <x:v>語る方のお名前を登録し、このスマホで3問を始めます。</x:v>
       </x:c>
       <x:c r="G12" s="40" t="str">
         <x:v>子</x:v>
@@ -1376,7 +1433,7 @@
         <x:v>子端末で母が3問を語る</x:v>
       </x:c>
       <x:c r="F13" s="40" t="str">
-        <x:v>購入して続ける／今回はここまで</x:v>
+        <x:v>3問のあと、購入して続けるか、今回はここまでにするか選べます。</x:v>
       </x:c>
       <x:c r="G13" s="40" t="str">
         <x:v>子</x:v>
@@ -1450,7 +1507,7 @@
         <x:v>子が購入して贈る</x:v>
       </x:c>
       <x:c r="F14" s="40" t="str">
-        <x:v>母のスマホへ接続案内</x:v>
+        <x:v>購入後、本人のスマホへ続きを始める案内を送れます。</x:v>
       </x:c>
       <x:c r="G14" s="40" t="str">
         <x:v>子</x:v>
@@ -1524,7 +1581,7 @@
         <x:v>母：LINE等の案内→SMS OTP→既存Personへ接続</x:v>
       </x:c>
       <x:c r="F15" s="40" t="str">
-        <x:v>同じ3問の続き</x:v>
+        <x:v>本人確認後、同じ3問の続きから利用できます。</x:v>
       </x:c>
       <x:c r="G15" s="40" t="str">
         <x:v>母</x:v>
@@ -1598,7 +1655,7 @@
         <x:v>母：はじまりの章→本編をはじめる</x:v>
       </x:c>
       <x:c r="F16" s="40" t="str">
-        <x:v>一人でも一緒でも続ける</x:v>
+        <x:v>本人は一人でも、ご家族と一緒でも続けられます。</x:v>
       </x:c>
       <x:c r="G16" s="40" t="str">
         <x:v>母</x:v>
@@ -1672,7 +1729,7 @@
         <x:v>HP→大切な人の物語→本人に送る</x:v>
       </x:c>
       <x:c r="F17" s="40" t="str">
-        <x:v>子Account登録</x:v>
+        <x:v>LINEなどで3問を送り、本人の返答後に購入を決められます。</x:v>
       </x:c>
       <x:c r="G17" s="40" t="str">
         <x:v>なし</x:v>
@@ -1746,7 +1803,7 @@
         <x:v>子Accountで親Personを作り招待を送る</x:v>
       </x:c>
       <x:c r="F18" s="40" t="str">
-        <x:v>親の3問完了を待つ</x:v>
+        <x:v>送信後は、本人が3問を終えるまでお待ちください。</x:v>
       </x:c>
       <x:c r="G18" s="40" t="str">
         <x:v>子</x:v>
@@ -1820,7 +1877,7 @@
         <x:v>親：招待リンクを開いて3問を語る</x:v>
       </x:c>
       <x:c r="F19" s="40" t="str">
-        <x:v>続けたい／今回はここまで</x:v>
+        <x:v>この3問は無料です。Account登録をせずに体験できます。</x:v>
       </x:c>
       <x:c r="G19" s="40" t="str">
         <x:v>なし（体験リンク）</x:v>
@@ -1894,7 +1951,7 @@
         <x:v>親：続きをやってみたい／今回はここまでを選ぶ</x:v>
       </x:c>
       <x:c r="F20" s="40" t="str">
-        <x:v>続行希望時だけ子へ通知</x:v>
+        <x:v>続けたい場合だけご家族に知らせます。今回はここまででも構いません。</x:v>
       </x:c>
       <x:c r="G20" s="40" t="str">
         <x:v>なし（体験リンク）</x:v>
@@ -1968,7 +2025,7 @@
         <x:v>子：続行希望の通知→購入して贈る</x:v>
       </x:c>
       <x:c r="F21" s="40" t="str">
-        <x:v>注文内容確認</x:v>
+        <x:v>本人が続けたいと答えた後、ご家族が購入して贈れます。</x:v>
       </x:c>
       <x:c r="G21" s="40" t="str">
         <x:v>子</x:v>
@@ -2042,7 +2099,7 @@
         <x:v>親：SMS OTP→既存Personへ接続</x:v>
       </x:c>
       <x:c r="F22" s="40" t="str">
-        <x:v>同じ3問の続き</x:v>
+        <x:v>本人確認後、同じ3問の続きから利用できます。</x:v>
       </x:c>
       <x:c r="G22" s="40" t="str">
         <x:v>親</x:v>
@@ -2116,7 +2173,7 @@
         <x:v>子：購入を本人にお願いする</x:v>
       </x:c>
       <x:c r="F23" s="40" t="str">
-        <x:v>親へ本人購入の案内</x:v>
+        <x:v>本人へ購入案内を送り、ご本人に手続きをお願いできます。</x:v>
       </x:c>
       <x:c r="G23" s="40" t="str">
         <x:v>子</x:v>
@@ -2190,7 +2247,7 @@
         <x:v>親：本人Accountへ接続して購入</x:v>
       </x:c>
       <x:c r="F24" s="40" t="str">
-        <x:v>はじまりの章</x:v>
+        <x:v>本人確認と購入後、「はじまりの章」へ進みます。</x:v>
       </x:c>
       <x:c r="G24" s="40" t="str">
         <x:v>親（購入時接続）</x:v>
@@ -2264,7 +2321,7 @@
         <x:v>親：はじまりの章→本編をはじめる</x:v>
       </x:c>
       <x:c r="F25" s="40" t="str">
-        <x:v>9テーマ</x:v>
+        <x:v>本編を開始すると、9つのテーマを順番に辿れます。</x:v>
       </x:c>
       <x:c r="G25" s="40" t="str">
         <x:v>親</x:v>
@@ -2323,7 +2380,7 @@
     </x:row>
     <x:row r="26" ht="54" customHeight="1">
       <x:c r="A26" s="43" t="str">
-        <x:v>B-DIRECT-010</x:v>
+        <x:v>B-DIRECT-GIFT-010</x:v>
       </x:c>
       <x:c r="B26" s="40" t="str">
         <x:v>B 家族起点</x:v>
@@ -2338,7 +2395,7 @@
         <x:v>HP→親に贈る→子が購入</x:v>
       </x:c>
       <x:c r="F26" s="40" t="str">
-        <x:v>親のスマホへ接続案内</x:v>
+        <x:v>無料体験をせずに購入し、本人へ開始案内を送れます。</x:v>
       </x:c>
       <x:c r="G26" s="40" t="str">
         <x:v>子</x:v>
@@ -2397,7 +2454,7 @@
     </x:row>
     <x:row r="27" ht="54" customHeight="1">
       <x:c r="A27" s="43" t="str">
-        <x:v>B-DIRECT-020</x:v>
+        <x:v>B-DIRECT-GIFT-020</x:v>
       </x:c>
       <x:c r="B27" s="40" t="str">
         <x:v>B 家族起点</x:v>
@@ -2412,7 +2469,7 @@
         <x:v>親：案内→SMS OTP→既存Personへ接続</x:v>
       </x:c>
       <x:c r="F27" s="40" t="str">
-        <x:v>はじまりの章</x:v>
+        <x:v>本人確認後、「はじまりの章」から始められます。</x:v>
       </x:c>
       <x:c r="G27" s="40" t="str">
         <x:v>親</x:v>
@@ -2471,7 +2528,7 @@
     </x:row>
     <x:row r="28" ht="54" customHeight="1">
       <x:c r="A28" s="43" t="str">
-        <x:v>B-DIRECT-030</x:v>
+        <x:v>B-DIRECT-GIFT-030</x:v>
       </x:c>
       <x:c r="B28" s="40" t="str">
         <x:v>B 家族起点</x:v>
@@ -2486,7 +2543,7 @@
         <x:v>親：はじまりの章→本編をはじめる</x:v>
       </x:c>
       <x:c r="F28" s="40" t="str">
-        <x:v>9テーマ</x:v>
+        <x:v>本人は一人でも、ご家族と一緒でも続けられます。</x:v>
       </x:c>
       <x:c r="G28" s="40" t="str">
         <x:v>親</x:v>
@@ -2550,6 +2607,9 @@
   </x:mergeCells>
   <x:conditionalFormatting sqref="A5:X28">
     <x:cfRule type="expression" dxfId="0" priority="1">
+      <x:formula>$X5="要確認"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="3" priority="2">
       <x:formula>$X5="要確認"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -2568,14 +2628,16 @@
   <x:cols>
     <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="34" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -2591,6 +2653,8 @@
       <x:c r="H1" s="28"/>
       <x:c r="I1" s="28"/>
       <x:c r="J1" s="28"/>
+      <x:c r="K1" s="28"/>
+      <x:c r="L1" s="28"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="30" t="str">
@@ -2605,6 +2669,8 @@
       <x:c r="H2" s="30"/>
       <x:c r="I2" s="30"/>
       <x:c r="J2" s="30"/>
+      <x:c r="K2" s="30"/>
+      <x:c r="L2" s="30"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3"/>
@@ -2617,40 +2683,48 @@
       <x:c r="H3"/>
       <x:c r="I3"/>
       <x:c r="J3"/>
+      <x:c r="K3"/>
+      <x:c r="L3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="37" t="str">
+      <x:c r="A4" s="47" t="str">
         <x:v>Setting ID</x:v>
       </x:c>
-      <x:c r="B4" s="37" t="str">
+      <x:c r="B4" s="47" t="str">
         <x:v>設定・同意</x:v>
       </x:c>
-      <x:c r="C4" s="37" t="str">
+      <x:c r="C4" s="47" t="str">
         <x:v>Account登録</x:v>
       </x:c>
-      <x:c r="D4" s="37" t="str">
+      <x:c r="D4" s="47" t="str">
+        <x:v>対象Person作成</x:v>
+      </x:c>
+      <x:c r="E4" s="47" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="E4" s="37" t="str">
+      <x:c r="F4" s="47" t="str">
         <x:v>購入</x:v>
       </x:c>
-      <x:c r="F4" s="37" t="str">
+      <x:c r="G4" s="47" t="str">
+        <x:v>本人接続</x:v>
+      </x:c>
+      <x:c r="H4" s="47" t="str">
         <x:v>本編開始</x:v>
       </x:c>
-      <x:c r="G4" s="37" t="str">
+      <x:c r="I4" s="47" t="str">
         <x:v>制作中</x:v>
       </x:c>
-      <x:c r="H4" s="37" t="str">
+      <x:c r="J4" s="47" t="str">
         <x:v>仕上げ</x:v>
       </x:c>
-      <x:c r="I4" s="37" t="str">
+      <x:c r="K4" s="47" t="str">
         <x:v>完成後</x:v>
       </x:c>
-      <x:c r="J4" s="37" t="str">
+      <x:c r="L4" s="47" t="str">
         <x:v>備考</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="36" customHeight="1">
+    <x:row r="5" ht="40" customHeight="1">
       <x:c r="A5" s="40" t="str">
         <x:v>S01</x:v>
       </x:c>
@@ -2664,11 +2738,11 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="E5" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F5" s="40" t="str">
         <x:v>△</x:v>
       </x:c>
-      <x:c r="F5" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="G5" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
@@ -2676,13 +2750,19 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="I5" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="J5" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K5" s="40" t="str">
         <x:v>△</x:v>
       </x:c>
-      <x:c r="J5" s="40" t="str">
+      <x:c r="L5" s="40" t="str">
         <x:v>登録時を基本</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="36" customHeight="1">
+    <x:row r="6" ht="40" customHeight="1">
       <x:c r="A6" s="40" t="str">
         <x:v>S02</x:v>
       </x:c>
@@ -2690,7 +2770,7 @@
         <x:v>対象Person確認</x:v>
       </x:c>
       <x:c r="C6" s="40" t="str">
-        <x:v>●</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="D6" s="40" t="str">
         <x:v>●</x:v>
@@ -2702,19 +2782,25 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="G6" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>●</x:v>
       </x:c>
       <x:c r="H6" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="I6" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="J6" s="40" t="str">
         <x:v>●</x:v>
       </x:c>
-      <x:c r="I6" s="40" t="str">
+      <x:c r="K6" s="40" t="str">
         <x:v>△</x:v>
       </x:c>
-      <x:c r="J6" s="40" t="str">
-        <x:v>親支援では特に重要</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="36" customHeight="1">
+      <x:c r="L6" s="40" t="str">
+        <x:v>本人起点ではAccount登録とPerson作成が同時の場合あり</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="40" customHeight="1">
       <x:c r="A7" s="40" t="str">
         <x:v>S03</x:v>
       </x:c>
@@ -2734,7 +2820,7 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="G7" s="40" t="str">
-        <x:v>△</x:v>
+        <x:v>●</x:v>
       </x:c>
       <x:c r="H7" s="40" t="str">
         <x:v>△</x:v>
@@ -2743,10 +2829,16 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="J7" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="K7" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="L7" s="40" t="str">
         <x:v>本人に短く説明、停止可</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="36" customHeight="1">
+    <x:row r="8" ht="40" customHeight="1">
       <x:c r="A8" s="40" t="str">
         <x:v>S04</x:v>
       </x:c>
@@ -2760,25 +2852,31 @@
         <x:v>●</x:v>
       </x:c>
       <x:c r="E8" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>△</x:v>
       </x:c>
       <x:c r="F8" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="G8" s="40" t="str">
-        <x:v>△</x:v>
+        <x:v>●</x:v>
       </x:c>
       <x:c r="H8" s="40" t="str">
-        <x:v>△</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="I8" s="40" t="str">
         <x:v>△</x:v>
       </x:c>
       <x:c r="J8" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="K8" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="L8" s="40" t="str">
         <x:v>内容共有とは別</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="36" customHeight="1">
+    <x:row r="9" ht="40" customHeight="1">
       <x:c r="A9" s="40" t="str">
         <x:v>S05</x:v>
       </x:c>
@@ -2789,10 +2887,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="D9" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E9" s="40" t="str">
         <x:v>●</x:v>
-      </x:c>
-      <x:c r="E9" s="40" t="str">
-        <x:v>—</x:v>
       </x:c>
       <x:c r="F9" s="40" t="str">
         <x:v>—</x:v>
@@ -2801,16 +2899,22 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="H9" s="40" t="str">
-        <x:v>△</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="I9" s="40" t="str">
         <x:v>△</x:v>
       </x:c>
       <x:c r="J9" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="K9" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="L9" s="40" t="str">
         <x:v>語り単位</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="36" customHeight="1">
+    <x:row r="10" ht="40" customHeight="1">
       <x:c r="A10" s="40" t="str">
         <x:v>S06</x:v>
       </x:c>
@@ -2830,19 +2934,25 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="G10" s="40" t="str">
-        <x:v>△</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="H10" s="40" t="str">
-        <x:v>●</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="I10" s="40" t="str">
         <x:v>△</x:v>
       </x:c>
       <x:c r="J10" s="40" t="str">
+        <x:v>●</x:v>
+      </x:c>
+      <x:c r="K10" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="L10" s="40" t="str">
         <x:v>仕上げで最終確認</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="36" customHeight="1">
+    <x:row r="11" ht="40" customHeight="1">
       <x:c r="A11" s="40" t="str">
         <x:v>S07</x:v>
       </x:c>
@@ -2865,16 +2975,22 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="H11" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I11" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="J11" s="40" t="str">
         <x:v>●</x:v>
       </x:c>
-      <x:c r="I11" s="40" t="str">
+      <x:c r="K11" s="40" t="str">
         <x:v>△</x:v>
       </x:c>
-      <x:c r="J11" s="40" t="str">
+      <x:c r="L11" s="40" t="str">
         <x:v>作品単位</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="36" customHeight="1">
+    <x:row r="12" ht="40" customHeight="1">
       <x:c r="A12" s="40" t="str">
         <x:v>S08</x:v>
       </x:c>
@@ -2897,16 +3013,22 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="H12" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I12" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="J12" s="40" t="str">
         <x:v>●</x:v>
       </x:c>
-      <x:c r="I12" s="40" t="str">
+      <x:c r="K12" s="40" t="str">
         <x:v>△</x:v>
       </x:c>
-      <x:c r="J12" s="40" t="str">
+      <x:c r="L12" s="40" t="str">
         <x:v>家族共有と独立</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="36" customHeight="1">
+    <x:row r="13" ht="40" customHeight="1">
       <x:c r="A13" s="40" t="str">
         <x:v>S09</x:v>
       </x:c>
@@ -2923,22 +3045,28 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F13" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G13" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="H13" s="40" t="str">
         <x:v>●</x:v>
       </x:c>
-      <x:c r="G13" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H13" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="I13" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="J13" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K13" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="L13" s="40" t="str">
         <x:v>本人の明示操作</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="36" customHeight="1">
+    <x:row r="14" ht="40" customHeight="1">
       <x:c r="A14" s="40" t="str">
         <x:v>S10</x:v>
       </x:c>
@@ -2958,22 +3086,28 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="G14" s="40" t="str">
-        <x:v>△</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="H14" s="40" t="str">
-        <x:v>△</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="I14" s="40" t="str">
         <x:v>△</x:v>
       </x:c>
       <x:c r="J14" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="K14" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="L14" s="40" t="str">
         <x:v>個人データの収集と混同しない</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:J1"/>
-    <x:mergeCell ref="A2:J2"/>
+    <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A2:L2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3032,31 +3166,31 @@
       <x:c r="I3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="37" t="str">
+      <x:c r="A4" s="47" t="str">
         <x:v>Case</x:v>
       </x:c>
-      <x:c r="B4" s="37" t="str">
+      <x:c r="B4" s="47" t="str">
         <x:v>位置づけ</x:v>
       </x:c>
-      <x:c r="C4" s="37" t="str">
+      <x:c r="C4" s="47" t="str">
         <x:v>HPに来た人</x:v>
       </x:c>
-      <x:c r="D4" s="37" t="str">
+      <x:c r="D4" s="47" t="str">
         <x:v>語る人</x:v>
       </x:c>
-      <x:c r="E4" s="37" t="str">
+      <x:c r="E4" s="47" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="F4" s="37" t="str">
+      <x:c r="F4" s="47" t="str">
         <x:v>同席・遠隔</x:v>
       </x:c>
-      <x:c r="G4" s="37" t="str">
+      <x:c r="G4" s="47" t="str">
         <x:v>購入者候補</x:v>
       </x:c>
-      <x:c r="H4" s="37" t="str">
+      <x:c r="H4" s="47" t="str">
         <x:v>本人Accountが必要になる時</x:v>
       </x:c>
-      <x:c r="I4" s="37" t="str">
+      <x:c r="I4" s="47" t="str">
         <x:v>要点</x:v>
       </x:c>
     </x:row>
@@ -3197,22 +3331,22 @@
       <x:c r="F3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="37" t="str">
+      <x:c r="A4" s="47" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B4" s="37" t="str">
+      <x:c r="B4" s="47" t="str">
         <x:v>論点</x:v>
       </x:c>
-      <x:c r="C4" s="37" t="str">
+      <x:c r="C4" s="47" t="str">
         <x:v>現状案</x:v>
       </x:c>
-      <x:c r="D4" s="37" t="str">
+      <x:c r="D4" s="47" t="str">
         <x:v>状態</x:v>
       </x:c>
-      <x:c r="E4" s="37" t="str">
+      <x:c r="E4" s="47" t="str">
         <x:v>決める理由</x:v>
       </x:c>
-      <x:c r="F4" s="37" t="str">
+      <x:c r="F4" s="47" t="str">
         <x:v>次アクション</x:v>
       </x:c>
     </x:row>
@@ -3403,6 +3537,9 @@
   </x:mergeCells>
   <x:conditionalFormatting sqref="A5:F13">
     <x:cfRule type="expression" dxfId="1" priority="1">
+      <x:formula>$D5="要確認"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="4" priority="2">
       <x:formula>$D5="要確認"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -3472,34 +3609,34 @@
       <x:c r="J3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="37" t="str">
+      <x:c r="A4" s="47" t="str">
         <x:v>Setting ID</x:v>
       </x:c>
-      <x:c r="B4" s="37" t="str">
+      <x:c r="B4" s="47" t="str">
         <x:v>設定・同意名</x:v>
       </x:c>
-      <x:c r="C4" s="37" t="str">
+      <x:c r="C4" s="47" t="str">
         <x:v>利用者が設定する画面</x:v>
       </x:c>
-      <x:c r="D4" s="37" t="str">
+      <x:c r="D4" s="47" t="str">
         <x:v>初期値</x:v>
       </x:c>
-      <x:c r="E4" s="37" t="str">
+      <x:c r="E4" s="47" t="str">
         <x:v>設定できる人</x:v>
       </x:c>
-      <x:c r="F4" s="37" t="str">
+      <x:c r="F4" s="47" t="str">
         <x:v>変更できる時期</x:v>
       </x:c>
-      <x:c r="G4" s="37" t="str">
+      <x:c r="G4" s="47" t="str">
         <x:v>保存先</x:v>
       </x:c>
-      <x:c r="H4" s="37" t="str">
+      <x:c r="H4" s="47" t="str">
         <x:v>関連Flow ID</x:v>
       </x:c>
-      <x:c r="I4" s="37" t="str">
+      <x:c r="I4" s="47" t="str">
         <x:v>実装状態</x:v>
       </x:c>
-      <x:c r="J4" s="37" t="str">
+      <x:c r="J4" s="47" t="str">
         <x:v>根拠仕様</x:v>
       </x:c>
     </x:row>
@@ -3590,7 +3727,7 @@
         <x:v>project_supporters／family_subject_bindings.initiated_by</x:v>
       </x:c>
       <x:c r="H7" s="40" t="str">
-        <x:v>B-CO-020、B-REMOTE-020、B-DIRECT-010</x:v>
+        <x:v>B-CO-020、B-REMOTE-020、B-DIRECT-GIFT-010</x:v>
       </x:c>
       <x:c r="I7" s="40" t="str">
         <x:v>一部実装</x:v>
@@ -3782,7 +3919,7 @@
         <x:v>experience_contracts.main_experience_started_at／main_started_by／guarantee_days／guarantee_expires_at</x:v>
       </x:c>
       <x:c r="H13" s="40" t="str">
-        <x:v>A-TRIAL-040、A-DIRECT-020、B-CO-GIFT-060、B-REMOTE-SELF-050、B-DIRECT-030</x:v>
+        <x:v>A-TRIAL-040、A-DIRECT-020、B-CO-GIFT-060、B-REMOTE-SELF-050、B-DIRECT-GIFT-030</x:v>
       </x:c>
       <x:c r="I13" s="40" t="str">
         <x:v>一部実装</x:v>
@@ -3830,6 +3967,9 @@
   </x:mergeCells>
   <x:conditionalFormatting sqref="A5:J14">
     <x:cfRule type="expression" dxfId="2" priority="1">
+      <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="5" priority="2">
       <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>

</xml_diff>

<commit_message>
docs: confirm trial story sharing default
</commit_message>
<xml_diff>
--- a/docs/product/user-flow/user-flow-master.xlsx
+++ b/docs/product/user-flow/user-flow-master.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="R58243710d7024acd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_利用動線" sheetId="2" r:id="R86e095bca6d244cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定同意" sheetId="3" r:id="R3c0f70032b4141c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ケース一覧" sheetId="4" r:id="R44fd16095399437f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_運営チェック" sheetId="5" r:id="R3836304b6ca64cfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_実装対応" sheetId="6" r:id="Rec3e7c3b368e43a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="R83777268435841a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_利用動線" sheetId="2" r:id="Rf8aa06f76e4d40eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定同意" sheetId="3" r:id="Re7e93e5089714709"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ケース一覧" sheetId="4" r:id="R9eb018af881d4074"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_運営チェック" sheetId="5" r:id="R185b6bc38c604d37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_実装対応" sheetId="6" r:id="Rd9d78a01f15a47c3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -82,7 +82,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -129,6 +129,16 @@
         <x:fgColor rgb="FFEEF4F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF315B5B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF4F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -151,7 +161,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="51">
+  <x:cellXfs count="58">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -259,11 +269,58 @@
     <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="6">
+  <x:dxfs count="9">
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:color rgb="FF8A5A00"/>
@@ -548,13 +605,13 @@
       <x:c r="C3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="47" t="str">
+      <x:c r="A4" s="54" t="str">
         <x:v>シート</x:v>
       </x:c>
-      <x:c r="B4" s="47" t="str">
+      <x:c r="B4" s="54" t="str">
         <x:v>役割</x:v>
       </x:c>
-      <x:c r="C4" s="47" t="str">
+      <x:c r="C4" s="54" t="str">
         <x:v>ポイント</x:v>
       </x:c>
     </x:row>
@@ -619,13 +676,13 @@
       <x:c r="C10" s="41"/>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
-      <x:c r="A11" s="50" t="str">
+      <x:c r="A11" s="57" t="str">
         <x:v>更新ルール</x:v>
       </x:c>
-      <x:c r="B11" s="50" t="str">
+      <x:c r="B11" s="57" t="str">
         <x:v>同名ファイルを更新</x:v>
       </x:c>
-      <x:c r="C11" s="50" t="str">
+      <x:c r="C11" s="57" t="str">
         <x:v>別バージョンのExcelを増やさず、変更理由と履歴はGitで管理する。</x:v>
       </x:c>
     </x:row>
@@ -751,76 +808,76 @@
       <x:c r="X3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="47" t="str">
+      <x:c r="A4" s="54" t="str">
         <x:v>Flow ID</x:v>
       </x:c>
-      <x:c r="B4" s="47" t="str">
+      <x:c r="B4" s="54" t="str">
         <x:v>Case</x:v>
       </x:c>
-      <x:c r="C4" s="47" t="str">
+      <x:c r="C4" s="54" t="str">
         <x:v>Subcase</x:v>
       </x:c>
-      <x:c r="D4" s="47" t="str">
+      <x:c r="D4" s="54" t="str">
         <x:v>Step</x:v>
       </x:c>
-      <x:c r="E4" s="47" t="str">
+      <x:c r="E4" s="54" t="str">
         <x:v>ユーザー行動</x:v>
       </x:c>
-      <x:c r="F4" s="47" t="str">
+      <x:c r="F4" s="54" t="str">
         <x:v>ユーザーへの説明</x:v>
       </x:c>
-      <x:c r="G4" s="47" t="str">
+      <x:c r="G4" s="54" t="str">
         <x:v>利用中Account</x:v>
       </x:c>
-      <x:c r="H4" s="47" t="str">
+      <x:c r="H4" s="54" t="str">
         <x:v>このStepの操作者</x:v>
       </x:c>
-      <x:c r="I4" s="47" t="str">
+      <x:c r="I4" s="54" t="str">
         <x:v>このStepで語る人</x:v>
       </x:c>
-      <x:c r="J4" s="47" t="str">
+      <x:c r="J4" s="54" t="str">
         <x:v>Person</x:v>
       </x:c>
-      <x:c r="K4" s="47" t="str">
+      <x:c r="K4" s="54" t="str">
         <x:v>Payer</x:v>
       </x:c>
-      <x:c r="L4" s="47" t="str">
+      <x:c r="L4" s="54" t="str">
         <x:v>Supporter</x:v>
       </x:c>
-      <x:c r="M4" s="47" t="str">
+      <x:c r="M4" s="54" t="str">
         <x:v>Device</x:v>
       </x:c>
-      <x:c r="N4" s="47" t="str">
+      <x:c r="N4" s="54" t="str">
         <x:v>現在状態</x:v>
       </x:c>
-      <x:c r="O4" s="47" t="str">
+      <x:c r="O4" s="54" t="str">
         <x:v>分岐条件</x:v>
       </x:c>
-      <x:c r="P4" s="47" t="str">
+      <x:c r="P4" s="54" t="str">
         <x:v>次の状態</x:v>
       </x:c>
-      <x:c r="Q4" s="47" t="str">
+      <x:c r="Q4" s="54" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="R4" s="47" t="str">
+      <x:c r="R4" s="54" t="str">
         <x:v>購入</x:v>
       </x:c>
-      <x:c r="S4" s="47" t="str">
+      <x:c r="S4" s="54" t="str">
         <x:v>本人認証</x:v>
       </x:c>
-      <x:c r="T4" s="47" t="str">
+      <x:c r="T4" s="54" t="str">
         <x:v>設定・同意</x:v>
       </x:c>
-      <x:c r="U4" s="47" t="str">
+      <x:c r="U4" s="54" t="str">
         <x:v>内容共有</x:v>
       </x:c>
-      <x:c r="V4" s="47" t="str">
+      <x:c r="V4" s="54" t="str">
         <x:v>進捗共有</x:v>
       </x:c>
-      <x:c r="W4" s="47" t="str">
+      <x:c r="W4" s="54" t="str">
         <x:v>内部メモ</x:v>
       </x:c>
-      <x:c r="X4" s="47" t="str">
+      <x:c r="X4" s="54" t="str">
         <x:v>確定度</x:v>
       </x:c>
     </x:row>
@@ -960,7 +1017,7 @@
         <x:v>語り共有初期値</x:v>
       </x:c>
       <x:c r="U6" s="40" t="str">
-        <x:v>自分だけ候補</x:v>
+        <x:v>本人のみ</x:v>
       </x:c>
       <x:c r="V6" s="40" t="str">
         <x:v>—</x:v>
@@ -969,7 +1026,7 @@
         <x:v>同じPersonへ保存</x:v>
       </x:c>
       <x:c r="X6" s="40" t="str">
-        <x:v>要確認</x:v>
+        <x:v>確定</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -1478,7 +1535,7 @@
         <x:v>語り共有初期値・進捗共有</x:v>
       </x:c>
       <x:c r="U13" s="40" t="str">
-        <x:v>自分だけ候補</x:v>
+        <x:v>本人のみ</x:v>
       </x:c>
       <x:c r="V13" s="40" t="str">
         <x:v>ON候補</x:v>
@@ -1922,7 +1979,7 @@
         <x:v>体験同意</x:v>
       </x:c>
       <x:c r="U19" s="40" t="str">
-        <x:v>自動共有なし</x:v>
+        <x:v>本人のみ</x:v>
       </x:c>
       <x:c r="V19" s="40" t="str">
         <x:v>完了≠続行</x:v>
@@ -2610,6 +2667,9 @@
       <x:formula>$X5="要確認"</x:formula>
     </x:cfRule>
     <x:cfRule type="expression" dxfId="3" priority="2">
+      <x:formula>$X5="要確認"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="6" priority="3">
       <x:formula>$X5="要確認"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -2687,40 +2747,40 @@
       <x:c r="L3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="47" t="str">
+      <x:c r="A4" s="54" t="str">
         <x:v>Setting ID</x:v>
       </x:c>
-      <x:c r="B4" s="47" t="str">
+      <x:c r="B4" s="54" t="str">
         <x:v>設定・同意</x:v>
       </x:c>
-      <x:c r="C4" s="47" t="str">
+      <x:c r="C4" s="54" t="str">
         <x:v>Account登録</x:v>
       </x:c>
-      <x:c r="D4" s="47" t="str">
+      <x:c r="D4" s="54" t="str">
         <x:v>対象Person作成</x:v>
       </x:c>
-      <x:c r="E4" s="47" t="str">
+      <x:c r="E4" s="54" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="F4" s="47" t="str">
+      <x:c r="F4" s="54" t="str">
         <x:v>購入</x:v>
       </x:c>
-      <x:c r="G4" s="47" t="str">
+      <x:c r="G4" s="54" t="str">
         <x:v>本人接続</x:v>
       </x:c>
-      <x:c r="H4" s="47" t="str">
+      <x:c r="H4" s="54" t="str">
         <x:v>本編開始</x:v>
       </x:c>
-      <x:c r="I4" s="47" t="str">
+      <x:c r="I4" s="54" t="str">
         <x:v>制作中</x:v>
       </x:c>
-      <x:c r="J4" s="47" t="str">
+      <x:c r="J4" s="54" t="str">
         <x:v>仕上げ</x:v>
       </x:c>
-      <x:c r="K4" s="47" t="str">
+      <x:c r="K4" s="54" t="str">
         <x:v>完成後</x:v>
       </x:c>
-      <x:c r="L4" s="47" t="str">
+      <x:c r="L4" s="54" t="str">
         <x:v>備考</x:v>
       </x:c>
     </x:row>
@@ -2881,7 +2941,7 @@
         <x:v>S05</x:v>
       </x:c>
       <x:c r="B9" s="40" t="str">
-        <x:v>語り共有 自分だけ／家族</x:v>
+        <x:v>語り共有 本人のみ／家族</x:v>
       </x:c>
       <x:c r="C9" s="40" t="str">
         <x:v>—</x:v>
@@ -2911,7 +2971,7 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="L9" s="40" t="str">
-        <x:v>語り単位</x:v>
+        <x:v>初期値は本人のみ。進捗共有とは別</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40" customHeight="1">
@@ -3166,31 +3226,31 @@
       <x:c r="I3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="47" t="str">
+      <x:c r="A4" s="54" t="str">
         <x:v>Case</x:v>
       </x:c>
-      <x:c r="B4" s="47" t="str">
+      <x:c r="B4" s="54" t="str">
         <x:v>位置づけ</x:v>
       </x:c>
-      <x:c r="C4" s="47" t="str">
+      <x:c r="C4" s="54" t="str">
         <x:v>HPに来た人</x:v>
       </x:c>
-      <x:c r="D4" s="47" t="str">
+      <x:c r="D4" s="54" t="str">
         <x:v>語る人</x:v>
       </x:c>
-      <x:c r="E4" s="47" t="str">
+      <x:c r="E4" s="54" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="F4" s="47" t="str">
+      <x:c r="F4" s="54" t="str">
         <x:v>同席・遠隔</x:v>
       </x:c>
-      <x:c r="G4" s="47" t="str">
+      <x:c r="G4" s="54" t="str">
         <x:v>購入者候補</x:v>
       </x:c>
-      <x:c r="H4" s="47" t="str">
+      <x:c r="H4" s="54" t="str">
         <x:v>本人Accountが必要になる時</x:v>
       </x:c>
-      <x:c r="I4" s="47" t="str">
+      <x:c r="I4" s="54" t="str">
         <x:v>要点</x:v>
       </x:c>
     </x:row>
@@ -3331,22 +3391,22 @@
       <x:c r="F3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="47" t="str">
+      <x:c r="A4" s="54" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B4" s="47" t="str">
+      <x:c r="B4" s="54" t="str">
         <x:v>論点</x:v>
       </x:c>
-      <x:c r="C4" s="47" t="str">
+      <x:c r="C4" s="54" t="str">
         <x:v>現状案</x:v>
       </x:c>
-      <x:c r="D4" s="47" t="str">
+      <x:c r="D4" s="54" t="str">
         <x:v>状態</x:v>
       </x:c>
-      <x:c r="E4" s="47" t="str">
+      <x:c r="E4" s="54" t="str">
         <x:v>決める理由</x:v>
       </x:c>
-      <x:c r="F4" s="47" t="str">
+      <x:c r="F4" s="54" t="str">
         <x:v>次アクション</x:v>
       </x:c>
     </x:row>
@@ -3358,16 +3418,16 @@
         <x:v>無料3問の語り共有初期値</x:v>
       </x:c>
       <x:c r="C5" s="40" t="str">
-        <x:v>自分だけを第一候補</x:v>
+        <x:v>本人のみ。Supporterには進捗だけを共有</x:v>
       </x:c>
       <x:c r="D5" s="40" t="str">
-        <x:v>要確認</x:v>
+        <x:v>確定</x:v>
       </x:c>
       <x:c r="E5" s="40" t="str">
         <x:v>親支援時のプライバシーと体験を左右</x:v>
       </x:c>
       <x:c r="F5" s="40" t="str">
-        <x:v>UIと既存仕様を照合</x:v>
+        <x:v>B同席・子購入の実装へ反映</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="50" customHeight="1">
@@ -3540,6 +3600,9 @@
       <x:formula>$D5="要確認"</x:formula>
     </x:cfRule>
     <x:cfRule type="expression" dxfId="4" priority="2">
+      <x:formula>$D5="要確認"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="7" priority="3">
       <x:formula>$D5="要確認"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -3609,34 +3672,34 @@
       <x:c r="J3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="47" t="str">
+      <x:c r="A4" s="54" t="str">
         <x:v>Setting ID</x:v>
       </x:c>
-      <x:c r="B4" s="47" t="str">
+      <x:c r="B4" s="54" t="str">
         <x:v>設定・同意名</x:v>
       </x:c>
-      <x:c r="C4" s="47" t="str">
+      <x:c r="C4" s="54" t="str">
         <x:v>利用者が設定する画面</x:v>
       </x:c>
-      <x:c r="D4" s="47" t="str">
+      <x:c r="D4" s="54" t="str">
         <x:v>初期値</x:v>
       </x:c>
-      <x:c r="E4" s="47" t="str">
+      <x:c r="E4" s="54" t="str">
         <x:v>設定できる人</x:v>
       </x:c>
-      <x:c r="F4" s="47" t="str">
+      <x:c r="F4" s="54" t="str">
         <x:v>変更できる時期</x:v>
       </x:c>
-      <x:c r="G4" s="47" t="str">
+      <x:c r="G4" s="54" t="str">
         <x:v>保存先</x:v>
       </x:c>
-      <x:c r="H4" s="47" t="str">
+      <x:c r="H4" s="54" t="str">
         <x:v>関連Flow ID</x:v>
       </x:c>
-      <x:c r="I4" s="47" t="str">
+      <x:c r="I4" s="54" t="str">
         <x:v>実装状態</x:v>
       </x:c>
-      <x:c r="J4" s="47" t="str">
+      <x:c r="J4" s="54" t="str">
         <x:v>根拠仕様</x:v>
       </x:c>
     </x:row>
@@ -3773,13 +3836,13 @@
         <x:v>S05</x:v>
       </x:c>
       <x:c r="B9" s="40" t="str">
-        <x:v>語り共有 自分だけ／家族</x:v>
+        <x:v>語り共有 本人のみ／家族</x:v>
       </x:c>
       <x:c r="C9" s="40" t="str">
         <x:v>録音保存時／語り設定</x:v>
       </x:c>
       <x:c r="D9" s="40" t="str">
-        <x:v>自分だけ候補</x:v>
+        <x:v>本人のみ（Supporterへの自動共有なし）</x:v>
       </x:c>
       <x:c r="E9" s="40" t="str">
         <x:v>本人。Supporterは本人の公開範囲を拡張しない。</x:v>
@@ -3972,6 +4035,9 @@
     <x:cfRule type="expression" dxfId="5" priority="2">
       <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
     </x:cfRule>
+    <x:cfRule type="expression" dxfId="8" priority="3">
+      <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
+    </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="I5:I14">

</xml_diff>

<commit_message>
docs: add delegated support style
</commit_message>
<xml_diff>
--- a/docs/product/user-flow/user-flow-master.xlsx
+++ b/docs/product/user-flow/user-flow-master.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="R83777268435841a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_利用動線" sheetId="2" r:id="Rf8aa06f76e4d40eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定同意" sheetId="3" r:id="Re7e93e5089714709"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ケース一覧" sheetId="4" r:id="R9eb018af881d4074"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_運営チェック" sheetId="5" r:id="R185b6bc38c604d37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_実装対応" sheetId="6" r:id="Rd9d78a01f15a47c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="R4f2c39fdb6fb4df0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_利用動線" sheetId="2" r:id="R08d36ea6b2ec41d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定同意" sheetId="3" r:id="Rf8e54bb235c24001"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ケース一覧" sheetId="4" r:id="R25c98bfd1b8d41e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_運営チェック" sheetId="5" r:id="R01cc07579652463b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_実装対応" sheetId="6" r:id="R6996979a404c4678"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_支援スタイル・権限" sheetId="7" r:id="R188b9cdbebe24e39"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +19,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="11">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -81,8 +82,14 @@
       <x:color rgb="FF233B3B"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF233B3B"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -139,6 +146,26 @@
         <x:fgColor rgb="FFEEF4F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF315B5B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF4F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF315B5B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF4F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -161,7 +188,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="58">
+  <x:cellXfs count="75">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -286,11 +313,114 @@
     <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="9">
+  <x:dxfs count="15">
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:color rgb="FF8A5A00"/>
@@ -605,13 +735,13 @@
       <x:c r="C3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="54" t="str">
+      <x:c r="A4" s="70" t="str">
         <x:v>シート</x:v>
       </x:c>
-      <x:c r="B4" s="54" t="str">
+      <x:c r="B4" s="70" t="str">
         <x:v>役割</x:v>
       </x:c>
-      <x:c r="C4" s="54" t="str">
+      <x:c r="C4" s="70" t="str">
         <x:v>ポイント</x:v>
       </x:c>
     </x:row>
@@ -671,18 +801,29 @@
       </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
-      <x:c r="A10" s="41"/>
-      <x:c r="B10" s="41"/>
-      <x:c r="C10" s="41"/>
+      <x:c r="A10" s="40" t="str">
+        <x:v>06_支援スタイル・権限</x:v>
+      </x:c>
+      <x:c r="B10" s="40" t="str">
+        <x:v>操作権限の基準</x:v>
+      </x:c>
+      <x:c r="C10" s="40" t="str">
+        <x:v>本人Accountなしのおまかせを含む3つの支援スタイルを定義する。</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
-      <x:c r="A11" s="57" t="str">
+      <x:c r="A11" s="41"/>
+      <x:c r="B11" s="41"/>
+      <x:c r="C11" s="41"/>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
+      <x:c r="A12" s="73" t="str">
         <x:v>更新ルール</x:v>
       </x:c>
-      <x:c r="B11" s="57" t="str">
+      <x:c r="B12" s="73" t="str">
         <x:v>同名ファイルを更新</x:v>
       </x:c>
-      <x:c r="C11" s="57" t="str">
+      <x:c r="C12" s="73" t="str">
         <x:v>別バージョンのExcelを増やさず、変更理由と履歴はGitで管理する。</x:v>
       </x:c>
     </x:row>
@@ -701,28 +842,29 @@
   <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="17" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="7" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="35" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="29" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="7" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="35" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="29" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="13" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="13" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="13" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="14" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="25" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="13" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="25" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="27" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="12" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="25" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="27" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="12" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="16" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="26" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="18" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="18" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="32" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="11" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="12" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="16" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="26" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="24" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="18" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="34" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="11" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -752,10 +894,11 @@
       <x:c r="V1" s="28"/>
       <x:c r="W1" s="28"/>
       <x:c r="X1" s="28"/>
+      <x:c r="Y1" s="28"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="30" t="str">
-        <x:v>黄色行は最終確認余地あり。Account＝認証・認可主体、操作者＝画面操作、語る人＝発話者、Person＝誰の人生か。</x:v>
+        <x:v>Person＝作品の主体。Account＝認証・認可主体。本人Account、Supporter Account、または両方が同じPersonの制作を担える。</x:v>
       </x:c>
       <x:c r="B2" s="30"/>
       <x:c r="C2" s="30"/>
@@ -780,6 +923,7 @@
       <x:c r="V2" s="30"/>
       <x:c r="W2" s="30"/>
       <x:c r="X2" s="30"/>
+      <x:c r="Y2" s="30"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3"/>
@@ -806,82 +950,86 @@
       <x:c r="V3"/>
       <x:c r="W3"/>
       <x:c r="X3"/>
+      <x:c r="Y3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="54" t="str">
+      <x:c r="A4" s="70" t="str">
         <x:v>Flow ID</x:v>
       </x:c>
-      <x:c r="B4" s="54" t="str">
+      <x:c r="B4" s="70" t="str">
         <x:v>Case</x:v>
       </x:c>
-      <x:c r="C4" s="54" t="str">
+      <x:c r="C4" s="70" t="str">
         <x:v>Subcase</x:v>
       </x:c>
-      <x:c r="D4" s="54" t="str">
+      <x:c r="D4" s="70" t="str">
+        <x:v>支援スタイル</x:v>
+      </x:c>
+      <x:c r="E4" s="70" t="str">
         <x:v>Step</x:v>
       </x:c>
-      <x:c r="E4" s="54" t="str">
+      <x:c r="F4" s="70" t="str">
         <x:v>ユーザー行動</x:v>
       </x:c>
-      <x:c r="F4" s="54" t="str">
+      <x:c r="G4" s="70" t="str">
         <x:v>ユーザーへの説明</x:v>
       </x:c>
-      <x:c r="G4" s="54" t="str">
+      <x:c r="H4" s="70" t="str">
         <x:v>利用中Account</x:v>
       </x:c>
-      <x:c r="H4" s="54" t="str">
+      <x:c r="I4" s="70" t="str">
         <x:v>このStepの操作者</x:v>
       </x:c>
-      <x:c r="I4" s="54" t="str">
+      <x:c r="J4" s="70" t="str">
         <x:v>このStepで語る人</x:v>
       </x:c>
-      <x:c r="J4" s="54" t="str">
+      <x:c r="K4" s="70" t="str">
         <x:v>Person</x:v>
       </x:c>
-      <x:c r="K4" s="54" t="str">
+      <x:c r="L4" s="70" t="str">
         <x:v>Payer</x:v>
       </x:c>
-      <x:c r="L4" s="54" t="str">
+      <x:c r="M4" s="70" t="str">
         <x:v>Supporter</x:v>
       </x:c>
-      <x:c r="M4" s="54" t="str">
+      <x:c r="N4" s="70" t="str">
         <x:v>Device</x:v>
       </x:c>
-      <x:c r="N4" s="54" t="str">
+      <x:c r="O4" s="70" t="str">
         <x:v>現在状態</x:v>
       </x:c>
-      <x:c r="O4" s="54" t="str">
+      <x:c r="P4" s="70" t="str">
         <x:v>分岐条件</x:v>
       </x:c>
-      <x:c r="P4" s="54" t="str">
+      <x:c r="Q4" s="70" t="str">
         <x:v>次の状態</x:v>
       </x:c>
-      <x:c r="Q4" s="54" t="str">
+      <x:c r="R4" s="70" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="R4" s="54" t="str">
+      <x:c r="S4" s="70" t="str">
         <x:v>購入</x:v>
       </x:c>
-      <x:c r="S4" s="54" t="str">
+      <x:c r="T4" s="70" t="str">
         <x:v>本人認証</x:v>
       </x:c>
-      <x:c r="T4" s="54" t="str">
+      <x:c r="U4" s="70" t="str">
         <x:v>設定・同意</x:v>
       </x:c>
-      <x:c r="U4" s="54" t="str">
+      <x:c r="V4" s="70" t="str">
         <x:v>内容共有</x:v>
       </x:c>
-      <x:c r="V4" s="54" t="str">
+      <x:c r="W4" s="70" t="str">
         <x:v>進捗共有</x:v>
       </x:c>
-      <x:c r="W4" s="54" t="str">
+      <x:c r="X4" s="70" t="str">
         <x:v>内部メモ</x:v>
       </x:c>
-      <x:c r="X4" s="54" t="str">
+      <x:c r="Y4" s="70" t="str">
         <x:v>確定度</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="54" customHeight="1">
+    <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" s="43" t="str">
         <x:v>A-TRIAL-010</x:v>
       </x:c>
@@ -891,47 +1039,47 @@
       <x:c r="C5" s="40" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="D5" s="40" t="n">
+      <x:c r="D5" s="40" t="str">
+        <x:v>自分で進める</x:v>
+      </x:c>
+      <x:c r="E5" s="40" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E5" s="40" t="str">
+      <x:c r="F5" s="40" t="str">
         <x:v>HP→無料3問→自分の物語</x:v>
       </x:c>
-      <x:c r="F5" s="40" t="str">
+      <x:c r="G5" s="40" t="str">
         <x:v>まず3問、無料で試せます。3問後に続けるか決められます。</x:v>
       </x:c>
-      <x:c r="G5" s="40" t="str">
+      <x:c r="H5" s="40" t="str">
         <x:v>なし</x:v>
       </x:c>
-      <x:c r="H5" s="40" t="str">
+      <x:c r="I5" s="40" t="str">
         <x:v>本人</x:v>
       </x:c>
-      <x:c r="I5" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="J5" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K5" s="40" t="str">
         <x:v>未作成</x:v>
       </x:c>
-      <x:c r="K5" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="L5" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="M5" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="N5" s="40" t="str">
         <x:v>本人端末</x:v>
       </x:c>
-      <x:c r="N5" s="40" t="str">
+      <x:c r="O5" s="40" t="str">
         <x:v>未登録</x:v>
       </x:c>
-      <x:c r="O5" s="40" t="str">
+      <x:c r="P5" s="40" t="str">
         <x:v>自分の物語／無料3問を選択</x:v>
       </x:c>
-      <x:c r="P5" s="40" t="str">
+      <x:c r="Q5" s="40" t="str">
         <x:v>本人Account・本人Person作成</x:v>
-      </x:c>
-      <x:c r="Q5" s="40" t="str">
-        <x:v>未</x:v>
       </x:c>
       <x:c r="R5" s="40" t="str">
         <x:v>未</x:v>
@@ -940,22 +1088,25 @@
         <x:v>未</x:v>
       </x:c>
       <x:c r="T5" s="40" t="str">
+        <x:v>未</x:v>
+      </x:c>
+      <x:c r="U5" s="40" t="str">
         <x:v>規約・プライバシー</x:v>
       </x:c>
-      <x:c r="U5" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="V5" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="W5" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="X5" s="40" t="str">
         <x:v>無料3問は購入条件ではない</x:v>
       </x:c>
-      <x:c r="X5" s="40" t="str">
+      <x:c r="Y5" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="54" customHeight="1">
+    <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" s="43" t="str">
         <x:v>A-TRIAL-020</x:v>
       </x:c>
@@ -965,17 +1116,17 @@
       <x:c r="C6" s="40" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="D6" s="40" t="n">
+      <x:c r="D6" s="40" t="str">
+        <x:v>自分で進める</x:v>
+      </x:c>
+      <x:c r="E6" s="40" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E6" s="40" t="str">
+      <x:c r="F6" s="40" t="str">
         <x:v>Account登録→幼い頃の3問を語る</x:v>
       </x:c>
-      <x:c r="F6" s="40" t="str">
+      <x:c r="G6" s="40" t="str">
         <x:v>ここまで無料です。続ける場合は内容と料金をご確認ください。</x:v>
-      </x:c>
-      <x:c r="G6" s="40" t="str">
-        <x:v>本人</x:v>
       </x:c>
       <x:c r="H6" s="40" t="str">
         <x:v>本人</x:v>
@@ -987,49 +1138,52 @@
         <x:v>本人</x:v>
       </x:c>
       <x:c r="K6" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="L6" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="M6" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="N6" s="40" t="str">
         <x:v>本人端末</x:v>
       </x:c>
-      <x:c r="N6" s="40" t="str">
+      <x:c r="O6" s="40" t="str">
         <x:v>Account・Person作成済／未購入</x:v>
       </x:c>
-      <x:c r="O6" s="40" t="str">
+      <x:c r="P6" s="40" t="str">
         <x:v>3問完了</x:v>
       </x:c>
-      <x:c r="P6" s="40" t="str">
+      <x:c r="Q6" s="40" t="str">
         <x:v>体験完了／未購入</x:v>
       </x:c>
-      <x:c r="Q6" s="40" t="str">
+      <x:c r="R6" s="40" t="str">
         <x:v>済</x:v>
       </x:c>
-      <x:c r="R6" s="40" t="str">
+      <x:c r="S6" s="40" t="str">
         <x:v>未</x:v>
       </x:c>
-      <x:c r="S6" s="40" t="str">
+      <x:c r="T6" s="40" t="str">
         <x:v>済</x:v>
       </x:c>
-      <x:c r="T6" s="40" t="str">
+      <x:c r="U6" s="40" t="str">
         <x:v>語り共有初期値</x:v>
       </x:c>
-      <x:c r="U6" s="40" t="str">
+      <x:c r="V6" s="40" t="str">
         <x:v>本人のみ</x:v>
       </x:c>
-      <x:c r="V6" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="W6" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="X6" s="40" t="str">
         <x:v>同じPersonへ保存</x:v>
       </x:c>
-      <x:c r="X6" s="40" t="str">
+      <x:c r="Y6" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="54" customHeight="1">
+    <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" s="43" t="str">
         <x:v>A-TRIAL-030</x:v>
       </x:c>
@@ -1039,47 +1193,47 @@
       <x:c r="C7" s="40" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="D7" s="40" t="n">
+      <x:c r="D7" s="40" t="str">
+        <x:v>自分で進める</x:v>
+      </x:c>
+      <x:c r="E7" s="40" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E7" s="40" t="str">
+      <x:c r="F7" s="40" t="str">
         <x:v>本人が購入</x:v>
       </x:c>
-      <x:c r="F7" s="40" t="str">
+      <x:c r="G7" s="40" t="str">
         <x:v>購入後、「はじまりの章」から本編を始められます。</x:v>
-      </x:c>
-      <x:c r="G7" s="40" t="str">
-        <x:v>本人</x:v>
       </x:c>
       <x:c r="H7" s="40" t="str">
         <x:v>本人</x:v>
       </x:c>
       <x:c r="I7" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="J7" s="40" t="str">
-        <x:v>本人</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="K7" s="40" t="str">
         <x:v>本人</x:v>
       </x:c>
       <x:c r="L7" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="M7" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="N7" s="40" t="str">
         <x:v>本人端末</x:v>
       </x:c>
-      <x:c r="N7" s="40" t="str">
+      <x:c r="O7" s="40" t="str">
         <x:v>体験完了／未購入</x:v>
       </x:c>
-      <x:c r="O7" s="40" t="str">
+      <x:c r="P7" s="40" t="str">
         <x:v>本人購入を確定</x:v>
       </x:c>
-      <x:c r="P7" s="40" t="str">
+      <x:c r="Q7" s="40" t="str">
         <x:v>支払済／本編未開始</x:v>
-      </x:c>
-      <x:c r="Q7" s="40" t="str">
-        <x:v>済</x:v>
       </x:c>
       <x:c r="R7" s="40" t="str">
         <x:v>済</x:v>
@@ -1088,22 +1242,25 @@
         <x:v>済</x:v>
       </x:c>
       <x:c r="T7" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="U7" s="40" t="str">
         <x:v>購入条件・30日保証</x:v>
       </x:c>
-      <x:c r="U7" s="40" t="str">
+      <x:c r="V7" s="40" t="str">
         <x:v>維持</x:v>
       </x:c>
-      <x:c r="V7" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="W7" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="X7" s="40" t="str">
         <x:v>同じPerson・Projectへ接続</x:v>
       </x:c>
-      <x:c r="X7" s="40" t="str">
+      <x:c r="Y7" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="54" customHeight="1">
+    <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" s="43" t="str">
         <x:v>A-TRIAL-040</x:v>
       </x:c>
@@ -1113,17 +1270,17 @@
       <x:c r="C8" s="40" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="D8" s="40" t="n">
+      <x:c r="D8" s="40" t="str">
+        <x:v>自分で進める</x:v>
+      </x:c>
+      <x:c r="E8" s="40" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E8" s="40" t="str">
+      <x:c r="F8" s="40" t="str">
         <x:v>はじまりの章→本編をはじめる</x:v>
       </x:c>
-      <x:c r="F8" s="40" t="str">
+      <x:c r="G8" s="40" t="str">
         <x:v>本編を開始すると、9つのテーマを順番に辿れます。</x:v>
-      </x:c>
-      <x:c r="G8" s="40" t="str">
-        <x:v>本人</x:v>
       </x:c>
       <x:c r="H8" s="40" t="str">
         <x:v>本人</x:v>
@@ -1138,22 +1295,22 @@
         <x:v>本人</x:v>
       </x:c>
       <x:c r="L8" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="M8" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="N8" s="40" t="str">
         <x:v>本人端末</x:v>
       </x:c>
-      <x:c r="N8" s="40" t="str">
+      <x:c r="O8" s="40" t="str">
         <x:v>支払済／本編未開始</x:v>
       </x:c>
-      <x:c r="O8" s="40" t="str">
+      <x:c r="P8" s="40" t="str">
         <x:v>本人が明示して本編開始</x:v>
       </x:c>
-      <x:c r="P8" s="40" t="str">
+      <x:c r="Q8" s="40" t="str">
         <x:v>本編利用中／保証終了</x:v>
-      </x:c>
-      <x:c r="Q8" s="40" t="str">
-        <x:v>済</x:v>
       </x:c>
       <x:c r="R8" s="40" t="str">
         <x:v>済</x:v>
@@ -1162,22 +1319,25 @@
         <x:v>済</x:v>
       </x:c>
       <x:c r="T8" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="U8" s="40" t="str">
         <x:v>本編開始確認</x:v>
       </x:c>
-      <x:c r="U8" s="40" t="str">
+      <x:c r="V8" s="40" t="str">
         <x:v>語りごと</x:v>
       </x:c>
-      <x:c r="V8" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="W8" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="X8" s="40" t="str">
         <x:v>本編開始日時をサーバー確定</x:v>
       </x:c>
-      <x:c r="X8" s="40" t="str">
+      <x:c r="Y8" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="54" customHeight="1">
+    <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" s="43" t="str">
         <x:v>A-DIRECT-010</x:v>
       </x:c>
@@ -1187,71 +1347,74 @@
       <x:c r="C9" s="40" t="str">
         <x:v>直接購入</x:v>
       </x:c>
-      <x:c r="D9" s="40" t="n">
+      <x:c r="D9" s="40" t="str">
+        <x:v>自分で進める</x:v>
+      </x:c>
+      <x:c r="E9" s="40" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E9" s="40" t="str">
+      <x:c r="F9" s="40" t="str">
         <x:v>HP→内容・料金→縦糸横糸をはじめる</x:v>
       </x:c>
-      <x:c r="F9" s="40" t="str">
+      <x:c r="G9" s="40" t="str">
         <x:v>無料体験をせず、そのまま購入して始められます。</x:v>
       </x:c>
-      <x:c r="G9" s="40" t="str">
+      <x:c r="H9" s="40" t="str">
         <x:v>なし→本人</x:v>
       </x:c>
-      <x:c r="H9" s="40" t="str">
+      <x:c r="I9" s="40" t="str">
         <x:v>本人</x:v>
       </x:c>
-      <x:c r="I9" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="J9" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K9" s="40" t="str">
         <x:v>未作成→本人</x:v>
       </x:c>
-      <x:c r="K9" s="40" t="str">
+      <x:c r="L9" s="40" t="str">
         <x:v>本人</x:v>
       </x:c>
-      <x:c r="L9" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="M9" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="N9" s="40" t="str">
         <x:v>本人端末</x:v>
       </x:c>
-      <x:c r="N9" s="40" t="str">
+      <x:c r="O9" s="40" t="str">
         <x:v>未登録／未購入</x:v>
       </x:c>
-      <x:c r="O9" s="40" t="str">
+      <x:c r="P9" s="40" t="str">
         <x:v>無料3問を経ず購入</x:v>
       </x:c>
-      <x:c r="P9" s="40" t="str">
+      <x:c r="Q9" s="40" t="str">
         <x:v>支払済／本編未開始</x:v>
       </x:c>
-      <x:c r="Q9" s="40" t="str">
+      <x:c r="R9" s="40" t="str">
         <x:v>なし</x:v>
       </x:c>
-      <x:c r="R9" s="40" t="str">
+      <x:c r="S9" s="40" t="str">
         <x:v>済</x:v>
       </x:c>
-      <x:c r="S9" s="40" t="str">
+      <x:c r="T9" s="40" t="str">
         <x:v>本人登録</x:v>
       </x:c>
-      <x:c r="T9" s="40" t="str">
+      <x:c r="U9" s="40" t="str">
         <x:v>規約・購入条件・30日保証</x:v>
       </x:c>
-      <x:c r="U9" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="V9" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="W9" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="X9" s="40" t="str">
         <x:v>無料3問は任意</x:v>
       </x:c>
-      <x:c r="X9" s="40" t="str">
+      <x:c r="Y9" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="54" customHeight="1">
+    <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" s="43" t="str">
         <x:v>A-DIRECT-020</x:v>
       </x:c>
@@ -1261,17 +1424,17 @@
       <x:c r="C10" s="40" t="str">
         <x:v>直接購入</x:v>
       </x:c>
-      <x:c r="D10" s="40" t="n">
+      <x:c r="D10" s="40" t="str">
+        <x:v>自分で進める</x:v>
+      </x:c>
+      <x:c r="E10" s="40" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E10" s="40" t="str">
+      <x:c r="F10" s="40" t="str">
         <x:v>はじまりの章→本編をはじめる</x:v>
       </x:c>
-      <x:c r="F10" s="40" t="str">
+      <x:c r="G10" s="40" t="str">
         <x:v>本編を開始すると、9つのテーマを順番に辿れます。</x:v>
-      </x:c>
-      <x:c r="G10" s="40" t="str">
-        <x:v>本人</x:v>
       </x:c>
       <x:c r="H10" s="40" t="str">
         <x:v>本人</x:v>
@@ -1286,46 +1449,49 @@
         <x:v>本人</x:v>
       </x:c>
       <x:c r="L10" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="M10" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="N10" s="40" t="str">
         <x:v>本人端末</x:v>
       </x:c>
-      <x:c r="N10" s="40" t="str">
+      <x:c r="O10" s="40" t="str">
         <x:v>支払済／本編未開始</x:v>
       </x:c>
-      <x:c r="O10" s="40" t="str">
+      <x:c r="P10" s="40" t="str">
         <x:v>本人が明示して本編開始</x:v>
       </x:c>
-      <x:c r="P10" s="40" t="str">
+      <x:c r="Q10" s="40" t="str">
         <x:v>本編利用中／保証終了</x:v>
       </x:c>
-      <x:c r="Q10" s="40" t="str">
+      <x:c r="R10" s="40" t="str">
         <x:v>なし</x:v>
-      </x:c>
-      <x:c r="R10" s="40" t="str">
-        <x:v>済</x:v>
       </x:c>
       <x:c r="S10" s="40" t="str">
         <x:v>済</x:v>
       </x:c>
       <x:c r="T10" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="U10" s="40" t="str">
         <x:v>本編開始確認</x:v>
       </x:c>
-      <x:c r="U10" s="40" t="str">
+      <x:c r="V10" s="40" t="str">
         <x:v>語りごと</x:v>
       </x:c>
-      <x:c r="V10" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="W10" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="X10" s="40" t="str">
         <x:v>本編開始日時をサーバー確定</x:v>
       </x:c>
-      <x:c r="X10" s="40" t="str">
+      <x:c r="Y10" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="54" customHeight="1">
+    <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" s="43" t="str">
         <x:v>B-CO-010</x:v>
       </x:c>
@@ -1335,71 +1501,74 @@
       <x:c r="C11" s="40" t="str">
         <x:v>同席3問</x:v>
       </x:c>
-      <x:c r="D11" s="40" t="n">
+      <x:c r="D11" s="40" t="str">
+        <x:v>未選択</x:v>
+      </x:c>
+      <x:c r="E11" s="40" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E11" s="40" t="str">
+      <x:c r="F11" s="40" t="str">
         <x:v>HP→大切な人の物語→一緒に試す</x:v>
       </x:c>
-      <x:c r="F11" s="40" t="str">
-        <x:v>このスマホで一緒に3問試せます。続ける場合は、あとから本人のスマホでも使えます。</x:v>
-      </x:c>
       <x:c r="G11" s="40" t="str">
+        <x:v>このスマホで一緒に3問試せます。続ける場合は、本人のスマホをつなぐか、ご家族がおまかせで進められます。</x:v>
+      </x:c>
+      <x:c r="H11" s="40" t="str">
         <x:v>なし</x:v>
       </x:c>
-      <x:c r="H11" s="40" t="str">
-        <x:v>子</x:v>
-      </x:c>
       <x:c r="I11" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="J11" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K11" s="40" t="str">
         <x:v>未作成</x:v>
       </x:c>
-      <x:c r="K11" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="L11" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="M11" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="N11" s="40" t="str">
         <x:v>子端末</x:v>
       </x:c>
-      <x:c r="N11" s="40" t="str">
+      <x:c r="O11" s="40" t="str">
         <x:v>未登録</x:v>
       </x:c>
-      <x:c r="O11" s="40" t="str">
+      <x:c r="P11" s="40" t="str">
         <x:v>一緒に3問を選択</x:v>
       </x:c>
-      <x:c r="P11" s="40" t="str">
+      <x:c r="Q11" s="40" t="str">
         <x:v>子Account作成</x:v>
-      </x:c>
-      <x:c r="Q11" s="40" t="str">
-        <x:v>未</x:v>
       </x:c>
       <x:c r="R11" s="40" t="str">
         <x:v>未</x:v>
       </x:c>
       <x:c r="S11" s="40" t="str">
+        <x:v>未</x:v>
+      </x:c>
+      <x:c r="T11" s="40" t="str">
         <x:v>親なし</x:v>
       </x:c>
-      <x:c r="T11" s="40" t="str">
+      <x:c r="U11" s="40" t="str">
         <x:v>規約・支援説明</x:v>
       </x:c>
-      <x:c r="U11" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="V11" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="W11" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="X11" s="40" t="str">
         <x:v>子本人の試用とは分離</x:v>
       </x:c>
-      <x:c r="X11" s="40" t="str">
+      <x:c r="Y11" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="54" customHeight="1">
+    <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" s="43" t="str">
         <x:v>B-CO-020</x:v>
       </x:c>
@@ -1409,71 +1578,74 @@
       <x:c r="C12" s="40" t="str">
         <x:v>同席3問</x:v>
       </x:c>
-      <x:c r="D12" s="40" t="n">
+      <x:c r="D12" s="40" t="str">
+        <x:v>未選択→一緒に／おまかせ</x:v>
+      </x:c>
+      <x:c r="E12" s="40" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E12" s="40" t="str">
+      <x:c r="F12" s="40" t="str">
         <x:v>子Accountで親の姓名を登録</x:v>
       </x:c>
-      <x:c r="F12" s="40" t="str">
+      <x:c r="G12" s="40" t="str">
         <x:v>語る方のお名前を登録し、このスマホで3問を始めます。</x:v>
       </x:c>
-      <x:c r="G12" s="40" t="str">
-        <x:v>子</x:v>
-      </x:c>
       <x:c r="H12" s="40" t="str">
         <x:v>子</x:v>
       </x:c>
       <x:c r="I12" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="J12" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K12" s="40" t="str">
         <x:v>親</x:v>
       </x:c>
-      <x:c r="K12" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
       <x:c r="L12" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="M12" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N12" s="40" t="str">
         <x:v>子端末</x:v>
       </x:c>
-      <x:c r="N12" s="40" t="str">
+      <x:c r="O12" s="40" t="str">
         <x:v>子Account作成済／親Person未作成</x:v>
       </x:c>
-      <x:c r="O12" s="40" t="str">
+      <x:c r="P12" s="40" t="str">
         <x:v>親の記録を始める</x:v>
       </x:c>
-      <x:c r="P12" s="40" t="str">
+      <x:c r="Q12" s="40" t="str">
         <x:v>親Person・支援関係作成</x:v>
-      </x:c>
-      <x:c r="Q12" s="40" t="str">
-        <x:v>未</x:v>
       </x:c>
       <x:c r="R12" s="40" t="str">
         <x:v>未</x:v>
       </x:c>
       <x:c r="S12" s="40" t="str">
+        <x:v>未</x:v>
+      </x:c>
+      <x:c r="T12" s="40" t="str">
         <x:v>親なし</x:v>
       </x:c>
-      <x:c r="T12" s="40" t="str">
+      <x:c r="U12" s="40" t="str">
         <x:v>対象Person・支援・進捗説明</x:v>
       </x:c>
-      <x:c r="U12" s="40" t="str">
+      <x:c r="V12" s="40" t="str">
         <x:v>未設定</x:v>
       </x:c>
-      <x:c r="V12" s="40" t="str">
+      <x:c r="W12" s="40" t="str">
         <x:v>設定候補</x:v>
       </x:c>
-      <x:c r="W12" s="40" t="str">
+      <x:c r="X12" s="40" t="str">
         <x:v>actor Accountとsubject Personを分離</x:v>
       </x:c>
-      <x:c r="X12" s="40" t="str">
+      <x:c r="Y12" s="40" t="str">
         <x:v>要確認</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="54" customHeight="1">
+    <x:row r="13" ht="58" customHeight="1">
       <x:c r="A13" s="43" t="str">
         <x:v>B-CO-030</x:v>
       </x:c>
@@ -1483,71 +1655,74 @@
       <x:c r="C13" s="40" t="str">
         <x:v>同席3問</x:v>
       </x:c>
-      <x:c r="D13" s="40" t="n">
+      <x:c r="D13" s="40" t="str">
+        <x:v>一緒に／おまかせ</x:v>
+      </x:c>
+      <x:c r="E13" s="40" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E13" s="40" t="str">
+      <x:c r="F13" s="40" t="str">
         <x:v>子端末で母が3問を語る</x:v>
       </x:c>
-      <x:c r="F13" s="40" t="str">
+      <x:c r="G13" s="40" t="str">
         <x:v>3問のあと、購入して続けるか、今回はここまでにするか選べます。</x:v>
       </x:c>
-      <x:c r="G13" s="40" t="str">
-        <x:v>子</x:v>
-      </x:c>
       <x:c r="H13" s="40" t="str">
         <x:v>子</x:v>
       </x:c>
       <x:c r="I13" s="40" t="str">
-        <x:v>母</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="J13" s="40" t="str">
         <x:v>母</x:v>
       </x:c>
       <x:c r="K13" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>母</x:v>
       </x:c>
       <x:c r="L13" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="M13" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N13" s="40" t="str">
         <x:v>子iPhone</x:v>
       </x:c>
-      <x:c r="N13" s="40" t="str">
+      <x:c r="O13" s="40" t="str">
         <x:v>母Person作成済／未購入</x:v>
       </x:c>
-      <x:c r="O13" s="40" t="str">
+      <x:c r="P13" s="40" t="str">
         <x:v>3問完了</x:v>
       </x:c>
-      <x:c r="P13" s="40" t="str">
+      <x:c r="Q13" s="40" t="str">
         <x:v>体験完了／購入判断</x:v>
       </x:c>
-      <x:c r="Q13" s="40" t="str">
+      <x:c r="R13" s="40" t="str">
         <x:v>済</x:v>
       </x:c>
-      <x:c r="R13" s="40" t="str">
+      <x:c r="S13" s="40" t="str">
         <x:v>未</x:v>
       </x:c>
-      <x:c r="S13" s="40" t="str">
+      <x:c r="T13" s="40" t="str">
         <x:v>母なし</x:v>
       </x:c>
-      <x:c r="T13" s="40" t="str">
-        <x:v>語り共有初期値・進捗共有</x:v>
-      </x:c>
       <x:c r="U13" s="40" t="str">
-        <x:v>本人のみ</x:v>
+        <x:v>支援スタイル・語り共有・進捗共有</x:v>
       </x:c>
       <x:c r="V13" s="40" t="str">
-        <x:v>ON候補</x:v>
+        <x:v>制作Supporterと共有（語り単位で本人のみへ変更可）</x:v>
       </x:c>
       <x:c r="W13" s="40" t="str">
+        <x:v>共有</x:v>
+      </x:c>
+      <x:c r="X13" s="40" t="str">
         <x:v>Account＝子、語る人＝母、Person＝母</x:v>
       </x:c>
-      <x:c r="X13" s="40" t="str">
-        <x:v>要確認</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="54" customHeight="1">
+      <x:c r="Y13" s="40" t="str">
+        <x:v>確定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" s="43" t="str">
         <x:v>B-CO-GIFT-040</x:v>
       </x:c>
@@ -1557,195 +1732,201 @@
       <x:c r="C14" s="40" t="str">
         <x:v>同席3問・子購入</x:v>
       </x:c>
-      <x:c r="D14" s="40" t="n">
+      <x:c r="D14" s="40" t="str">
+        <x:v>一緒に／おまかせ</x:v>
+      </x:c>
+      <x:c r="E14" s="40" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E14" s="40" t="str">
+      <x:c r="F14" s="40" t="str">
         <x:v>子が購入して贈る</x:v>
       </x:c>
-      <x:c r="F14" s="40" t="str">
-        <x:v>購入後、本人のスマホへ続きを始める案内を送れます。</x:v>
-      </x:c>
       <x:c r="G14" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>購入後、本人のスマホで続けるか、ご家族がおまかせで進めるか選べます。</x:v>
       </x:c>
       <x:c r="H14" s="40" t="str">
         <x:v>子</x:v>
       </x:c>
       <x:c r="I14" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="J14" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K14" s="40" t="str">
         <x:v>母</x:v>
       </x:c>
-      <x:c r="K14" s="40" t="str">
-        <x:v>子</x:v>
-      </x:c>
       <x:c r="L14" s="40" t="str">
         <x:v>子</x:v>
       </x:c>
       <x:c r="M14" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N14" s="40" t="str">
         <x:v>子端末</x:v>
       </x:c>
-      <x:c r="N14" s="40" t="str">
+      <x:c r="O14" s="40" t="str">
         <x:v>体験完了／未購入</x:v>
       </x:c>
-      <x:c r="O14" s="40" t="str">
+      <x:c r="P14" s="40" t="str">
         <x:v>子が購入を確定</x:v>
       </x:c>
-      <x:c r="P14" s="40" t="str">
+      <x:c r="Q14" s="40" t="str">
         <x:v>支払済／母未接続</x:v>
-      </x:c>
-      <x:c r="Q14" s="40" t="str">
-        <x:v>済</x:v>
       </x:c>
       <x:c r="R14" s="40" t="str">
         <x:v>済</x:v>
       </x:c>
       <x:c r="S14" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="T14" s="40" t="str">
         <x:v>母なし</x:v>
       </x:c>
-      <x:c r="T14" s="40" t="str">
+      <x:c r="U14" s="40" t="str">
         <x:v>購入条件・45日保証</x:v>
       </x:c>
-      <x:c r="U14" s="40" t="str">
+      <x:c r="V14" s="40" t="str">
         <x:v>維持</x:v>
       </x:c>
-      <x:c r="V14" s="40" t="str">
+      <x:c r="W14" s="40" t="str">
         <x:v>設定通り</x:v>
       </x:c>
-      <x:c r="W14" s="40" t="str">
+      <x:c r="X14" s="40" t="str">
         <x:v>購入だけで本編開始しない</x:v>
       </x:c>
-      <x:c r="X14" s="40" t="str">
+      <x:c r="Y14" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="54" customHeight="1">
+    <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" s="43" t="str">
-        <x:v>B-CO-GIFT-050</x:v>
+        <x:v>B-CO-DELEGATED-050</x:v>
       </x:c>
       <x:c r="B15" s="40" t="str">
         <x:v>B 家族起点</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
-        <x:v>同席3問・子購入</x:v>
-      </x:c>
-      <x:c r="D15" s="40" t="n">
+        <x:v>同席3問・子購入・おまかせ</x:v>
+      </x:c>
+      <x:c r="D15" s="40" t="str">
+        <x:v>おまかせする</x:v>
+      </x:c>
+      <x:c r="E15" s="40" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E15" s="40" t="str">
-        <x:v>母：LINE等の案内→SMS OTP→既存Personへ接続</x:v>
-      </x:c>
       <x:c r="F15" s="40" t="str">
-        <x:v>本人確認後、同じ3問の続きから利用できます。</x:v>
+        <x:v>娘が母の了承を確認し、おまかせで進める</x:v>
       </x:c>
       <x:c r="G15" s="40" t="str">
+        <x:v>ご本人の意向を確認し、娘さんが制作を引き受けます。本人のAccountは必要ありません。</x:v>
+      </x:c>
+      <x:c r="H15" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="I15" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="J15" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K15" s="40" t="str">
         <x:v>母</x:v>
       </x:c>
-      <x:c r="H15" s="40" t="str">
-        <x:v>母</x:v>
-      </x:c>
-      <x:c r="I15" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="J15" s="40" t="str">
-        <x:v>母</x:v>
-      </x:c>
-      <x:c r="K15" s="40" t="str">
-        <x:v>子</x:v>
-      </x:c>
       <x:c r="L15" s="40" t="str">
         <x:v>子</x:v>
       </x:c>
       <x:c r="M15" s="40" t="str">
-        <x:v>母iPhone</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="N15" s="40" t="str">
-        <x:v>支払済／母未接続</x:v>
+        <x:v>子iPhone</x:v>
       </x:c>
       <x:c r="O15" s="40" t="str">
-        <x:v>母が本人接続へ同意しSMS認証</x:v>
+        <x:v>支払済／母Accountなし</x:v>
       </x:c>
       <x:c r="P15" s="40" t="str">
-        <x:v>母Account接続済／本編未開始</x:v>
+        <x:v>本人の了承を確認し、おまかせを選択</x:v>
       </x:c>
       <x:c r="Q15" s="40" t="str">
-        <x:v>済</x:v>
+        <x:v>娘が制作可能／本編未開始</x:v>
       </x:c>
       <x:c r="R15" s="40" t="str">
         <x:v>済</x:v>
       </x:c>
       <x:c r="S15" s="40" t="str">
-        <x:v>母SMS</x:v>
+        <x:v>済</x:v>
       </x:c>
       <x:c r="T15" s="40" t="str">
-        <x:v>本人接続・進捗共有</x:v>
+        <x:v>不要</x:v>
       </x:c>
       <x:c r="U15" s="40" t="str">
-        <x:v>本人権限</x:v>
+        <x:v>おまかせ確認・制作権限</x:v>
       </x:c>
       <x:c r="V15" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>制作Supporterと共有</x:v>
       </x:c>
       <x:c r="W15" s="40" t="str">
-        <x:v>新しいPerson・Projectを作らない</x:v>
+        <x:v>共有</x:v>
       </x:c>
       <x:c r="X15" s="40" t="str">
+        <x:v>support_mode＝おまかせ。本人Accountは任意</x:v>
+      </x:c>
+      <x:c r="Y15" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="54" customHeight="1">
+    <x:row r="16" ht="58" customHeight="1">
       <x:c r="A16" s="43" t="str">
-        <x:v>B-CO-GIFT-060</x:v>
+        <x:v>B-CO-DELEGATED-060</x:v>
       </x:c>
       <x:c r="B16" s="40" t="str">
         <x:v>B 家族起点</x:v>
       </x:c>
       <x:c r="C16" s="40" t="str">
-        <x:v>同席3問・子購入</x:v>
-      </x:c>
-      <x:c r="D16" s="40" t="n">
+        <x:v>同席3問・子購入・おまかせ</x:v>
+      </x:c>
+      <x:c r="D16" s="40" t="str">
+        <x:v>おまかせする</x:v>
+      </x:c>
+      <x:c r="E16" s="40" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="E16" s="40" t="str">
-        <x:v>母：はじまりの章→本編をはじめる</x:v>
-      </x:c>
       <x:c r="F16" s="40" t="str">
-        <x:v>本人は一人でも、ご家族と一緒でも続けられます。</x:v>
+        <x:v>娘が母の意思を確認して本編をはじめる</x:v>
       </x:c>
       <x:c r="G16" s="40" t="str">
+        <x:v>ご本人と続けることを確認したら、娘さんが本編開始を確定できます。</x:v>
+      </x:c>
+      <x:c r="H16" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="I16" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="J16" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K16" s="40" t="str">
         <x:v>母</x:v>
       </x:c>
-      <x:c r="H16" s="40" t="str">
-        <x:v>母</x:v>
-      </x:c>
-      <x:c r="I16" s="40" t="str">
-        <x:v>母</x:v>
-      </x:c>
-      <x:c r="J16" s="40" t="str">
-        <x:v>母</x:v>
-      </x:c>
-      <x:c r="K16" s="40" t="str">
-        <x:v>子</x:v>
-      </x:c>
       <x:c r="L16" s="40" t="str">
         <x:v>子</x:v>
       </x:c>
       <x:c r="M16" s="40" t="str">
-        <x:v>母iPhone</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="N16" s="40" t="str">
-        <x:v>支払済／母接続済／本編未開始</x:v>
+        <x:v>子iPhone</x:v>
       </x:c>
       <x:c r="O16" s="40" t="str">
-        <x:v>母が明示して本編開始</x:v>
+        <x:v>支払済／おまかせ設定済／本編未開始</x:v>
       </x:c>
       <x:c r="P16" s="40" t="str">
+        <x:v>本人の続行意思を確認した娘が本編開始</x:v>
+      </x:c>
+      <x:c r="Q16" s="40" t="str">
         <x:v>本編利用中／45日保証終了</x:v>
-      </x:c>
-      <x:c r="Q16" s="40" t="str">
-        <x:v>済</x:v>
       </x:c>
       <x:c r="R16" s="40" t="str">
         <x:v>済</x:v>
@@ -1754,569 +1935,593 @@
         <x:v>済</x:v>
       </x:c>
       <x:c r="T16" s="40" t="str">
+        <x:v>不要</x:v>
+      </x:c>
+      <x:c r="U16" s="40" t="str">
         <x:v>本編開始確認</x:v>
       </x:c>
-      <x:c r="U16" s="40" t="str">
-        <x:v>語りごと</x:v>
-      </x:c>
       <x:c r="V16" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>制作Supporterと共有</x:v>
       </x:c>
       <x:c r="W16" s="40" t="str">
-        <x:v>娘はSupporterのまま</x:v>
+        <x:v>共有</x:v>
       </x:c>
       <x:c r="X16" s="40" t="str">
+        <x:v>actor＝娘、subject＝母として開始を記録</x:v>
+      </x:c>
+      <x:c r="Y16" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="54" customHeight="1">
+    <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" s="43" t="str">
-        <x:v>B-REMOTE-010</x:v>
+        <x:v>B-CO-DELEGATED-070</x:v>
       </x:c>
       <x:c r="B17" s="40" t="str">
         <x:v>B 家族起点</x:v>
       </x:c>
       <x:c r="C17" s="40" t="str">
-        <x:v>遠隔3問</x:v>
-      </x:c>
-      <x:c r="D17" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E17" s="40" t="str">
-        <x:v>HP→大切な人の物語→本人に送る</x:v>
+        <x:v>同席3問・子購入・おまかせ</x:v>
+      </x:c>
+      <x:c r="D17" s="40" t="str">
+        <x:v>おまかせする</x:v>
+      </x:c>
+      <x:c r="E17" s="40" t="n">
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F17" s="40" t="str">
-        <x:v>LINEなどで3問を送り、本人の返答後に購入を決められます。</x:v>
+        <x:v>娘が遠隔で文章・写真・共有・本を仕上げる</x:v>
       </x:c>
       <x:c r="G17" s="40" t="str">
-        <x:v>なし</x:v>
+        <x:v>離れている時も、写真追加や文章整理、本への仕上げを進められます。</x:v>
       </x:c>
       <x:c r="H17" s="40" t="str">
         <x:v>子</x:v>
       </x:c>
       <x:c r="I17" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="J17" s="40" t="str">
-        <x:v>未作成</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="K17" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>母</x:v>
       </x:c>
       <x:c r="L17" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="M17" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N17" s="40" t="str">
         <x:v>子端末</x:v>
       </x:c>
-      <x:c r="N17" s="40" t="str">
-        <x:v>未登録</x:v>
-      </x:c>
       <x:c r="O17" s="40" t="str">
-        <x:v>本人に3問を送るを選択</x:v>
+        <x:v>本編利用中／母Accountなし</x:v>
       </x:c>
       <x:c r="P17" s="40" t="str">
-        <x:v>子Account作成</x:v>
+        <x:v>本人の意向を確認しながら制作</x:v>
       </x:c>
       <x:c r="Q17" s="40" t="str">
-        <x:v>招待予定</x:v>
+        <x:v>仕上げ・最終確定・製本注文</x:v>
       </x:c>
       <x:c r="R17" s="40" t="str">
-        <x:v>未</x:v>
+        <x:v>済</x:v>
       </x:c>
       <x:c r="S17" s="40" t="str">
-        <x:v>親なし</x:v>
+        <x:v>済</x:v>
       </x:c>
       <x:c r="T17" s="40" t="str">
-        <x:v>規約・支援説明</x:v>
+        <x:v>不要</x:v>
       </x:c>
       <x:c r="U17" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>共有・収録・Web・QR・最終確定</x:v>
       </x:c>
       <x:c r="V17" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>制作Supporterと共有（変更可）</x:v>
       </x:c>
       <x:c r="W17" s="40" t="str">
-        <x:v>Cはこのフローの受取人側ビュー</x:v>
+        <x:v>共有</x:v>
       </x:c>
       <x:c r="X17" s="40" t="str">
+        <x:v>本人Accountは後から任意で接続可能</x:v>
+      </x:c>
+      <x:c r="Y17" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="54" customHeight="1">
+    <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" s="43" t="str">
-        <x:v>B-REMOTE-020</x:v>
+        <x:v>B-CO-GIFT-050</x:v>
       </x:c>
       <x:c r="B18" s="40" t="str">
         <x:v>B 家族起点</x:v>
       </x:c>
       <x:c r="C18" s="40" t="str">
+        <x:v>同席3問・子購入</x:v>
+      </x:c>
+      <x:c r="D18" s="40" t="str">
+        <x:v>一緒に進める</x:v>
+      </x:c>
+      <x:c r="E18" s="40" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F18" s="40" t="str">
+        <x:v>母：LINE等の案内→SMS OTP→既存Personへ接続</x:v>
+      </x:c>
+      <x:c r="G18" s="40" t="str">
+        <x:v>本人確認後、同じ3問の続きから利用できます。</x:v>
+      </x:c>
+      <x:c r="H18" s="40" t="str">
+        <x:v>母</x:v>
+      </x:c>
+      <x:c r="I18" s="40" t="str">
+        <x:v>母</x:v>
+      </x:c>
+      <x:c r="J18" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K18" s="40" t="str">
+        <x:v>母</x:v>
+      </x:c>
+      <x:c r="L18" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="M18" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N18" s="40" t="str">
+        <x:v>母iPhone</x:v>
+      </x:c>
+      <x:c r="O18" s="40" t="str">
+        <x:v>支払済／母未接続</x:v>
+      </x:c>
+      <x:c r="P18" s="40" t="str">
+        <x:v>母が本人接続へ同意しSMS認証</x:v>
+      </x:c>
+      <x:c r="Q18" s="40" t="str">
+        <x:v>母Account接続済／本編未開始</x:v>
+      </x:c>
+      <x:c r="R18" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="S18" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="T18" s="40" t="str">
+        <x:v>母SMS</x:v>
+      </x:c>
+      <x:c r="U18" s="40" t="str">
+        <x:v>本人接続・進捗共有</x:v>
+      </x:c>
+      <x:c r="V18" s="40" t="str">
+        <x:v>本人権限</x:v>
+      </x:c>
+      <x:c r="W18" s="40" t="str">
+        <x:v>設定通り</x:v>
+      </x:c>
+      <x:c r="X18" s="40" t="str">
+        <x:v>新しいPerson・Projectを作らない</x:v>
+      </x:c>
+      <x:c r="Y18" s="40" t="str">
+        <x:v>確定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="58" customHeight="1">
+      <x:c r="A19" s="43" t="str">
+        <x:v>B-CO-GIFT-060</x:v>
+      </x:c>
+      <x:c r="B19" s="40" t="str">
+        <x:v>B 家族起点</x:v>
+      </x:c>
+      <x:c r="C19" s="40" t="str">
+        <x:v>同席3問・子購入</x:v>
+      </x:c>
+      <x:c r="D19" s="40" t="str">
+        <x:v>一緒に進める</x:v>
+      </x:c>
+      <x:c r="E19" s="40" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F19" s="40" t="str">
+        <x:v>母：はじまりの章→本編をはじめる</x:v>
+      </x:c>
+      <x:c r="G19" s="40" t="str">
+        <x:v>本人は一人でも、ご家族と一緒でも続けられます。</x:v>
+      </x:c>
+      <x:c r="H19" s="40" t="str">
+        <x:v>母</x:v>
+      </x:c>
+      <x:c r="I19" s="40" t="str">
+        <x:v>母</x:v>
+      </x:c>
+      <x:c r="J19" s="40" t="str">
+        <x:v>母</x:v>
+      </x:c>
+      <x:c r="K19" s="40" t="str">
+        <x:v>母</x:v>
+      </x:c>
+      <x:c r="L19" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="M19" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N19" s="40" t="str">
+        <x:v>母iPhone</x:v>
+      </x:c>
+      <x:c r="O19" s="40" t="str">
+        <x:v>支払済／母接続済／本編未開始</x:v>
+      </x:c>
+      <x:c r="P19" s="40" t="str">
+        <x:v>母が明示して本編開始</x:v>
+      </x:c>
+      <x:c r="Q19" s="40" t="str">
+        <x:v>本編利用中／45日保証終了</x:v>
+      </x:c>
+      <x:c r="R19" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="S19" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="T19" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="U19" s="40" t="str">
+        <x:v>本編開始確認</x:v>
+      </x:c>
+      <x:c r="V19" s="40" t="str">
+        <x:v>語りごと</x:v>
+      </x:c>
+      <x:c r="W19" s="40" t="str">
+        <x:v>設定通り</x:v>
+      </x:c>
+      <x:c r="X19" s="40" t="str">
+        <x:v>娘はSupporterのまま</x:v>
+      </x:c>
+      <x:c r="Y19" s="40" t="str">
+        <x:v>確定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="58" customHeight="1">
+      <x:c r="A20" s="43" t="str">
+        <x:v>B-REMOTE-010</x:v>
+      </x:c>
+      <x:c r="B20" s="40" t="str">
+        <x:v>B 家族起点</x:v>
+      </x:c>
+      <x:c r="C20" s="40" t="str">
         <x:v>遠隔3問</x:v>
       </x:c>
-      <x:c r="D18" s="40" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E18" s="40" t="str">
-        <x:v>子Accountで親Personを作り招待を送る</x:v>
-      </x:c>
-      <x:c r="F18" s="40" t="str">
-        <x:v>送信後は、本人が3問を終えるまでお待ちください。</x:v>
-      </x:c>
-      <x:c r="G18" s="40" t="str">
-        <x:v>子</x:v>
-      </x:c>
-      <x:c r="H18" s="40" t="str">
-        <x:v>子</x:v>
-      </x:c>
-      <x:c r="I18" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="J18" s="40" t="str">
-        <x:v>親</x:v>
-      </x:c>
-      <x:c r="K18" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="L18" s="40" t="str">
-        <x:v>子</x:v>
-      </x:c>
-      <x:c r="M18" s="40" t="str">
-        <x:v>子→親</x:v>
-      </x:c>
-      <x:c r="N18" s="40" t="str">
-        <x:v>親Person作成済／招待前</x:v>
-      </x:c>
-      <x:c r="O18" s="40" t="str">
-        <x:v>LINE・SMS・リンクで送信</x:v>
-      </x:c>
-      <x:c r="P18" s="40" t="str">
-        <x:v>招待中／未購入</x:v>
-      </x:c>
-      <x:c r="Q18" s="40" t="str">
-        <x:v>招待</x:v>
-      </x:c>
-      <x:c r="R18" s="40" t="str">
+      <x:c r="D20" s="40" t="str">
+        <x:v>未選択</x:v>
+      </x:c>
+      <x:c r="E20" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F20" s="40" t="str">
+        <x:v>HP→大切な人の物語→本人に送る</x:v>
+      </x:c>
+      <x:c r="G20" s="40" t="str">
+        <x:v>LINEなどで3問を送り、本人の返答後に購入を決められます。</x:v>
+      </x:c>
+      <x:c r="H20" s="40" t="str">
+        <x:v>なし</x:v>
+      </x:c>
+      <x:c r="I20" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="J20" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K20" s="40" t="str">
+        <x:v>未作成</x:v>
+      </x:c>
+      <x:c r="L20" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="M20" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="N20" s="40" t="str">
+        <x:v>子端末</x:v>
+      </x:c>
+      <x:c r="O20" s="40" t="str">
+        <x:v>未登録</x:v>
+      </x:c>
+      <x:c r="P20" s="40" t="str">
+        <x:v>本人に3問を送るを選択</x:v>
+      </x:c>
+      <x:c r="Q20" s="40" t="str">
+        <x:v>子Account作成</x:v>
+      </x:c>
+      <x:c r="R20" s="40" t="str">
+        <x:v>招待予定</x:v>
+      </x:c>
+      <x:c r="S20" s="40" t="str">
         <x:v>未</x:v>
       </x:c>
-      <x:c r="S18" s="40" t="str">
-        <x:v>親不要</x:v>
-      </x:c>
-      <x:c r="T18" s="40" t="str">
-        <x:v>招待・進捗説明</x:v>
-      </x:c>
-      <x:c r="U18" s="40" t="str">
-        <x:v>未設定</x:v>
-      </x:c>
-      <x:c r="V18" s="40" t="str">
-        <x:v>設定候補</x:v>
-      </x:c>
-      <x:c r="W18" s="40" t="str">
-        <x:v>送信成功を推定しない</x:v>
-      </x:c>
-      <x:c r="X18" s="40" t="str">
-        <x:v>要確認</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="54" customHeight="1">
-      <x:c r="A19" s="43" t="str">
-        <x:v>C-TRIAL-010</x:v>
-      </x:c>
-      <x:c r="B19" s="40" t="str">
-        <x:v>C 受取人側ビュー</x:v>
-      </x:c>
-      <x:c r="C19" s="40" t="str">
-        <x:v>B遠隔3問から派生</x:v>
-      </x:c>
-      <x:c r="D19" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E19" s="40" t="str">
-        <x:v>親：招待リンクを開いて3問を語る</x:v>
-      </x:c>
-      <x:c r="F19" s="40" t="str">
-        <x:v>この3問は無料です。Account登録をせずに体験できます。</x:v>
-      </x:c>
-      <x:c r="G19" s="40" t="str">
-        <x:v>なし（体験リンク）</x:v>
-      </x:c>
-      <x:c r="H19" s="40" t="str">
-        <x:v>親</x:v>
-      </x:c>
-      <x:c r="I19" s="40" t="str">
-        <x:v>親</x:v>
-      </x:c>
-      <x:c r="J19" s="40" t="str">
-        <x:v>親</x:v>
-      </x:c>
-      <x:c r="K19" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="L19" s="40" t="str">
-        <x:v>招待者</x:v>
-      </x:c>
-      <x:c r="M19" s="40" t="str">
-        <x:v>親端末</x:v>
-      </x:c>
-      <x:c r="N19" s="40" t="str">
-        <x:v>招待中／未購入</x:v>
-      </x:c>
-      <x:c r="O19" s="40" t="str">
-        <x:v>有効な体験リンクを開く</x:v>
-      </x:c>
-      <x:c r="P19" s="40" t="str">
-        <x:v>体験完了／続行意思待ち</x:v>
-      </x:c>
-      <x:c r="Q19" s="40" t="str">
-        <x:v>済</x:v>
-      </x:c>
-      <x:c r="R19" s="40" t="str">
-        <x:v>未</x:v>
-      </x:c>
-      <x:c r="S19" s="40" t="str">
-        <x:v>不要</x:v>
-      </x:c>
-      <x:c r="T19" s="40" t="str">
-        <x:v>体験同意</x:v>
-      </x:c>
-      <x:c r="U19" s="40" t="str">
-        <x:v>本人のみ</x:v>
-      </x:c>
-      <x:c r="V19" s="40" t="str">
-        <x:v>完了≠続行</x:v>
-      </x:c>
-      <x:c r="W19" s="40" t="str">
-        <x:v>Account登録を必須にしない</x:v>
-      </x:c>
-      <x:c r="X19" s="40" t="str">
+      <x:c r="T20" s="40" t="str">
+        <x:v>親なし</x:v>
+      </x:c>
+      <x:c r="U20" s="40" t="str">
+        <x:v>規約・支援説明</x:v>
+      </x:c>
+      <x:c r="V20" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="W20" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="X20" s="40" t="str">
+        <x:v>Cはこのフローの受取人側ビュー</x:v>
+      </x:c>
+      <x:c r="Y20" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="54" customHeight="1">
-      <x:c r="A20" s="43" t="str">
-        <x:v>C-TRIAL-020</x:v>
-      </x:c>
-      <x:c r="B20" s="40" t="str">
-        <x:v>C 受取人側ビュー</x:v>
-      </x:c>
-      <x:c r="C20" s="40" t="str">
-        <x:v>B遠隔3問から派生</x:v>
-      </x:c>
-      <x:c r="D20" s="40" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E20" s="40" t="str">
-        <x:v>親：続きをやってみたい／今回はここまでを選ぶ</x:v>
-      </x:c>
-      <x:c r="F20" s="40" t="str">
-        <x:v>続けたい場合だけご家族に知らせます。今回はここまででも構いません。</x:v>
-      </x:c>
-      <x:c r="G20" s="40" t="str">
-        <x:v>なし（体験リンク）</x:v>
-      </x:c>
-      <x:c r="H20" s="40" t="str">
-        <x:v>親</x:v>
-      </x:c>
-      <x:c r="I20" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="J20" s="40" t="str">
-        <x:v>親</x:v>
-      </x:c>
-      <x:c r="K20" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="L20" s="40" t="str">
-        <x:v>招待者</x:v>
-      </x:c>
-      <x:c r="M20" s="40" t="str">
-        <x:v>親端末</x:v>
-      </x:c>
-      <x:c r="N20" s="40" t="str">
-        <x:v>体験完了／未購入</x:v>
-      </x:c>
-      <x:c r="O20" s="40" t="str">
-        <x:v>親が続行希望を明示</x:v>
-      </x:c>
-      <x:c r="P20" s="40" t="str">
-        <x:v>購入者決定待ち</x:v>
-      </x:c>
-      <x:c r="Q20" s="40" t="str">
-        <x:v>済</x:v>
-      </x:c>
-      <x:c r="R20" s="40" t="str">
-        <x:v>未</x:v>
-      </x:c>
-      <x:c r="S20" s="40" t="str">
-        <x:v>不要</x:v>
-      </x:c>
-      <x:c r="T20" s="40" t="str">
-        <x:v>続行意思・通知先説明</x:v>
-      </x:c>
-      <x:c r="U20" s="40" t="str">
-        <x:v>維持</x:v>
-      </x:c>
-      <x:c r="V20" s="40" t="str">
-        <x:v>完了≠続行</x:v>
-      </x:c>
-      <x:c r="W20" s="40" t="str">
-        <x:v>Cは独立契約フローではない</x:v>
-      </x:c>
-      <x:c r="X20" s="40" t="str">
-        <x:v>確定</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="54" customHeight="1">
+    <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" s="43" t="str">
-        <x:v>B-REMOTE-GIFT-030</x:v>
+        <x:v>B-REMOTE-020</x:v>
       </x:c>
       <x:c r="B21" s="40" t="str">
         <x:v>B 家族起点</x:v>
       </x:c>
       <x:c r="C21" s="40" t="str">
-        <x:v>遠隔3問・子購入</x:v>
-      </x:c>
-      <x:c r="D21" s="40" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E21" s="40" t="str">
-        <x:v>子：続行希望の通知→購入して贈る</x:v>
+        <x:v>遠隔3問</x:v>
+      </x:c>
+      <x:c r="D21" s="40" t="str">
+        <x:v>本人が自分で／一緒に</x:v>
+      </x:c>
+      <x:c r="E21" s="40" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F21" s="40" t="str">
-        <x:v>本人が続けたいと答えた後、ご家族が購入して贈れます。</x:v>
+        <x:v>子Accountで親Personを作り招待を送る</x:v>
       </x:c>
       <x:c r="G21" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>送信後は、本人が3問を終えるまでお待ちください。</x:v>
       </x:c>
       <x:c r="H21" s="40" t="str">
         <x:v>子</x:v>
       </x:c>
       <x:c r="I21" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="J21" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K21" s="40" t="str">
         <x:v>親</x:v>
       </x:c>
-      <x:c r="K21" s="40" t="str">
-        <x:v>子</x:v>
-      </x:c>
       <x:c r="L21" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="M21" s="40" t="str">
-        <x:v>子端末</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="N21" s="40" t="str">
-        <x:v>続行希望／未購入</x:v>
+        <x:v>子→親</x:v>
       </x:c>
       <x:c r="O21" s="40" t="str">
-        <x:v>子が購入を選択</x:v>
+        <x:v>親Person作成済／招待前</x:v>
       </x:c>
       <x:c r="P21" s="40" t="str">
-        <x:v>支払済／親未接続</x:v>
+        <x:v>LINE・SMS・リンクで送信</x:v>
       </x:c>
       <x:c r="Q21" s="40" t="str">
-        <x:v>済</x:v>
+        <x:v>招待中／未購入</x:v>
       </x:c>
       <x:c r="R21" s="40" t="str">
-        <x:v>済</x:v>
+        <x:v>招待</x:v>
       </x:c>
       <x:c r="S21" s="40" t="str">
+        <x:v>未</x:v>
+      </x:c>
+      <x:c r="T21" s="40" t="str">
         <x:v>親不要</x:v>
       </x:c>
-      <x:c r="T21" s="40" t="str">
-        <x:v>購入条件・45日保証</x:v>
-      </x:c>
       <x:c r="U21" s="40" t="str">
-        <x:v>維持</x:v>
+        <x:v>招待・進捗説明</x:v>
       </x:c>
       <x:c r="V21" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>未設定</x:v>
       </x:c>
       <x:c r="W21" s="40" t="str">
-        <x:v>二重購入を防止</x:v>
+        <x:v>設定候補</x:v>
       </x:c>
       <x:c r="X21" s="40" t="str">
-        <x:v>確定</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="54" customHeight="1">
+        <x:v>送信成功を推定しない</x:v>
+      </x:c>
+      <x:c r="Y21" s="40" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" s="43" t="str">
-        <x:v>B-REMOTE-GIFT-040</x:v>
+        <x:v>C-TRIAL-010</x:v>
       </x:c>
       <x:c r="B22" s="40" t="str">
-        <x:v>B 家族起点</x:v>
+        <x:v>C 受取人側ビュー</x:v>
       </x:c>
       <x:c r="C22" s="40" t="str">
-        <x:v>遠隔3問・子購入</x:v>
-      </x:c>
-      <x:c r="D22" s="40" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="E22" s="40" t="str">
-        <x:v>親：SMS OTP→既存Personへ接続</x:v>
+        <x:v>B遠隔3問から派生</x:v>
+      </x:c>
+      <x:c r="D22" s="40" t="str">
+        <x:v>自分で進める</x:v>
+      </x:c>
+      <x:c r="E22" s="40" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F22" s="40" t="str">
-        <x:v>本人確認後、同じ3問の続きから利用できます。</x:v>
+        <x:v>親：招待リンクを開いて3問を語る</x:v>
       </x:c>
       <x:c r="G22" s="40" t="str">
+        <x:v>この3問は無料です。Account登録をせずに体験できます。</x:v>
+      </x:c>
+      <x:c r="H22" s="40" t="str">
+        <x:v>なし（体験リンク）</x:v>
+      </x:c>
+      <x:c r="I22" s="40" t="str">
         <x:v>親</x:v>
-      </x:c>
-      <x:c r="H22" s="40" t="str">
-        <x:v>親</x:v>
-      </x:c>
-      <x:c r="I22" s="40" t="str">
-        <x:v>—</x:v>
       </x:c>
       <x:c r="J22" s="40" t="str">
         <x:v>親</x:v>
       </x:c>
       <x:c r="K22" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>親</x:v>
       </x:c>
       <x:c r="L22" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="M22" s="40" t="str">
+        <x:v>招待者</x:v>
+      </x:c>
+      <x:c r="N22" s="40" t="str">
         <x:v>親端末</x:v>
       </x:c>
-      <x:c r="N22" s="40" t="str">
-        <x:v>支払済／親未接続</x:v>
-      </x:c>
       <x:c r="O22" s="40" t="str">
-        <x:v>親が本人接続へ同意しSMS認証</x:v>
+        <x:v>招待中／未購入</x:v>
       </x:c>
       <x:c r="P22" s="40" t="str">
-        <x:v>親Account接続済／本編未開始</x:v>
+        <x:v>有効な体験リンクを開く</x:v>
       </x:c>
       <x:c r="Q22" s="40" t="str">
-        <x:v>済</x:v>
+        <x:v>体験完了／続行意思待ち</x:v>
       </x:c>
       <x:c r="R22" s="40" t="str">
         <x:v>済</x:v>
       </x:c>
       <x:c r="S22" s="40" t="str">
-        <x:v>親SMS</x:v>
+        <x:v>未</x:v>
       </x:c>
       <x:c r="T22" s="40" t="str">
-        <x:v>本人接続・進捗共有</x:v>
+        <x:v>不要</x:v>
       </x:c>
       <x:c r="U22" s="40" t="str">
-        <x:v>本人権限</x:v>
+        <x:v>体験同意</x:v>
       </x:c>
       <x:c r="V22" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>本人のみ</x:v>
       </x:c>
       <x:c r="W22" s="40" t="str">
-        <x:v>45日保証は本編開始前まで</x:v>
+        <x:v>完了≠続行</x:v>
       </x:c>
       <x:c r="X22" s="40" t="str">
+        <x:v>Account登録を必須にしない</x:v>
+      </x:c>
+      <x:c r="Y22" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="54" customHeight="1">
+    <x:row r="23" ht="58" customHeight="1">
       <x:c r="A23" s="43" t="str">
-        <x:v>B-REMOTE-SELF-030</x:v>
+        <x:v>C-TRIAL-020</x:v>
       </x:c>
       <x:c r="B23" s="40" t="str">
-        <x:v>B 家族起点</x:v>
+        <x:v>C 受取人側ビュー</x:v>
       </x:c>
       <x:c r="C23" s="40" t="str">
-        <x:v>遠隔3問・本人購入</x:v>
-      </x:c>
-      <x:c r="D23" s="40" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E23" s="40" t="str">
-        <x:v>子：購入を本人にお願いする</x:v>
+        <x:v>B遠隔3問から派生</x:v>
+      </x:c>
+      <x:c r="D23" s="40" t="str">
+        <x:v>自分で進める</x:v>
+      </x:c>
+      <x:c r="E23" s="40" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F23" s="40" t="str">
-        <x:v>本人へ購入案内を送り、ご本人に手続きをお願いできます。</x:v>
+        <x:v>親：続きをやってみたい／今回はここまでを選ぶ</x:v>
       </x:c>
       <x:c r="G23" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>続けたい場合だけご家族に知らせます。今回はここまででも構いません。</x:v>
       </x:c>
       <x:c r="H23" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>なし（体験リンク）</x:v>
       </x:c>
       <x:c r="I23" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>親</x:v>
       </x:c>
       <x:c r="J23" s="40" t="str">
-        <x:v>親</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="K23" s="40" t="str">
         <x:v>親</x:v>
       </x:c>
       <x:c r="L23" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="M23" s="40" t="str">
-        <x:v>子端末</x:v>
+        <x:v>招待者</x:v>
       </x:c>
       <x:c r="N23" s="40" t="str">
-        <x:v>続行希望／未購入</x:v>
+        <x:v>親端末</x:v>
       </x:c>
       <x:c r="O23" s="40" t="str">
-        <x:v>子が本人購入案内を選択</x:v>
+        <x:v>体験完了／未購入</x:v>
       </x:c>
       <x:c r="P23" s="40" t="str">
-        <x:v>本人購入案内中</x:v>
+        <x:v>親が続行希望を明示</x:v>
       </x:c>
       <x:c r="Q23" s="40" t="str">
+        <x:v>購入者決定待ち</x:v>
+      </x:c>
+      <x:c r="R23" s="40" t="str">
         <x:v>済</x:v>
       </x:c>
-      <x:c r="R23" s="40" t="str">
+      <x:c r="S23" s="40" t="str">
         <x:v>未</x:v>
       </x:c>
-      <x:c r="S23" s="40" t="str">
-        <x:v>購入時に必要</x:v>
-      </x:c>
       <x:c r="T23" s="40" t="str">
-        <x:v>通知先・購入案内</x:v>
+        <x:v>不要</x:v>
       </x:c>
       <x:c r="U23" s="40" t="str">
+        <x:v>続行意思・通知先説明</x:v>
+      </x:c>
+      <x:c r="V23" s="40" t="str">
         <x:v>維持</x:v>
       </x:c>
-      <x:c r="V23" s="40" t="str">
-        <x:v>設定通り</x:v>
-      </x:c>
       <x:c r="W23" s="40" t="str">
-        <x:v>購入義務や代理課金ではない</x:v>
+        <x:v>完了≠続行</x:v>
       </x:c>
       <x:c r="X23" s="40" t="str">
+        <x:v>Cは独立契約フローではない</x:v>
+      </x:c>
+      <x:c r="Y23" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="54" customHeight="1">
+    <x:row r="24" ht="58" customHeight="1">
       <x:c r="A24" s="43" t="str">
-        <x:v>B-REMOTE-SELF-040</x:v>
+        <x:v>B-REMOTE-GIFT-030</x:v>
       </x:c>
       <x:c r="B24" s="40" t="str">
         <x:v>B 家族起点</x:v>
       </x:c>
       <x:c r="C24" s="40" t="str">
-        <x:v>遠隔3問・本人購入</x:v>
-      </x:c>
-      <x:c r="D24" s="40" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="E24" s="40" t="str">
-        <x:v>親：本人Accountへ接続して購入</x:v>
+        <x:v>遠隔3問・子購入</x:v>
+      </x:c>
+      <x:c r="D24" s="40" t="str">
+        <x:v>一緒に進める</x:v>
+      </x:c>
+      <x:c r="E24" s="40" t="n">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F24" s="40" t="str">
-        <x:v>本人確認と購入後、「はじまりの章」へ進みます。</x:v>
+        <x:v>子：続行希望の通知→購入して贈る</x:v>
       </x:c>
       <x:c r="G24" s="40" t="str">
-        <x:v>親（購入時接続）</x:v>
+        <x:v>本人が続けたいと答えた後、ご家族が購入して贈れます。</x:v>
       </x:c>
       <x:c r="H24" s="40" t="str">
-        <x:v>親</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="I24" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="J24" s="40" t="str">
-        <x:v>親</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="K24" s="40" t="str">
         <x:v>親</x:v>
@@ -2325,63 +2530,66 @@
         <x:v>子</x:v>
       </x:c>
       <x:c r="M24" s="40" t="str">
-        <x:v>親端末</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="N24" s="40" t="str">
-        <x:v>本人購入案内中</x:v>
+        <x:v>子端末</x:v>
       </x:c>
       <x:c r="O24" s="40" t="str">
-        <x:v>親が本人購入を確定</x:v>
+        <x:v>続行希望／未購入</x:v>
       </x:c>
       <x:c r="P24" s="40" t="str">
-        <x:v>支払済／本編未開始</x:v>
+        <x:v>子が購入を選択</x:v>
       </x:c>
       <x:c r="Q24" s="40" t="str">
-        <x:v>済</x:v>
+        <x:v>支払済／親未接続</x:v>
       </x:c>
       <x:c r="R24" s="40" t="str">
         <x:v>済</x:v>
       </x:c>
       <x:c r="S24" s="40" t="str">
-        <x:v>親SMS／要確認</x:v>
+        <x:v>済</x:v>
       </x:c>
       <x:c r="T24" s="40" t="str">
-        <x:v>本人接続・購入条件・30日保証</x:v>
+        <x:v>親不要</x:v>
       </x:c>
       <x:c r="U24" s="40" t="str">
-        <x:v>本人権限</x:v>
+        <x:v>購入条件・45日保証</x:v>
       </x:c>
       <x:c r="V24" s="40" t="str">
+        <x:v>維持</x:v>
+      </x:c>
+      <x:c r="W24" s="40" t="str">
         <x:v>設定通り</x:v>
       </x:c>
-      <x:c r="W24" s="40" t="str">
-        <x:v>購入とAccount接続の厳密な順序は要確認</x:v>
-      </x:c>
       <x:c r="X24" s="40" t="str">
-        <x:v>要確認</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="54" customHeight="1">
+        <x:v>二重購入を防止</x:v>
+      </x:c>
+      <x:c r="Y24" s="40" t="str">
+        <x:v>確定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="58" customHeight="1">
       <x:c r="A25" s="43" t="str">
-        <x:v>B-REMOTE-SELF-050</x:v>
+        <x:v>B-REMOTE-GIFT-040</x:v>
       </x:c>
       <x:c r="B25" s="40" t="str">
         <x:v>B 家族起点</x:v>
       </x:c>
       <x:c r="C25" s="40" t="str">
-        <x:v>遠隔3問・本人購入</x:v>
-      </x:c>
-      <x:c r="D25" s="40" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="E25" s="40" t="str">
-        <x:v>親：はじまりの章→本編をはじめる</x:v>
+        <x:v>遠隔3問・子購入</x:v>
+      </x:c>
+      <x:c r="D25" s="40" t="str">
+        <x:v>一緒に進める</x:v>
+      </x:c>
+      <x:c r="E25" s="40" t="n">
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F25" s="40" t="str">
-        <x:v>本編を開始すると、9つのテーマを順番に辿れます。</x:v>
+        <x:v>親：SMS OTP→既存Personへ接続</x:v>
       </x:c>
       <x:c r="G25" s="40" t="str">
-        <x:v>親</x:v>
+        <x:v>本人確認後、同じ3問の続きから利用できます。</x:v>
       </x:c>
       <x:c r="H25" s="40" t="str">
         <x:v>親</x:v>
@@ -2390,7 +2598,7 @@
         <x:v>親</x:v>
       </x:c>
       <x:c r="J25" s="40" t="str">
-        <x:v>親</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="K25" s="40" t="str">
         <x:v>親</x:v>
@@ -2399,19 +2607,19 @@
         <x:v>子</x:v>
       </x:c>
       <x:c r="M25" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N25" s="40" t="str">
         <x:v>親端末</x:v>
       </x:c>
-      <x:c r="N25" s="40" t="str">
-        <x:v>支払済／本編未開始</x:v>
-      </x:c>
       <x:c r="O25" s="40" t="str">
-        <x:v>親が明示して本編開始</x:v>
+        <x:v>支払済／親未接続</x:v>
       </x:c>
       <x:c r="P25" s="40" t="str">
-        <x:v>本編利用中／30日保証終了</x:v>
+        <x:v>親が本人接続へ同意しSMS認証</x:v>
       </x:c>
       <x:c r="Q25" s="40" t="str">
-        <x:v>済</x:v>
+        <x:v>親Account接続済／本編未開始</x:v>
       </x:c>
       <x:c r="R25" s="40" t="str">
         <x:v>済</x:v>
@@ -2420,190 +2628,199 @@
         <x:v>済</x:v>
       </x:c>
       <x:c r="T25" s="40" t="str">
-        <x:v>本編開始確認</x:v>
+        <x:v>親SMS</x:v>
       </x:c>
       <x:c r="U25" s="40" t="str">
-        <x:v>語りごと</x:v>
+        <x:v>本人接続・進捗共有</x:v>
       </x:c>
       <x:c r="V25" s="40" t="str">
+        <x:v>本人権限</x:v>
+      </x:c>
+      <x:c r="W25" s="40" t="str">
         <x:v>設定通り</x:v>
       </x:c>
-      <x:c r="W25" s="40" t="str">
-        <x:v>同じPersonを継続</x:v>
-      </x:c>
       <x:c r="X25" s="40" t="str">
+        <x:v>45日保証は本編開始前まで</x:v>
+      </x:c>
+      <x:c r="Y25" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="54" customHeight="1">
+    <x:row r="26" ht="58" customHeight="1">
       <x:c r="A26" s="43" t="str">
-        <x:v>B-DIRECT-GIFT-010</x:v>
+        <x:v>B-REMOTE-SELF-030</x:v>
       </x:c>
       <x:c r="B26" s="40" t="str">
         <x:v>B 家族起点</x:v>
       </x:c>
       <x:c r="C26" s="40" t="str">
-        <x:v>3問なし・子購入</x:v>
-      </x:c>
-      <x:c r="D26" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E26" s="40" t="str">
-        <x:v>HP→親に贈る→子が購入</x:v>
+        <x:v>遠隔3問・本人購入</x:v>
+      </x:c>
+      <x:c r="D26" s="40" t="str">
+        <x:v>自分で進める</x:v>
+      </x:c>
+      <x:c r="E26" s="40" t="n">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F26" s="40" t="str">
-        <x:v>無料体験をせずに購入し、本人へ開始案内を送れます。</x:v>
+        <x:v>子：購入を本人にお願いする</x:v>
       </x:c>
       <x:c r="G26" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>本人へ購入案内を送り、ご本人に手続きをお願いできます。</x:v>
       </x:c>
       <x:c r="H26" s="40" t="str">
         <x:v>子</x:v>
       </x:c>
       <x:c r="I26" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>子</x:v>
       </x:c>
       <x:c r="J26" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K26" s="40" t="str">
         <x:v>親</x:v>
       </x:c>
-      <x:c r="K26" s="40" t="str">
-        <x:v>子</x:v>
-      </x:c>
       <x:c r="L26" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>親</x:v>
       </x:c>
       <x:c r="M26" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N26" s="40" t="str">
         <x:v>子端末</x:v>
       </x:c>
-      <x:c r="N26" s="40" t="str">
-        <x:v>親Person作成済／未購入</x:v>
-      </x:c>
       <x:c r="O26" s="40" t="str">
-        <x:v>無料3問を経ずギフト購入</x:v>
+        <x:v>続行希望／未購入</x:v>
       </x:c>
       <x:c r="P26" s="40" t="str">
-        <x:v>支払済／親未接続</x:v>
+        <x:v>子が本人購入案内を選択</x:v>
       </x:c>
       <x:c r="Q26" s="40" t="str">
-        <x:v>なし</x:v>
+        <x:v>本人購入案内中</x:v>
       </x:c>
       <x:c r="R26" s="40" t="str">
         <x:v>済</x:v>
       </x:c>
       <x:c r="S26" s="40" t="str">
-        <x:v>親未</x:v>
+        <x:v>未</x:v>
       </x:c>
       <x:c r="T26" s="40" t="str">
-        <x:v>購入条件・45日保証</x:v>
+        <x:v>購入時に必要</x:v>
       </x:c>
       <x:c r="U26" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>通知先・購入案内</x:v>
       </x:c>
       <x:c r="V26" s="40" t="str">
-        <x:v>設定候補</x:v>
+        <x:v>維持</x:v>
       </x:c>
       <x:c r="W26" s="40" t="str">
-        <x:v>購入だけで本編開始しない</x:v>
+        <x:v>設定通り</x:v>
       </x:c>
       <x:c r="X26" s="40" t="str">
+        <x:v>購入義務や代理課金ではない</x:v>
+      </x:c>
+      <x:c r="Y26" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="54" customHeight="1">
+    <x:row r="27" ht="58" customHeight="1">
       <x:c r="A27" s="43" t="str">
-        <x:v>B-DIRECT-GIFT-020</x:v>
+        <x:v>B-REMOTE-SELF-040</x:v>
       </x:c>
       <x:c r="B27" s="40" t="str">
         <x:v>B 家族起点</x:v>
       </x:c>
       <x:c r="C27" s="40" t="str">
-        <x:v>3問なし・子購入</x:v>
-      </x:c>
-      <x:c r="D27" s="40" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E27" s="40" t="str">
-        <x:v>親：案内→SMS OTP→既存Personへ接続</x:v>
+        <x:v>遠隔3問・本人購入</x:v>
+      </x:c>
+      <x:c r="D27" s="40" t="str">
+        <x:v>自分で進める</x:v>
+      </x:c>
+      <x:c r="E27" s="40" t="n">
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F27" s="40" t="str">
-        <x:v>本人確認後、「はじまりの章」から始められます。</x:v>
+        <x:v>親：本人Accountへ接続して購入</x:v>
       </x:c>
       <x:c r="G27" s="40" t="str">
+        <x:v>本人確認と購入後、「はじまりの章」へ進みます。</x:v>
+      </x:c>
+      <x:c r="H27" s="40" t="str">
+        <x:v>親（購入時接続）</x:v>
+      </x:c>
+      <x:c r="I27" s="40" t="str">
         <x:v>親</x:v>
       </x:c>
-      <x:c r="H27" s="40" t="str">
+      <x:c r="J27" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K27" s="40" t="str">
         <x:v>親</x:v>
       </x:c>
-      <x:c r="I27" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="J27" s="40" t="str">
+      <x:c r="L27" s="40" t="str">
         <x:v>親</x:v>
       </x:c>
-      <x:c r="K27" s="40" t="str">
-        <x:v>子</x:v>
-      </x:c>
-      <x:c r="L27" s="40" t="str">
-        <x:v>子</x:v>
-      </x:c>
       <x:c r="M27" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N27" s="40" t="str">
         <x:v>親端末</x:v>
       </x:c>
-      <x:c r="N27" s="40" t="str">
-        <x:v>支払済／親未接続</x:v>
-      </x:c>
       <x:c r="O27" s="40" t="str">
-        <x:v>親が本人接続へ同意しSMS認証</x:v>
+        <x:v>本人購入案内中</x:v>
       </x:c>
       <x:c r="P27" s="40" t="str">
-        <x:v>親Account接続済／本編未開始</x:v>
+        <x:v>親が本人購入を確定</x:v>
       </x:c>
       <x:c r="Q27" s="40" t="str">
-        <x:v>なし</x:v>
+        <x:v>支払済／本編未開始</x:v>
       </x:c>
       <x:c r="R27" s="40" t="str">
         <x:v>済</x:v>
       </x:c>
       <x:c r="S27" s="40" t="str">
-        <x:v>親SMS</x:v>
+        <x:v>済</x:v>
       </x:c>
       <x:c r="T27" s="40" t="str">
-        <x:v>本人接続・進捗共有</x:v>
+        <x:v>親SMS／要確認</x:v>
       </x:c>
       <x:c r="U27" s="40" t="str">
+        <x:v>本人接続・購入条件・30日保証</x:v>
+      </x:c>
+      <x:c r="V27" s="40" t="str">
         <x:v>本人権限</x:v>
       </x:c>
-      <x:c r="V27" s="40" t="str">
+      <x:c r="W27" s="40" t="str">
         <x:v>設定通り</x:v>
       </x:c>
-      <x:c r="W27" s="40" t="str">
-        <x:v>同じPerson・Projectへ接続</x:v>
-      </x:c>
       <x:c r="X27" s="40" t="str">
-        <x:v>確定</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="54" customHeight="1">
+        <x:v>購入とAccount接続の厳密な順序は要確認</x:v>
+      </x:c>
+      <x:c r="Y27" s="40" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="58" customHeight="1">
       <x:c r="A28" s="43" t="str">
-        <x:v>B-DIRECT-GIFT-030</x:v>
+        <x:v>B-REMOTE-SELF-050</x:v>
       </x:c>
       <x:c r="B28" s="40" t="str">
         <x:v>B 家族起点</x:v>
       </x:c>
       <x:c r="C28" s="40" t="str">
-        <x:v>3問なし・子購入</x:v>
-      </x:c>
-      <x:c r="D28" s="40" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E28" s="40" t="str">
+        <x:v>遠隔3問・本人購入</x:v>
+      </x:c>
+      <x:c r="D28" s="40" t="str">
+        <x:v>自分で進める</x:v>
+      </x:c>
+      <x:c r="E28" s="40" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F28" s="40" t="str">
         <x:v>親：はじまりの章→本編をはじめる</x:v>
       </x:c>
-      <x:c r="F28" s="40" t="str">
-        <x:v>本人は一人でも、ご家族と一緒でも続けられます。</x:v>
-      </x:c>
       <x:c r="G28" s="40" t="str">
-        <x:v>親</x:v>
+        <x:v>本編を開始すると、9つのテーマを順番に辿れます。</x:v>
       </x:c>
       <x:c r="H28" s="40" t="str">
         <x:v>親</x:v>
@@ -2615,25 +2832,25 @@
         <x:v>親</x:v>
       </x:c>
       <x:c r="K28" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>親</x:v>
       </x:c>
       <x:c r="L28" s="40" t="str">
-        <x:v>子</x:v>
+        <x:v>親</x:v>
       </x:c>
       <x:c r="M28" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N28" s="40" t="str">
         <x:v>親端末</x:v>
       </x:c>
-      <x:c r="N28" s="40" t="str">
-        <x:v>支払済／親接続済／本編未開始</x:v>
-      </x:c>
       <x:c r="O28" s="40" t="str">
+        <x:v>支払済／本編未開始</x:v>
+      </x:c>
+      <x:c r="P28" s="40" t="str">
         <x:v>親が明示して本編開始</x:v>
       </x:c>
-      <x:c r="P28" s="40" t="str">
-        <x:v>本編利用中／45日保証終了</x:v>
-      </x:c>
       <x:c r="Q28" s="40" t="str">
-        <x:v>なし</x:v>
+        <x:v>本編利用中／30日保証終了</x:v>
       </x:c>
       <x:c r="R28" s="40" t="str">
         <x:v>済</x:v>
@@ -2642,25 +2859,490 @@
         <x:v>済</x:v>
       </x:c>
       <x:c r="T28" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="U28" s="40" t="str">
         <x:v>本編開始確認</x:v>
       </x:c>
-      <x:c r="U28" s="40" t="str">
+      <x:c r="V28" s="40" t="str">
         <x:v>語りごと</x:v>
       </x:c>
-      <x:c r="V28" s="40" t="str">
+      <x:c r="W28" s="40" t="str">
         <x:v>設定通り</x:v>
       </x:c>
-      <x:c r="W28" s="40" t="str">
+      <x:c r="X28" s="40" t="str">
+        <x:v>同じPersonを継続</x:v>
+      </x:c>
+      <x:c r="Y28" s="40" t="str">
+        <x:v>確定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="58" customHeight="1">
+      <x:c r="A29" s="43" t="str">
+        <x:v>B-DIRECT-GIFT-010</x:v>
+      </x:c>
+      <x:c r="B29" s="40" t="str">
+        <x:v>B 家族起点</x:v>
+      </x:c>
+      <x:c r="C29" s="40" t="str">
+        <x:v>3問なし・子購入</x:v>
+      </x:c>
+      <x:c r="D29" s="40" t="str">
+        <x:v>未選択→一緒に／おまかせ</x:v>
+      </x:c>
+      <x:c r="E29" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F29" s="40" t="str">
+        <x:v>HP→親に贈る→子が購入</x:v>
+      </x:c>
+      <x:c r="G29" s="40" t="str">
+        <x:v>無料体験をせずに購入し、本人接続か、ご家族のおまかせかを選べます。</x:v>
+      </x:c>
+      <x:c r="H29" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="I29" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="J29" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K29" s="40" t="str">
+        <x:v>親</x:v>
+      </x:c>
+      <x:c r="L29" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="M29" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N29" s="40" t="str">
+        <x:v>子端末</x:v>
+      </x:c>
+      <x:c r="O29" s="40" t="str">
+        <x:v>親Person作成済／未購入</x:v>
+      </x:c>
+      <x:c r="P29" s="40" t="str">
+        <x:v>無料3問を経ずギフト購入</x:v>
+      </x:c>
+      <x:c r="Q29" s="40" t="str">
+        <x:v>支払済／支援スタイル選択待ち</x:v>
+      </x:c>
+      <x:c r="R29" s="40" t="str">
+        <x:v>なし</x:v>
+      </x:c>
+      <x:c r="S29" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="T29" s="40" t="str">
+        <x:v>親未</x:v>
+      </x:c>
+      <x:c r="U29" s="40" t="str">
+        <x:v>購入条件・45日保証・支援スタイル</x:v>
+      </x:c>
+      <x:c r="V29" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="W29" s="40" t="str">
+        <x:v>設定候補</x:v>
+      </x:c>
+      <x:c r="X29" s="40" t="str">
+        <x:v>購入だけで本編開始しない</x:v>
+      </x:c>
+      <x:c r="Y29" s="40" t="str">
+        <x:v>確定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="58" customHeight="1">
+      <x:c r="A30" s="43" t="str">
+        <x:v>B-DIRECT-DELEGATED-020</x:v>
+      </x:c>
+      <x:c r="B30" s="40" t="str">
+        <x:v>B 家族起点</x:v>
+      </x:c>
+      <x:c r="C30" s="40" t="str">
+        <x:v>3問なし・子購入・おまかせ</x:v>
+      </x:c>
+      <x:c r="D30" s="40" t="str">
+        <x:v>おまかせする</x:v>
+      </x:c>
+      <x:c r="E30" s="40" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F30" s="40" t="str">
+        <x:v>子が本人の了承を確認し、おまかせで進める</x:v>
+      </x:c>
+      <x:c r="G30" s="40" t="str">
+        <x:v>ご本人の意向を確認し、ご家族が制作を引き受けます。本人のAccountは必要ありません。</x:v>
+      </x:c>
+      <x:c r="H30" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="I30" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="J30" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K30" s="40" t="str">
+        <x:v>親</x:v>
+      </x:c>
+      <x:c r="L30" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="M30" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N30" s="40" t="str">
+        <x:v>子端末</x:v>
+      </x:c>
+      <x:c r="O30" s="40" t="str">
+        <x:v>支払済／親Accountなし</x:v>
+      </x:c>
+      <x:c r="P30" s="40" t="str">
+        <x:v>本人の了承を確認し、おまかせを選択</x:v>
+      </x:c>
+      <x:c r="Q30" s="40" t="str">
+        <x:v>子が制作可能／本編未開始</x:v>
+      </x:c>
+      <x:c r="R30" s="40" t="str">
+        <x:v>なし</x:v>
+      </x:c>
+      <x:c r="S30" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="T30" s="40" t="str">
+        <x:v>不要</x:v>
+      </x:c>
+      <x:c r="U30" s="40" t="str">
+        <x:v>おまかせ確認・制作権限</x:v>
+      </x:c>
+      <x:c r="V30" s="40" t="str">
+        <x:v>制作Supporterと共有</x:v>
+      </x:c>
+      <x:c r="W30" s="40" t="str">
+        <x:v>共有</x:v>
+      </x:c>
+      <x:c r="X30" s="40" t="str">
+        <x:v>support_mode＝おまかせ。本人Accountは任意</x:v>
+      </x:c>
+      <x:c r="Y30" s="40" t="str">
+        <x:v>確定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="58" customHeight="1">
+      <x:c r="A31" s="43" t="str">
+        <x:v>B-DIRECT-DELEGATED-030</x:v>
+      </x:c>
+      <x:c r="B31" s="40" t="str">
+        <x:v>B 家族起点</x:v>
+      </x:c>
+      <x:c r="C31" s="40" t="str">
+        <x:v>3問なし・子購入・おまかせ</x:v>
+      </x:c>
+      <x:c r="D31" s="40" t="str">
+        <x:v>おまかせする</x:v>
+      </x:c>
+      <x:c r="E31" s="40" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F31" s="40" t="str">
+        <x:v>子が本人の意思を確認して本編をはじめる</x:v>
+      </x:c>
+      <x:c r="G31" s="40" t="str">
+        <x:v>ご本人と続けることを確認したら、ご家族が本編開始を確定できます。</x:v>
+      </x:c>
+      <x:c r="H31" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="I31" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="J31" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K31" s="40" t="str">
+        <x:v>親</x:v>
+      </x:c>
+      <x:c r="L31" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="M31" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N31" s="40" t="str">
+        <x:v>子端末</x:v>
+      </x:c>
+      <x:c r="O31" s="40" t="str">
+        <x:v>支払済／おまかせ設定済／本編未開始</x:v>
+      </x:c>
+      <x:c r="P31" s="40" t="str">
+        <x:v>本人の続行意思を確認した子が本編開始</x:v>
+      </x:c>
+      <x:c r="Q31" s="40" t="str">
+        <x:v>本編利用中／45日保証終了</x:v>
+      </x:c>
+      <x:c r="R31" s="40" t="str">
+        <x:v>なし</x:v>
+      </x:c>
+      <x:c r="S31" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="T31" s="40" t="str">
+        <x:v>不要</x:v>
+      </x:c>
+      <x:c r="U31" s="40" t="str">
+        <x:v>本編開始確認</x:v>
+      </x:c>
+      <x:c r="V31" s="40" t="str">
+        <x:v>制作Supporterと共有</x:v>
+      </x:c>
+      <x:c r="W31" s="40" t="str">
+        <x:v>共有</x:v>
+      </x:c>
+      <x:c r="X31" s="40" t="str">
+        <x:v>actor＝子、subject＝親として開始を記録</x:v>
+      </x:c>
+      <x:c r="Y31" s="40" t="str">
+        <x:v>確定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="58" customHeight="1">
+      <x:c r="A32" s="43" t="str">
+        <x:v>B-DIRECT-DELEGATED-040</x:v>
+      </x:c>
+      <x:c r="B32" s="40" t="str">
+        <x:v>B 家族起点</x:v>
+      </x:c>
+      <x:c r="C32" s="40" t="str">
+        <x:v>3問なし・子購入・おまかせ</x:v>
+      </x:c>
+      <x:c r="D32" s="40" t="str">
+        <x:v>おまかせする</x:v>
+      </x:c>
+      <x:c r="E32" s="40" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F32" s="40" t="str">
+        <x:v>子が文章・写真・共有・本を仕上げる</x:v>
+      </x:c>
+      <x:c r="G32" s="40" t="str">
+        <x:v>写真追加や文章整理、本への仕上げ、製本注文まで進められます。</x:v>
+      </x:c>
+      <x:c r="H32" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="I32" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="J32" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K32" s="40" t="str">
+        <x:v>親</x:v>
+      </x:c>
+      <x:c r="L32" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="M32" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N32" s="40" t="str">
+        <x:v>子端末</x:v>
+      </x:c>
+      <x:c r="O32" s="40" t="str">
+        <x:v>本編利用中／親Accountなし</x:v>
+      </x:c>
+      <x:c r="P32" s="40" t="str">
+        <x:v>本人の意向を確認しながら制作</x:v>
+      </x:c>
+      <x:c r="Q32" s="40" t="str">
+        <x:v>仕上げ・最終確定・製本注文</x:v>
+      </x:c>
+      <x:c r="R32" s="40" t="str">
+        <x:v>なし</x:v>
+      </x:c>
+      <x:c r="S32" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="T32" s="40" t="str">
+        <x:v>不要</x:v>
+      </x:c>
+      <x:c r="U32" s="40" t="str">
+        <x:v>共有・収録・Web・QR・最終確定</x:v>
+      </x:c>
+      <x:c r="V32" s="40" t="str">
+        <x:v>制作Supporterと共有（変更可）</x:v>
+      </x:c>
+      <x:c r="W32" s="40" t="str">
+        <x:v>共有</x:v>
+      </x:c>
+      <x:c r="X32" s="40" t="str">
+        <x:v>本人Accountは後から任意で接続可能</x:v>
+      </x:c>
+      <x:c r="Y32" s="40" t="str">
+        <x:v>確定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="58" customHeight="1">
+      <x:c r="A33" s="43" t="str">
+        <x:v>B-DIRECT-GIFT-020</x:v>
+      </x:c>
+      <x:c r="B33" s="40" t="str">
+        <x:v>B 家族起点</x:v>
+      </x:c>
+      <x:c r="C33" s="40" t="str">
+        <x:v>3問なし・子購入</x:v>
+      </x:c>
+      <x:c r="D33" s="40" t="str">
+        <x:v>一緒に進める</x:v>
+      </x:c>
+      <x:c r="E33" s="40" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F33" s="40" t="str">
+        <x:v>親：案内→SMS OTP→既存Personへ接続</x:v>
+      </x:c>
+      <x:c r="G33" s="40" t="str">
+        <x:v>本人確認後、「はじまりの章」から始められます。</x:v>
+      </x:c>
+      <x:c r="H33" s="40" t="str">
+        <x:v>親</x:v>
+      </x:c>
+      <x:c r="I33" s="40" t="str">
+        <x:v>親</x:v>
+      </x:c>
+      <x:c r="J33" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K33" s="40" t="str">
+        <x:v>親</x:v>
+      </x:c>
+      <x:c r="L33" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="M33" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N33" s="40" t="str">
+        <x:v>親端末</x:v>
+      </x:c>
+      <x:c r="O33" s="40" t="str">
+        <x:v>支払済／親未接続</x:v>
+      </x:c>
+      <x:c r="P33" s="40" t="str">
+        <x:v>親が本人接続へ同意しSMS認証</x:v>
+      </x:c>
+      <x:c r="Q33" s="40" t="str">
+        <x:v>親Account接続済／本編未開始</x:v>
+      </x:c>
+      <x:c r="R33" s="40" t="str">
+        <x:v>なし</x:v>
+      </x:c>
+      <x:c r="S33" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="T33" s="40" t="str">
+        <x:v>親SMS</x:v>
+      </x:c>
+      <x:c r="U33" s="40" t="str">
+        <x:v>本人接続・進捗共有</x:v>
+      </x:c>
+      <x:c r="V33" s="40" t="str">
+        <x:v>本人権限</x:v>
+      </x:c>
+      <x:c r="W33" s="40" t="str">
+        <x:v>設定通り</x:v>
+      </x:c>
+      <x:c r="X33" s="40" t="str">
+        <x:v>同じPerson・Projectへ接続</x:v>
+      </x:c>
+      <x:c r="Y33" s="40" t="str">
+        <x:v>確定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="58" customHeight="1">
+      <x:c r="A34" s="43" t="str">
+        <x:v>B-DIRECT-GIFT-030</x:v>
+      </x:c>
+      <x:c r="B34" s="40" t="str">
+        <x:v>B 家族起点</x:v>
+      </x:c>
+      <x:c r="C34" s="40" t="str">
+        <x:v>3問なし・子購入</x:v>
+      </x:c>
+      <x:c r="D34" s="40" t="str">
+        <x:v>一緒に進める</x:v>
+      </x:c>
+      <x:c r="E34" s="40" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F34" s="40" t="str">
+        <x:v>親：はじまりの章→本編をはじめる</x:v>
+      </x:c>
+      <x:c r="G34" s="40" t="str">
+        <x:v>本人は一人でも、ご家族と一緒でも続けられます。</x:v>
+      </x:c>
+      <x:c r="H34" s="40" t="str">
+        <x:v>親</x:v>
+      </x:c>
+      <x:c r="I34" s="40" t="str">
+        <x:v>親</x:v>
+      </x:c>
+      <x:c r="J34" s="40" t="str">
+        <x:v>親</x:v>
+      </x:c>
+      <x:c r="K34" s="40" t="str">
+        <x:v>親</x:v>
+      </x:c>
+      <x:c r="L34" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="M34" s="40" t="str">
+        <x:v>子</x:v>
+      </x:c>
+      <x:c r="N34" s="40" t="str">
+        <x:v>親端末</x:v>
+      </x:c>
+      <x:c r="O34" s="40" t="str">
+        <x:v>支払済／親接続済／本編未開始</x:v>
+      </x:c>
+      <x:c r="P34" s="40" t="str">
+        <x:v>親が明示して本編開始</x:v>
+      </x:c>
+      <x:c r="Q34" s="40" t="str">
+        <x:v>本編利用中／45日保証終了</x:v>
+      </x:c>
+      <x:c r="R34" s="40" t="str">
+        <x:v>なし</x:v>
+      </x:c>
+      <x:c r="S34" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="T34" s="40" t="str">
+        <x:v>済</x:v>
+      </x:c>
+      <x:c r="U34" s="40" t="str">
+        <x:v>本編開始確認</x:v>
+      </x:c>
+      <x:c r="V34" s="40" t="str">
+        <x:v>語りごと</x:v>
+      </x:c>
+      <x:c r="W34" s="40" t="str">
+        <x:v>設定通り</x:v>
+      </x:c>
+      <x:c r="X34" s="40" t="str">
         <x:v>娘はSupporterのまま</x:v>
       </x:c>
-      <x:c r="X28" s="40" t="str">
+      <x:c r="Y34" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:X1"/>
-    <x:mergeCell ref="A2:X2"/>
+    <x:mergeCell ref="A1:Y1"/>
+    <x:mergeCell ref="A2:Y2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A5:X28">
     <x:cfRule type="expression" dxfId="0" priority="1">
@@ -2673,8 +3355,19 @@
       <x:formula>$X5="要確認"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:conditionalFormatting sqref="A5:Y34">
+    <x:cfRule type="expression" dxfId="9" priority="4">
+      <x:formula>$Y5="要確認"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="12" priority="5">
+      <x:formula>$Y5="要確認"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="X5:X28">
+      <x:formula1>"確定,要確認"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="Y5:Y34">
       <x:formula1>"確定,要確認"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -2747,44 +3440,44 @@
       <x:c r="L3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="54" t="str">
+      <x:c r="A4" s="70" t="str">
         <x:v>Setting ID</x:v>
       </x:c>
-      <x:c r="B4" s="54" t="str">
+      <x:c r="B4" s="70" t="str">
         <x:v>設定・同意</x:v>
       </x:c>
-      <x:c r="C4" s="54" t="str">
+      <x:c r="C4" s="70" t="str">
         <x:v>Account登録</x:v>
       </x:c>
-      <x:c r="D4" s="54" t="str">
+      <x:c r="D4" s="70" t="str">
         <x:v>対象Person作成</x:v>
       </x:c>
-      <x:c r="E4" s="54" t="str">
+      <x:c r="E4" s="70" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="F4" s="54" t="str">
+      <x:c r="F4" s="70" t="str">
         <x:v>購入</x:v>
       </x:c>
-      <x:c r="G4" s="54" t="str">
+      <x:c r="G4" s="70" t="str">
         <x:v>本人接続</x:v>
       </x:c>
-      <x:c r="H4" s="54" t="str">
+      <x:c r="H4" s="70" t="str">
         <x:v>本編開始</x:v>
       </x:c>
-      <x:c r="I4" s="54" t="str">
+      <x:c r="I4" s="70" t="str">
         <x:v>制作中</x:v>
       </x:c>
-      <x:c r="J4" s="54" t="str">
+      <x:c r="J4" s="70" t="str">
         <x:v>仕上げ</x:v>
       </x:c>
-      <x:c r="K4" s="54" t="str">
+      <x:c r="K4" s="70" t="str">
         <x:v>完成後</x:v>
       </x:c>
-      <x:c r="L4" s="54" t="str">
+      <x:c r="L4" s="70" t="str">
         <x:v>備考</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="40" customHeight="1">
+    <x:row r="5" ht="44" customHeight="1">
       <x:c r="A5" s="40" t="str">
         <x:v>S01</x:v>
       </x:c>
@@ -2822,7 +3515,7 @@
         <x:v>登録時を基本</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="40" customHeight="1">
+    <x:row r="6" ht="44" customHeight="1">
       <x:c r="A6" s="40" t="str">
         <x:v>S02</x:v>
       </x:c>
@@ -2860,7 +3553,7 @@
         <x:v>本人起点ではAccount登録とPerson作成が同時の場合あり</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="40" customHeight="1">
+    <x:row r="7" ht="44" customHeight="1">
       <x:c r="A7" s="40" t="str">
         <x:v>S03</x:v>
       </x:c>
@@ -2898,7 +3591,7 @@
         <x:v>本人に短く説明、停止可</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="40" customHeight="1">
+    <x:row r="8" ht="44" customHeight="1">
       <x:c r="A8" s="40" t="str">
         <x:v>S04</x:v>
       </x:c>
@@ -2933,15 +3626,15 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="L8" s="40" t="str">
-        <x:v>内容共有とは別</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="40" customHeight="1">
+        <x:v>自分で＝任意。一緒に・おまかせ＝制作Supporterへ共有</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="44" customHeight="1">
       <x:c r="A9" s="40" t="str">
         <x:v>S05</x:v>
       </x:c>
       <x:c r="B9" s="40" t="str">
-        <x:v>語り共有 本人のみ／家族</x:v>
+        <x:v>語り共有 本人のみ／制作Supporter</x:v>
       </x:c>
       <x:c r="C9" s="40" t="str">
         <x:v>—</x:v>
@@ -2971,10 +3664,10 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="L9" s="40" t="str">
-        <x:v>初期値は本人のみ。進捗共有とは別</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="40" customHeight="1">
+        <x:v>自分で＝本人のみ。一緒に・おまかせ＝制作Supporterと共有。語り単位で変更可</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="44" customHeight="1">
       <x:c r="A10" s="40" t="str">
         <x:v>S06</x:v>
       </x:c>
@@ -3012,7 +3705,7 @@
         <x:v>仕上げで最終確認</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="40" customHeight="1">
+    <x:row r="11" ht="44" customHeight="1">
       <x:c r="A11" s="40" t="str">
         <x:v>S07</x:v>
       </x:c>
@@ -3050,7 +3743,7 @@
         <x:v>作品単位</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="40" customHeight="1">
+    <x:row r="12" ht="44" customHeight="1">
       <x:c r="A12" s="40" t="str">
         <x:v>S08</x:v>
       </x:c>
@@ -3088,7 +3781,7 @@
         <x:v>家族共有と独立</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="40" customHeight="1">
+    <x:row r="13" ht="44" customHeight="1">
       <x:c r="A13" s="40" t="str">
         <x:v>S09</x:v>
       </x:c>
@@ -3123,10 +3816,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="L13" s="40" t="str">
-        <x:v>本人の明示操作</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="40" customHeight="1">
+        <x:v>本人、または意向を確認したおまかせSupporterが明示操作</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="44" customHeight="1">
       <x:c r="A14" s="40" t="str">
         <x:v>S10</x:v>
       </x:c>
@@ -3162,6 +3855,44 @@
       </x:c>
       <x:c r="L14" s="40" t="str">
         <x:v>個人データの収集と混同しない</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="44" customHeight="1">
+      <x:c r="A15" s="40" t="str">
+        <x:v>S11</x:v>
+      </x:c>
+      <x:c r="B15" s="40" t="str">
+        <x:v>支援スタイル・おまかせ確認</x:v>
+      </x:c>
+      <x:c r="C15" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D15" s="40" t="str">
+        <x:v>●</x:v>
+      </x:c>
+      <x:c r="E15" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="F15" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="G15" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="H15" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="I15" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="J15" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="K15" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="L15" s="40" t="str">
+        <x:v>本人の了承を確認。本人Accountは任意。途中変更可</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3226,31 +3957,31 @@
       <x:c r="I3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="54" t="str">
+      <x:c r="A4" s="70" t="str">
         <x:v>Case</x:v>
       </x:c>
-      <x:c r="B4" s="54" t="str">
+      <x:c r="B4" s="70" t="str">
         <x:v>位置づけ</x:v>
       </x:c>
-      <x:c r="C4" s="54" t="str">
+      <x:c r="C4" s="70" t="str">
         <x:v>HPに来た人</x:v>
       </x:c>
-      <x:c r="D4" s="54" t="str">
+      <x:c r="D4" s="70" t="str">
         <x:v>語る人</x:v>
       </x:c>
-      <x:c r="E4" s="54" t="str">
+      <x:c r="E4" s="70" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="F4" s="54" t="str">
+      <x:c r="F4" s="70" t="str">
         <x:v>同席・遠隔</x:v>
       </x:c>
-      <x:c r="G4" s="54" t="str">
+      <x:c r="G4" s="70" t="str">
         <x:v>購入者候補</x:v>
       </x:c>
-      <x:c r="H4" s="54" t="str">
+      <x:c r="H4" s="70" t="str">
         <x:v>本人Accountが必要になる時</x:v>
       </x:c>
-      <x:c r="I4" s="54" t="str">
+      <x:c r="I4" s="70" t="str">
         <x:v>要点</x:v>
       </x:c>
     </x:row>
@@ -3306,10 +4037,10 @@
         <x:v>子または本人。別Subcaseで管理。</x:v>
       </x:c>
       <x:c r="H6" s="40" t="str">
-        <x:v>本格利用の本人接続時。無料3問だけなら不要な場合あり。</x:v>
+        <x:v>自分で・一緒にでは必要。おまかせでは任意で後から接続可。</x:v>
       </x:c>
       <x:c r="I6" s="40" t="str">
-        <x:v>分岐最多。Personを維持する</x:v>
+        <x:v>Person中心。自分で／一緒に／おまかせの3スタイル</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
@@ -3391,26 +4122,26 @@
       <x:c r="F3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="54" t="str">
+      <x:c r="A4" s="70" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B4" s="54" t="str">
+      <x:c r="B4" s="70" t="str">
         <x:v>論点</x:v>
       </x:c>
-      <x:c r="C4" s="54" t="str">
+      <x:c r="C4" s="70" t="str">
         <x:v>現状案</x:v>
       </x:c>
-      <x:c r="D4" s="54" t="str">
+      <x:c r="D4" s="70" t="str">
         <x:v>状態</x:v>
       </x:c>
-      <x:c r="E4" s="54" t="str">
+      <x:c r="E4" s="70" t="str">
         <x:v>決める理由</x:v>
       </x:c>
-      <x:c r="F4" s="54" t="str">
+      <x:c r="F4" s="70" t="str">
         <x:v>次アクション</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="50" customHeight="1">
+    <x:row r="5" ht="54" customHeight="1">
       <x:c r="A5" s="40" t="str">
         <x:v>Q01</x:v>
       </x:c>
@@ -3418,19 +4149,19 @@
         <x:v>無料3問の語り共有初期値</x:v>
       </x:c>
       <x:c r="C5" s="40" t="str">
-        <x:v>本人のみ。Supporterには進捗だけを共有</x:v>
+        <x:v>自分で＝本人のみ。一緒に・おまかせ＝制作Supporterと共有。語り単位で本人のみへ変更可</x:v>
       </x:c>
       <x:c r="D5" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
       <x:c r="E5" s="40" t="str">
-        <x:v>親支援時のプライバシーと体験を左右</x:v>
+        <x:v>支援に必要な閲覧権限と本人の選択余地を両立</x:v>
       </x:c>
       <x:c r="F5" s="40" t="str">
         <x:v>B同席・子購入の実装へ反映</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="50" customHeight="1">
+    <x:row r="6" ht="54" customHeight="1">
       <x:c r="A6" s="40" t="str">
         <x:v>Q02</x:v>
       </x:c>
@@ -3438,19 +4169,19 @@
         <x:v>親支援時の進捗共有初期値</x:v>
       </x:c>
       <x:c r="C6" s="40" t="str">
-        <x:v>本人へ短く説明しON候補</x:v>
+        <x:v>自分で＝任意。一緒に・おまかせ＝制作Supporterへ共有</x:v>
       </x:c>
       <x:c r="D6" s="40" t="str">
-        <x:v>要確認</x:v>
+        <x:v>確定</x:v>
       </x:c>
       <x:c r="E6" s="40" t="str">
-        <x:v>娘の遠隔フォローに必要</x:v>
+        <x:v>娘の遠隔フォローと制作継続に必要</x:v>
       </x:c>
       <x:c r="F6" s="40" t="str">
-        <x:v>同意タイミング確定</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="50" customHeight="1">
+        <x:v>支援スタイル選択時の説明へ反映</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="54" customHeight="1">
       <x:c r="A7" s="40" t="str">
         <x:v>Q03</x:v>
       </x:c>
@@ -3470,7 +4201,7 @@
         <x:v>期限・再訪条件を確定</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="50" customHeight="1">
+    <x:row r="8" ht="54" customHeight="1">
       <x:c r="A8" s="40" t="str">
         <x:v>Q04</x:v>
       </x:c>
@@ -3490,7 +4221,7 @@
         <x:v>HPフローで確認</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="50" customHeight="1">
+    <x:row r="9" ht="54" customHeight="1">
       <x:c r="A9" s="40" t="str">
         <x:v>Q05</x:v>
       </x:c>
@@ -3510,7 +4241,7 @@
         <x:v>本番Phone Auth前に実機確認</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="50" customHeight="1">
+    <x:row r="10" ht="54" customHeight="1">
       <x:c r="A10" s="40" t="str">
         <x:v>Q06</x:v>
       </x:c>
@@ -3530,7 +4261,7 @@
         <x:v>UI実装時に確認</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="50" customHeight="1">
+    <x:row r="11" ht="54" customHeight="1">
       <x:c r="A11" s="40" t="str">
         <x:v>Q07</x:v>
       </x:c>
@@ -3550,7 +4281,7 @@
         <x:v>購入前後の画面とRPCを照合</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="50" customHeight="1">
+    <x:row r="12" ht="54" customHeight="1">
       <x:c r="A12" s="40" t="str">
         <x:v>Q08</x:v>
       </x:c>
@@ -3570,7 +4301,7 @@
         <x:v>現行登録処理とDBを照合</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="50" customHeight="1">
+    <x:row r="13" ht="54" customHeight="1">
       <x:c r="A13" s="40" t="str">
         <x:v>Q09</x:v>
       </x:c>
@@ -3588,6 +4319,46 @@
       </x:c>
       <x:c r="F13" s="40" t="str">
         <x:v>現行publication／共有テーブルを照合</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="54" customHeight="1">
+      <x:c r="A14" s="40" t="str">
+        <x:v>Q10</x:v>
+      </x:c>
+      <x:c r="B14" s="40" t="str">
+        <x:v>おまかせ時の本人Account・代理操作</x:v>
+      </x:c>
+      <x:c r="C14" s="40" t="str">
+        <x:v>Person中心。本人Accountは任意。Supporterが制作・購入・本編開始・仕上げを代理操作</x:v>
+      </x:c>
+      <x:c r="D14" s="40" t="str">
+        <x:v>確定</x:v>
+      </x:c>
+      <x:c r="E14" s="40" t="str">
+        <x:v>高齢の語り手本人にAccountや端末操作を必須にしない</x:v>
+      </x:c>
+      <x:c r="F14" s="40" t="str">
+        <x:v>06_支援スタイル・権限とBおまかせフローへ反映</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="54" customHeight="1">
+      <x:c r="A15" s="40" t="str">
+        <x:v>Q11</x:v>
+      </x:c>
+      <x:c r="B15" s="40" t="str">
+        <x:v>支援スタイル・本人了承確認の保存先</x:v>
+      </x:c>
+      <x:c r="C15" s="40" t="str">
+        <x:v>support_mode、confirmed_by、confirmed_at等を記録する案</x:v>
+      </x:c>
+      <x:c r="D15" s="40" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
+      <x:c r="E15" s="40" t="str">
+        <x:v>本人Accountなしで広い制作権限を付与する根拠と監査履歴が必要</x:v>
+      </x:c>
+      <x:c r="F15" s="40" t="str">
+        <x:v>DB・RLS・監査ログ設計と照合</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3606,8 +4377,19 @@
       <x:formula>$D5="要確認"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:conditionalFormatting sqref="A5:F15">
+    <x:cfRule type="expression" dxfId="10" priority="4">
+      <x:formula>$D5="要確認"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="13" priority="5">
+      <x:formula>$D5="要確認"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="D5:D13">
+      <x:formula1>"確定,要確認"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D5:D15">
       <x:formula1>"確定,要確認"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -3672,38 +4454,38 @@
       <x:c r="J3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="54" t="str">
+      <x:c r="A4" s="70" t="str">
         <x:v>Setting ID</x:v>
       </x:c>
-      <x:c r="B4" s="54" t="str">
+      <x:c r="B4" s="70" t="str">
         <x:v>設定・同意名</x:v>
       </x:c>
-      <x:c r="C4" s="54" t="str">
+      <x:c r="C4" s="70" t="str">
         <x:v>利用者が設定する画面</x:v>
       </x:c>
-      <x:c r="D4" s="54" t="str">
+      <x:c r="D4" s="70" t="str">
         <x:v>初期値</x:v>
       </x:c>
-      <x:c r="E4" s="54" t="str">
+      <x:c r="E4" s="70" t="str">
         <x:v>設定できる人</x:v>
       </x:c>
-      <x:c r="F4" s="54" t="str">
+      <x:c r="F4" s="70" t="str">
         <x:v>変更できる時期</x:v>
       </x:c>
-      <x:c r="G4" s="54" t="str">
+      <x:c r="G4" s="70" t="str">
         <x:v>保存先</x:v>
       </x:c>
-      <x:c r="H4" s="54" t="str">
+      <x:c r="H4" s="70" t="str">
         <x:v>関連Flow ID</x:v>
       </x:c>
-      <x:c r="I4" s="54" t="str">
+      <x:c r="I4" s="70" t="str">
         <x:v>実装状態</x:v>
       </x:c>
-      <x:c r="J4" s="54" t="str">
+      <x:c r="J4" s="70" t="str">
         <x:v>根拠仕様</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="68" customHeight="1">
+    <x:row r="5" ht="74" customHeight="1">
       <x:c r="A5" s="40" t="str">
         <x:v>S01</x:v>
       </x:c>
@@ -3735,7 +4517,7 @@
         <x:v>docs/product-brand-ux-master-v2.0.md §0</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="68" customHeight="1">
+    <x:row r="6" ht="74" customHeight="1">
       <x:c r="A6" s="40" t="str">
         <x:v>S02</x:v>
       </x:c>
@@ -3767,7 +4549,7 @@
         <x:v>docs/family-assisted-early-release-spec-20260917.md §2・§4</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="68" customHeight="1">
+    <x:row r="7" ht="74" customHeight="1">
       <x:c r="A7" s="40" t="str">
         <x:v>S03</x:v>
       </x:c>
@@ -3799,7 +4581,7 @@
         <x:v>supabase/migrations/202609170002_family_subject_connection.sql</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="68" customHeight="1">
+    <x:row r="8" ht="74" customHeight="1">
       <x:c r="A8" s="40" t="str">
         <x:v>S04</x:v>
       </x:c>
@@ -3807,13 +4589,13 @@
         <x:v>進捗共有</x:v>
       </x:c>
       <x:c r="C8" s="40" t="str">
-        <x:v>親Person作成時の説明／家族とのつながり設定</x:v>
+        <x:v>支援スタイル選択／家族とのつながり設定</x:v>
       </x:c>
       <x:c r="D8" s="40" t="str">
-        <x:v>要確認（ON候補）</x:v>
+        <x:v>自分で＝任意。一緒に・おまかせ＝制作Supporterへ共有</x:v>
       </x:c>
       <x:c r="E8" s="40" t="str">
-        <x:v>本人。未接続時は同席確認を記録。</x:v>
+        <x:v>本人または本人の了承を確認したSupporter</x:v>
       </x:c>
       <x:c r="F8" s="40" t="str">
         <x:v>初回説明後・本人接続後・随時</x:v>
@@ -3822,7 +4604,7 @@
         <x:v>family_subject_bindings.progress_enabled</x:v>
       </x:c>
       <x:c r="H8" s="40" t="str">
-        <x:v>B-CO-020、B-CO-030、B-REMOTE-020</x:v>
+        <x:v>B-CO-020、B-CO-030、B-REMOTE-020、B-CO-DELEGATED-050</x:v>
       </x:c>
       <x:c r="I8" s="40" t="str">
         <x:v>一部実装</x:v>
@@ -3831,21 +4613,21 @@
         <x:v>docs/family-assisted-early-release-spec-20260917.md §5／202609170002_family_subject_connection.sql</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="68" customHeight="1">
+    <x:row r="9" ht="74" customHeight="1">
       <x:c r="A9" s="40" t="str">
         <x:v>S05</x:v>
       </x:c>
       <x:c r="B9" s="40" t="str">
-        <x:v>語り共有 本人のみ／家族</x:v>
+        <x:v>語り共有 本人のみ／制作Supporter</x:v>
       </x:c>
       <x:c r="C9" s="40" t="str">
         <x:v>録音保存時／語り設定</x:v>
       </x:c>
       <x:c r="D9" s="40" t="str">
-        <x:v>本人のみ（Supporterへの自動共有なし）</x:v>
+        <x:v>自分で＝本人のみ。一緒に・おまかせ＝制作Supporterと共有</x:v>
       </x:c>
       <x:c r="E9" s="40" t="str">
-        <x:v>本人。Supporterは本人の公開範囲を拡張しない。</x:v>
+        <x:v>本人または本人の了承を確認したSupporter。語り単位で本人のみに変更可。</x:v>
       </x:c>
       <x:c r="F9" s="40" t="str">
         <x:v>語り保存時・後から随時</x:v>
@@ -3854,16 +4636,16 @@
         <x:v>answers.access_override／story_sharing_preferences／story_share_recipients</x:v>
       </x:c>
       <x:c r="H9" s="40" t="str">
-        <x:v>A-TRIAL-020、B-CO-030、C-TRIAL-010</x:v>
+        <x:v>A-TRIAL-020、B-CO-030、C-TRIAL-010、B-CO-DELEGATED-070</x:v>
       </x:c>
       <x:c r="I9" s="40" t="str">
         <x:v>一部実装</x:v>
       </x:c>
       <x:c r="J9" s="40" t="str">
-        <x:v>docs/family-assisted-early-release-spec-20260917.md §5／202609170002_family_subject_connection.sql</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="68" customHeight="1">
+        <x:v>06_支援スタイル・権限／202609170002_family_subject_connection.sql</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="74" customHeight="1">
       <x:c r="A10" s="40" t="str">
         <x:v>S06</x:v>
       </x:c>
@@ -3874,10 +4656,10 @@
         <x:v>仕上げ／掲載する語りの選択</x:v>
       </x:c>
       <x:c r="D10" s="40" t="str">
-        <x:v>公開可能な語りを候補表示</x:v>
+        <x:v>共有可能な語りを候補表示</x:v>
       </x:c>
       <x:c r="E10" s="40" t="str">
-        <x:v>本人または許可された仕上げ権限者。最終確認は本人。</x:v>
+        <x:v>本人または許可された仕上げ権限者。おまかせではSupporterが代理確定可。</x:v>
       </x:c>
       <x:c r="F10" s="40" t="str">
         <x:v>制作中・仕上げ・最終確定前</x:v>
@@ -3886,16 +4668,16 @@
         <x:v>book_work_manifests.answer_ids／confirmed_at／confirmed_by</x:v>
       </x:c>
       <x:c r="H10" s="40" t="str">
-        <x:v>A-TRIAL-040、B-CO-GIFT-060、B-REMOTE-SELF-050</x:v>
+        <x:v>A-TRIAL-040、B-CO-GIFT-060、B-CO-DELEGATED-070、B-REMOTE-SELF-050、B-DIRECT-DELEGATED-040</x:v>
       </x:c>
       <x:c r="I10" s="40" t="str">
         <x:v>一部実装</x:v>
       </x:c>
       <x:c r="J10" s="40" t="str">
-        <x:v>supabase/migrations/202609160004_book_work_manifest.sql</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="68" customHeight="1">
+        <x:v>supabase/migrations/202609160004_book_work_manifest.sql／06_支援スタイル・権限</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="74" customHeight="1">
       <x:c r="A11" s="40" t="str">
         <x:v>S07</x:v>
       </x:c>
@@ -3909,7 +4691,7 @@
         <x:v>非共有</x:v>
       </x:c>
       <x:c r="E11" s="40" t="str">
-        <x:v>本人</x:v>
+        <x:v>本人またはおまかせ権限のSupporter</x:v>
       </x:c>
       <x:c r="F11" s="40" t="str">
         <x:v>仕上げ時・完成後</x:v>
@@ -3918,16 +4700,16 @@
         <x:v>要確認（作品単位の共有正を照合）</x:v>
       </x:c>
       <x:c r="H11" s="40" t="str">
-        <x:v>A-TRIAL-040、B-CO-GIFT-060、B-REMOTE-SELF-050</x:v>
+        <x:v>A-TRIAL-040、B-CO-GIFT-060、B-CO-DELEGATED-070、B-REMOTE-SELF-050</x:v>
       </x:c>
       <x:c r="I11" s="40" t="str">
         <x:v>要確認</x:v>
       </x:c>
       <x:c r="J11" s="40" t="str">
-        <x:v>docs/product-brand-ux-master-v2.0.md §7／docs/product-concepts-and-naming.md §3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="68" customHeight="1">
+        <x:v>docs/product-brand-ux-master-v2.0.md §7／06_支援スタイル・権限</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="74" customHeight="1">
       <x:c r="A12" s="40" t="str">
         <x:v>S08</x:v>
       </x:c>
@@ -3941,7 +4723,7 @@
         <x:v>掲載しない・非公開を基準</x:v>
       </x:c>
       <x:c r="E12" s="40" t="str">
-        <x:v>本人</x:v>
+        <x:v>本人またはおまかせ権限のSupporter</x:v>
       </x:c>
       <x:c r="F12" s="40" t="str">
         <x:v>仕上げ時・完成後の閲覧方法変更</x:v>
@@ -3950,16 +4732,16 @@
         <x:v>voice_publications関連。掲載・匿名閲覧の正となる列は要確認</x:v>
       </x:c>
       <x:c r="H12" s="40" t="str">
-        <x:v>A-TRIAL-040、B-CO-GIFT-060、B-REMOTE-SELF-050</x:v>
+        <x:v>A-TRIAL-040、B-CO-GIFT-060、B-CO-DELEGATED-070、B-REMOTE-SELF-050</x:v>
       </x:c>
       <x:c r="I12" s="40" t="str">
         <x:v>一部実装</x:v>
       </x:c>
       <x:c r="J12" s="40" t="str">
-        <x:v>docs/voice-publication-and-qr.md／docs/product-brand-ux-master-v2.0.md §7</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="68" customHeight="1">
+        <x:v>docs/voice-publication-and-qr.md／06_支援スタイル・権限</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="74" customHeight="1">
       <x:c r="A13" s="40" t="str">
         <x:v>S09</x:v>
       </x:c>
@@ -3973,7 +4755,7 @@
         <x:v>未開始</x:v>
       </x:c>
       <x:c r="E13" s="40" t="str">
-        <x:v>Person本人Account</x:v>
+        <x:v>Person本人Accountまたは本人の意向を確認したおまかせ権限のSupporter</x:v>
       </x:c>
       <x:c r="F13" s="40" t="str">
         <x:v>一度だけ。開始後は戻さない。</x:v>
@@ -3982,16 +4764,16 @@
         <x:v>experience_contracts.main_experience_started_at／main_started_by／guarantee_days／guarantee_expires_at</x:v>
       </x:c>
       <x:c r="H13" s="40" t="str">
-        <x:v>A-TRIAL-040、A-DIRECT-020、B-CO-GIFT-060、B-REMOTE-SELF-050、B-DIRECT-GIFT-030</x:v>
+        <x:v>A-TRIAL-040、A-DIRECT-020、B-CO-GIFT-060、B-CO-DELEGATED-060、B-REMOTE-SELF-050、B-DIRECT-GIFT-030、B-DIRECT-DELEGATED-030</x:v>
       </x:c>
       <x:c r="I13" s="40" t="str">
         <x:v>一部実装</x:v>
       </x:c>
       <x:c r="J13" s="40" t="str">
-        <x:v>docs/product-brand-ux-master-v2.0.md §11／202609150001_add_experience_contracts_v2.sql</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="68" customHeight="1">
+        <x:v>docs/product-brand-ux-master-v2.0.md §11／06_支援スタイル・権限</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="74" customHeight="1">
       <x:c r="A14" s="40" t="str">
         <x:v>S10</x:v>
       </x:c>
@@ -4021,6 +4803,38 @@
       </x:c>
       <x:c r="J14" s="40" t="str">
         <x:v>src/ExperienceContractSettings.jsx／supabase/functions/export-experience-data</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="74" customHeight="1">
+      <x:c r="A15" s="40" t="str">
+        <x:v>S11</x:v>
+      </x:c>
+      <x:c r="B15" s="40" t="str">
+        <x:v>支援スタイル・おまかせ確認</x:v>
+      </x:c>
+      <x:c r="C15" s="40" t="str">
+        <x:v>対象Person作成／大切な人の物語の設定</x:v>
+      </x:c>
+      <x:c r="D15" s="40" t="str">
+        <x:v>未選択</x:v>
+      </x:c>
+      <x:c r="E15" s="40" t="str">
+        <x:v>Supporter。おまかせ時は語り手本人の了承を確認。</x:v>
+      </x:c>
+      <x:c r="F15" s="40" t="str">
+        <x:v>開始時・購入時・本人接続時・随時</x:v>
+      </x:c>
+      <x:c r="G15" s="40" t="str">
+        <x:v>要確認（support_mode、confirmed_by、confirmed_at等）</x:v>
+      </x:c>
+      <x:c r="H15" s="40" t="str">
+        <x:v>B-CO-020、B-CO-DELEGATED-050、B-DIRECT-DELEGATED-020</x:v>
+      </x:c>
+      <x:c r="I15" s="40" t="str">
+        <x:v>未実装</x:v>
+      </x:c>
+      <x:c r="J15" s="40" t="str">
+        <x:v>06_支援スタイル・権限／04_運営チェック Q10・Q11</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4039,11 +4853,322 @@
       <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:conditionalFormatting sqref="A5:J15">
+    <x:cfRule type="expression" dxfId="11" priority="4">
+      <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="14" priority="5">
+      <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="I5:I14">
+      <x:formula1>"実装済み,一部実装,未実装,要確認"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I5:I15">
       <x:formula1>"実装済み,一部実装,未実装,要確認"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="31" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="57" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="28" t="str">
+        <x:v>支援スタイル・権限</x:v>
+      </x:c>
+      <x:c r="B1" s="28"/>
+      <x:c r="C1" s="28"/>
+      <x:c r="D1" s="28"/>
+      <x:c r="E1" s="28"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="30" t="str">
+        <x:v>Personが作品の主体。本人Account、Supporter Account、または両方が、選んだ支援スタイルに応じて同じPersonの制作を担う。</x:v>
+      </x:c>
+      <x:c r="B2" s="30"/>
+      <x:c r="C2" s="30"/>
+      <x:c r="D2" s="30"/>
+      <x:c r="E2" s="30"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+    </x:row>
+    <x:row r="4" ht="38" customHeight="1">
+      <x:c r="A4" s="70" t="str">
+        <x:v>操作・条件</x:v>
+      </x:c>
+      <x:c r="B4" s="70" t="str">
+        <x:v>自分で進める</x:v>
+      </x:c>
+      <x:c r="C4" s="70" t="str">
+        <x:v>一緒に進める</x:v>
+      </x:c>
+      <x:c r="D4" s="70" t="str">
+        <x:v>おまかせする</x:v>
+      </x:c>
+      <x:c r="E4" s="70" t="str">
+        <x:v>補足</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="48" customHeight="1">
+      <x:c r="A5" s="66" t="str">
+        <x:v>本人Account必須</x:v>
+      </x:c>
+      <x:c r="B5" s="40" t="str">
+        <x:v>○</x:v>
+      </x:c>
+      <x:c r="C5" s="40" t="str">
+        <x:v>○</x:v>
+      </x:c>
+      <x:c r="D5" s="74" t="str">
+        <x:v>×</x:v>
+      </x:c>
+      <x:c r="E5" s="40" t="str">
+        <x:v>おまかせでは本人Accountを後から任意で接続できる</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="48" customHeight="1">
+      <x:c r="A6" s="66" t="str">
+        <x:v>Supporter Account</x:v>
+      </x:c>
+      <x:c r="B6" s="40" t="str">
+        <x:v>任意</x:v>
+      </x:c>
+      <x:c r="C6" s="40" t="str">
+        <x:v>○</x:v>
+      </x:c>
+      <x:c r="D6" s="74" t="str">
+        <x:v>○</x:v>
+      </x:c>
+      <x:c r="E6" s="40" t="str">
+        <x:v>支援する家族・信頼できる人のAccount</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="48" customHeight="1">
+      <x:c r="A7" s="66" t="str">
+        <x:v>録音操作</x:v>
+      </x:c>
+      <x:c r="B7" s="40" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="C7" s="40" t="str">
+        <x:v>本人／Supporter</x:v>
+      </x:c>
+      <x:c r="D7" s="74" t="str">
+        <x:v>Supporter</x:v>
+      </x:c>
+      <x:c r="E7" s="40" t="str">
+        <x:v>語る人は常にPerson本人。端末操作は別の人でもよい</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="48" customHeight="1">
+      <x:c r="A8" s="66" t="str">
+        <x:v>全語りの閲覧</x:v>
+      </x:c>
+      <x:c r="B8" s="40" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="C8" s="40" t="str">
+        <x:v>本人＋制作Supporter</x:v>
+      </x:c>
+      <x:c r="D8" s="74" t="str">
+        <x:v>制作Supporter</x:v>
+      </x:c>
+      <x:c r="E8" s="40" t="str">
+        <x:v>語り単位で本人のみへ変更できる</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="48" customHeight="1">
+      <x:c r="A9" s="66" t="str">
+        <x:v>文章編集・語り直し</x:v>
+      </x:c>
+      <x:c r="B9" s="40" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="C9" s="40" t="str">
+        <x:v>双方</x:v>
+      </x:c>
+      <x:c r="D9" s="74" t="str">
+        <x:v>Supporter代理可</x:v>
+      </x:c>
+      <x:c r="E9" s="40" t="str">
+        <x:v>本人の意向を確認しながら行う</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="48" customHeight="1">
+      <x:c r="A10" s="66" t="str">
+        <x:v>写真追加</x:v>
+      </x:c>
+      <x:c r="B10" s="40" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="C10" s="40" t="str">
+        <x:v>双方</x:v>
+      </x:c>
+      <x:c r="D10" s="74" t="str">
+        <x:v>Supporter代理可</x:v>
+      </x:c>
+      <x:c r="E10" s="40" t="str">
+        <x:v>家族が離れた場所から追加できる</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="48" customHeight="1">
+      <x:c r="A11" s="66" t="str">
+        <x:v>共有範囲の設定</x:v>
+      </x:c>
+      <x:c r="B11" s="40" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="C11" s="40" t="str">
+        <x:v>双方</x:v>
+      </x:c>
+      <x:c r="D11" s="74" t="str">
+        <x:v>Supporter代理可</x:v>
+      </x:c>
+      <x:c r="E11" s="40" t="str">
+        <x:v>本人の意向を確認。既定は制作Supporterと共有</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="48" customHeight="1">
+      <x:c r="A12" s="66" t="str">
+        <x:v>ブック収録選択</x:v>
+      </x:c>
+      <x:c r="B12" s="40" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="C12" s="40" t="str">
+        <x:v>双方</x:v>
+      </x:c>
+      <x:c r="D12" s="74" t="str">
+        <x:v>Supporter代理可</x:v>
+      </x:c>
+      <x:c r="E12" s="40" t="str">
+        <x:v>本人に確認しながら掲載・除外を決める</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="48" customHeight="1">
+      <x:c r="A13" s="66" t="str">
+        <x:v>ブック編集</x:v>
+      </x:c>
+      <x:c r="B13" s="40" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="C13" s="40" t="str">
+        <x:v>双方</x:v>
+      </x:c>
+      <x:c r="D13" s="74" t="str">
+        <x:v>Supporter代理可</x:v>
+      </x:c>
+      <x:c r="E13" s="40" t="str">
+        <x:v>並び順、文章、写真、タイトル等</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="48" customHeight="1">
+      <x:c r="A14" s="66" t="str">
+        <x:v>Webブック・QR設定</x:v>
+      </x:c>
+      <x:c r="B14" s="40" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="C14" s="40" t="str">
+        <x:v>双方</x:v>
+      </x:c>
+      <x:c r="D14" s="74" t="str">
+        <x:v>Supporter代理可</x:v>
+      </x:c>
+      <x:c r="E14" s="40" t="str">
+        <x:v>公開範囲は作品単位。初期値は非公開側</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="48" customHeight="1">
+      <x:c r="A15" s="66" t="str">
+        <x:v>最終確定・製本注文・増刷</x:v>
+      </x:c>
+      <x:c r="B15" s="40" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="C15" s="40" t="str">
+        <x:v>本人中心／共同</x:v>
+      </x:c>
+      <x:c r="D15" s="74" t="str">
+        <x:v>Supporter代理可</x:v>
+      </x:c>
+      <x:c r="E15" s="40" t="str">
+        <x:v>操作主体と確定日時を記録する</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="48" customHeight="1">
+      <x:c r="A16" s="66" t="str">
+        <x:v>本編開始</x:v>
+      </x:c>
+      <x:c r="B16" s="40" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="C16" s="40" t="str">
+        <x:v>本人／共同</x:v>
+      </x:c>
+      <x:c r="D16" s="74" t="str">
+        <x:v>Supporter代理可</x:v>
+      </x:c>
+      <x:c r="E16" s="40" t="str">
+        <x:v>本人の続行意思を確認。開始時に返金保証終了</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="48" customHeight="1">
+      <x:c r="A17" s="66" t="str">
+        <x:v>支払い</x:v>
+      </x:c>
+      <x:c r="B17" s="40" t="str">
+        <x:v>本人等</x:v>
+      </x:c>
+      <x:c r="C17" s="40" t="str">
+        <x:v>どちらでも</x:v>
+      </x:c>
+      <x:c r="D17" s="74" t="str">
+        <x:v>Supporter想定</x:v>
+      </x:c>
+      <x:c r="E17" s="40" t="str">
+        <x:v>PayerはPerson・操作者と独立して記録する</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="48" customHeight="1">
+      <x:c r="A18" s="66" t="str">
+        <x:v>本人Accountの後付け</x:v>
+      </x:c>
+      <x:c r="B18" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C18" s="40" t="str">
+        <x:v>接続済み</x:v>
+      </x:c>
+      <x:c r="D18" s="74" t="str">
+        <x:v>任意</x:v>
+      </x:c>
+      <x:c r="E18" s="40" t="str">
+        <x:v>接続しても既存Person・Projectを新規作成しない</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A2:E2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: separate progress modes and supporter permissions
</commit_message>
<xml_diff>
--- a/docs/product/user-flow/user-flow-master.xlsx
+++ b/docs/product/user-flow/user-flow-master.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="R4f2c39fdb6fb4df0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_利用動線" sheetId="2" r:id="R08d36ea6b2ec41d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定同意" sheetId="3" r:id="Rf8e54bb235c24001"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ケース一覧" sheetId="4" r:id="R25c98bfd1b8d41e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_運営チェック" sheetId="5" r:id="R01cc07579652463b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_実装対応" sheetId="6" r:id="R6996979a404c4678"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_支援スタイル・権限" sheetId="7" r:id="R188b9cdbebe24e39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="Re93806d8928241dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_利用動線" sheetId="2" r:id="R682eaac39b764301"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定同意" sheetId="3" r:id="Re3a45a3e111f4fd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ケース一覧" sheetId="4" r:id="R8b404681be904d5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_運営チェック" sheetId="5" r:id="R09ef5931515a4d2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_実装対応" sheetId="6" r:id="R97853221312a4b2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_支援スタイル・権限" sheetId="7" r:id="R28f5b3081d014bbf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -89,7 +89,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="20">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -166,6 +166,26 @@
         <x:fgColor rgb="FFEEF4F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF315B5B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF4F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF315B5B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF4F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -188,7 +208,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="75">
+  <x:cellXfs count="91">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -356,11 +376,111 @@
     <x:xf numFmtId="0" fontId="7" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="15">
+  <x:dxfs count="21">
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:color rgb="FF8A5A00"/>
@@ -735,13 +855,13 @@
       <x:c r="C3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="70" t="str">
+      <x:c r="A4" s="86" t="str">
         <x:v>シート</x:v>
       </x:c>
-      <x:c r="B4" s="70" t="str">
+      <x:c r="B4" s="86" t="str">
         <x:v>役割</x:v>
       </x:c>
-      <x:c r="C4" s="70" t="str">
+      <x:c r="C4" s="86" t="str">
         <x:v>ポイント</x:v>
       </x:c>
     </x:row>
@@ -805,10 +925,10 @@
         <x:v>06_支援スタイル・権限</x:v>
       </x:c>
       <x:c r="B10" s="40" t="str">
-        <x:v>操作権限の基準</x:v>
+        <x:v>進め方と権限の基準</x:v>
       </x:c>
       <x:c r="C10" s="40" t="str">
-        <x:v>本人Accountなしのおまかせを含む3つの支援スタイルを定義する。</x:v>
+        <x:v>2つの進め方、個別のSupporter権限、本人Account、通知先を分けて定義する。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
@@ -817,13 +937,13 @@
       <x:c r="C11" s="41"/>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
-      <x:c r="A12" s="73" t="str">
+      <x:c r="A12" s="89" t="str">
         <x:v>更新ルール</x:v>
       </x:c>
-      <x:c r="B12" s="73" t="str">
+      <x:c r="B12" s="89" t="str">
         <x:v>同名ファイルを更新</x:v>
       </x:c>
-      <x:c r="C12" s="73" t="str">
+      <x:c r="C12" s="89" t="str">
         <x:v>別バージョンのExcelを増やさず、変更理由と履歴はGitで管理する。</x:v>
       </x:c>
     </x:row>
@@ -898,7 +1018,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="30" t="str">
-        <x:v>Person＝作品の主体。Account＝認証・認可主体。本人Account、Supporter Account、または両方が同じPersonの制作を担える。</x:v>
+        <x:v>進め方は主な操作主体だけを表す。Supporter権限、本人Account、通知先は別に管理し、途中で変更できる。</x:v>
       </x:c>
       <x:c r="B2" s="30"/>
       <x:c r="C2" s="30"/>
@@ -953,79 +1073,79 @@
       <x:c r="Y3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="70" t="str">
+      <x:c r="A4" s="86" t="str">
         <x:v>Flow ID</x:v>
       </x:c>
-      <x:c r="B4" s="70" t="str">
+      <x:c r="B4" s="86" t="str">
         <x:v>Case</x:v>
       </x:c>
-      <x:c r="C4" s="70" t="str">
+      <x:c r="C4" s="86" t="str">
         <x:v>Subcase</x:v>
       </x:c>
-      <x:c r="D4" s="70" t="str">
-        <x:v>支援スタイル</x:v>
-      </x:c>
-      <x:c r="E4" s="70" t="str">
+      <x:c r="D4" s="86" t="str">
+        <x:v>進め方</x:v>
+      </x:c>
+      <x:c r="E4" s="86" t="str">
         <x:v>Step</x:v>
       </x:c>
-      <x:c r="F4" s="70" t="str">
+      <x:c r="F4" s="86" t="str">
         <x:v>ユーザー行動</x:v>
       </x:c>
-      <x:c r="G4" s="70" t="str">
+      <x:c r="G4" s="86" t="str">
         <x:v>ユーザーへの説明</x:v>
       </x:c>
-      <x:c r="H4" s="70" t="str">
+      <x:c r="H4" s="86" t="str">
         <x:v>利用中Account</x:v>
       </x:c>
-      <x:c r="I4" s="70" t="str">
+      <x:c r="I4" s="86" t="str">
         <x:v>このStepの操作者</x:v>
       </x:c>
-      <x:c r="J4" s="70" t="str">
+      <x:c r="J4" s="86" t="str">
         <x:v>このStepで語る人</x:v>
       </x:c>
-      <x:c r="K4" s="70" t="str">
+      <x:c r="K4" s="86" t="str">
         <x:v>Person</x:v>
       </x:c>
-      <x:c r="L4" s="70" t="str">
+      <x:c r="L4" s="86" t="str">
         <x:v>Payer</x:v>
       </x:c>
-      <x:c r="M4" s="70" t="str">
+      <x:c r="M4" s="86" t="str">
         <x:v>Supporter</x:v>
       </x:c>
-      <x:c r="N4" s="70" t="str">
+      <x:c r="N4" s="86" t="str">
         <x:v>Device</x:v>
       </x:c>
-      <x:c r="O4" s="70" t="str">
+      <x:c r="O4" s="86" t="str">
         <x:v>現在状態</x:v>
       </x:c>
-      <x:c r="P4" s="70" t="str">
+      <x:c r="P4" s="86" t="str">
         <x:v>分岐条件</x:v>
       </x:c>
-      <x:c r="Q4" s="70" t="str">
+      <x:c r="Q4" s="86" t="str">
         <x:v>次の状態</x:v>
       </x:c>
-      <x:c r="R4" s="70" t="str">
+      <x:c r="R4" s="86" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="S4" s="70" t="str">
+      <x:c r="S4" s="86" t="str">
         <x:v>購入</x:v>
       </x:c>
-      <x:c r="T4" s="70" t="str">
+      <x:c r="T4" s="86" t="str">
         <x:v>本人認証</x:v>
       </x:c>
-      <x:c r="U4" s="70" t="str">
+      <x:c r="U4" s="86" t="str">
         <x:v>設定・同意</x:v>
       </x:c>
-      <x:c r="V4" s="70" t="str">
+      <x:c r="V4" s="86" t="str">
         <x:v>内容共有</x:v>
       </x:c>
-      <x:c r="W4" s="70" t="str">
+      <x:c r="W4" s="86" t="str">
         <x:v>進捗共有</x:v>
       </x:c>
-      <x:c r="X4" s="70" t="str">
+      <x:c r="X4" s="86" t="str">
         <x:v>内部メモ</x:v>
       </x:c>
-      <x:c r="Y4" s="70" t="str">
+      <x:c r="Y4" s="86" t="str">
         <x:v>確定度</x:v>
       </x:c>
     </x:row>
@@ -1040,7 +1160,7 @@
         <x:v>無料3問</x:v>
       </x:c>
       <x:c r="D5" s="40" t="str">
-        <x:v>自分で進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E5" s="40" t="n">
         <x:v>1</x:v>
@@ -1117,7 +1237,7 @@
         <x:v>無料3問</x:v>
       </x:c>
       <x:c r="D6" s="40" t="str">
-        <x:v>自分で進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E6" s="40" t="n">
         <x:v>2</x:v>
@@ -1194,7 +1314,7 @@
         <x:v>無料3問</x:v>
       </x:c>
       <x:c r="D7" s="40" t="str">
-        <x:v>自分で進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E7" s="40" t="n">
         <x:v>3</x:v>
@@ -1271,7 +1391,7 @@
         <x:v>無料3問</x:v>
       </x:c>
       <x:c r="D8" s="40" t="str">
-        <x:v>自分で進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E8" s="40" t="n">
         <x:v>4</x:v>
@@ -1348,7 +1468,7 @@
         <x:v>直接購入</x:v>
       </x:c>
       <x:c r="D9" s="40" t="str">
-        <x:v>自分で進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E9" s="40" t="n">
         <x:v>1</x:v>
@@ -1425,7 +1545,7 @@
         <x:v>直接購入</x:v>
       </x:c>
       <x:c r="D10" s="40" t="str">
-        <x:v>自分で進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E10" s="40" t="n">
         <x:v>2</x:v>
@@ -1579,7 +1699,7 @@
         <x:v>同席3問</x:v>
       </x:c>
       <x:c r="D12" s="40" t="str">
-        <x:v>未選択→一緒に／おまかせ</x:v>
+        <x:v>未選択</x:v>
       </x:c>
       <x:c r="E12" s="40" t="n">
         <x:v>2</x:v>
@@ -1630,7 +1750,7 @@
         <x:v>親なし</x:v>
       </x:c>
       <x:c r="U12" s="40" t="str">
-        <x:v>対象Person・支援・進捗説明</x:v>
+        <x:v>対象Person・進め方・Supporter権限</x:v>
       </x:c>
       <x:c r="V12" s="40" t="str">
         <x:v>未設定</x:v>
@@ -1656,7 +1776,7 @@
         <x:v>同席3問</x:v>
       </x:c>
       <x:c r="D13" s="40" t="str">
-        <x:v>一緒に／おまかせ</x:v>
+        <x:v>未選択（家族端末で体験）</x:v>
       </x:c>
       <x:c r="E13" s="40" t="n">
         <x:v>3</x:v>
@@ -1707,13 +1827,13 @@
         <x:v>母なし</x:v>
       </x:c>
       <x:c r="U13" s="40" t="str">
-        <x:v>支援スタイル・語り共有・進捗共有</x:v>
+        <x:v>進め方・Supporter権限・共有設定</x:v>
       </x:c>
       <x:c r="V13" s="40" t="str">
-        <x:v>制作Supporterと共有（語り単位で本人のみへ変更可）</x:v>
+        <x:v>語りを見る権限のあるSupporterと共有</x:v>
       </x:c>
       <x:c r="W13" s="40" t="str">
-        <x:v>共有</x:v>
+        <x:v>進捗を見る権限に従う</x:v>
       </x:c>
       <x:c r="X13" s="40" t="str">
         <x:v>Account＝子、語る人＝母、Person＝母</x:v>
@@ -1733,7 +1853,7 @@
         <x:v>同席3問・子購入</x:v>
       </x:c>
       <x:c r="D14" s="40" t="str">
-        <x:v>一緒に／おまかせ</x:v>
+        <x:v>未選択→本人が進める／家族におまかせする</x:v>
       </x:c>
       <x:c r="E14" s="40" t="n">
         <x:v>4</x:v>
@@ -1810,7 +1930,7 @@
         <x:v>同席3問・子購入・おまかせ</x:v>
       </x:c>
       <x:c r="D15" s="40" t="str">
-        <x:v>おまかせする</x:v>
+        <x:v>家族におまかせする</x:v>
       </x:c>
       <x:c r="E15" s="40" t="n">
         <x:v>5</x:v>
@@ -1861,16 +1981,16 @@
         <x:v>不要</x:v>
       </x:c>
       <x:c r="U15" s="40" t="str">
-        <x:v>おまかせ確認・制作権限</x:v>
+        <x:v>進め方・おまかせ確認・制作権限</x:v>
       </x:c>
       <x:c r="V15" s="40" t="str">
-        <x:v>制作Supporterと共有</x:v>
+        <x:v>語りを見る権限のあるSupporterと共有</x:v>
       </x:c>
       <x:c r="W15" s="40" t="str">
-        <x:v>共有</x:v>
+        <x:v>進捗を見る権限に従う</x:v>
       </x:c>
       <x:c r="X15" s="40" t="str">
-        <x:v>support_mode＝おまかせ。本人Accountは任意</x:v>
+        <x:v>primary_mode＝家族中心。制作権限は個別Permission</x:v>
       </x:c>
       <x:c r="Y15" s="40" t="str">
         <x:v>確定</x:v>
@@ -1887,7 +2007,7 @@
         <x:v>同席3問・子購入・おまかせ</x:v>
       </x:c>
       <x:c r="D16" s="40" t="str">
-        <x:v>おまかせする</x:v>
+        <x:v>家族におまかせする</x:v>
       </x:c>
       <x:c r="E16" s="40" t="n">
         <x:v>6</x:v>
@@ -1964,7 +2084,7 @@
         <x:v>同席3問・子購入・おまかせ</x:v>
       </x:c>
       <x:c r="D17" s="40" t="str">
-        <x:v>おまかせする</x:v>
+        <x:v>家族におまかせする</x:v>
       </x:c>
       <x:c r="E17" s="40" t="n">
         <x:v>7</x:v>
@@ -2041,7 +2161,7 @@
         <x:v>同席3問・子購入</x:v>
       </x:c>
       <x:c r="D18" s="40" t="str">
-        <x:v>一緒に進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E18" s="40" t="n">
         <x:v>5</x:v>
@@ -2118,7 +2238,7 @@
         <x:v>同席3問・子購入</x:v>
       </x:c>
       <x:c r="D19" s="40" t="str">
-        <x:v>一緒に進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E19" s="40" t="n">
         <x:v>6</x:v>
@@ -2272,7 +2392,7 @@
         <x:v>遠隔3問</x:v>
       </x:c>
       <x:c r="D21" s="40" t="str">
-        <x:v>本人が自分で／一緒に</x:v>
+        <x:v>未選択（本人へ送付）</x:v>
       </x:c>
       <x:c r="E21" s="40" t="n">
         <x:v>2</x:v>
@@ -2349,7 +2469,7 @@
         <x:v>B遠隔3問から派生</x:v>
       </x:c>
       <x:c r="D22" s="40" t="str">
-        <x:v>自分で進める</x:v>
+        <x:v>未選択（本人端末で体験）</x:v>
       </x:c>
       <x:c r="E22" s="40" t="n">
         <x:v>1</x:v>
@@ -2426,7 +2546,7 @@
         <x:v>B遠隔3問から派生</x:v>
       </x:c>
       <x:c r="D23" s="40" t="str">
-        <x:v>自分で進める</x:v>
+        <x:v>未選択（本人端末で体験）</x:v>
       </x:c>
       <x:c r="E23" s="40" t="n">
         <x:v>2</x:v>
@@ -2503,7 +2623,7 @@
         <x:v>遠隔3問・子購入</x:v>
       </x:c>
       <x:c r="D24" s="40" t="str">
-        <x:v>一緒に進める</x:v>
+        <x:v>未選択→本人が進める</x:v>
       </x:c>
       <x:c r="E24" s="40" t="n">
         <x:v>3</x:v>
@@ -2580,7 +2700,7 @@
         <x:v>遠隔3問・子購入</x:v>
       </x:c>
       <x:c r="D25" s="40" t="str">
-        <x:v>一緒に進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E25" s="40" t="n">
         <x:v>4</x:v>
@@ -2657,7 +2777,7 @@
         <x:v>遠隔3問・本人購入</x:v>
       </x:c>
       <x:c r="D26" s="40" t="str">
-        <x:v>自分で進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E26" s="40" t="n">
         <x:v>3</x:v>
@@ -2734,7 +2854,7 @@
         <x:v>遠隔3問・本人購入</x:v>
       </x:c>
       <x:c r="D27" s="40" t="str">
-        <x:v>自分で進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E27" s="40" t="n">
         <x:v>4</x:v>
@@ -2811,7 +2931,7 @@
         <x:v>遠隔3問・本人購入</x:v>
       </x:c>
       <x:c r="D28" s="40" t="str">
-        <x:v>自分で進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E28" s="40" t="n">
         <x:v>5</x:v>
@@ -2888,7 +3008,7 @@
         <x:v>3問なし・子購入</x:v>
       </x:c>
       <x:c r="D29" s="40" t="str">
-        <x:v>未選択→一緒に／おまかせ</x:v>
+        <x:v>未選択→本人が進める／家族におまかせする</x:v>
       </x:c>
       <x:c r="E29" s="40" t="n">
         <x:v>1</x:v>
@@ -2927,7 +3047,7 @@
         <x:v>無料3問を経ずギフト購入</x:v>
       </x:c>
       <x:c r="Q29" s="40" t="str">
-        <x:v>支払済／支援スタイル選択待ち</x:v>
+        <x:v>支払済／進め方選択待ち</x:v>
       </x:c>
       <x:c r="R29" s="40" t="str">
         <x:v>なし</x:v>
@@ -2939,7 +3059,7 @@
         <x:v>親未</x:v>
       </x:c>
       <x:c r="U29" s="40" t="str">
-        <x:v>購入条件・45日保証・支援スタイル</x:v>
+        <x:v>購入条件・45日保証・進め方</x:v>
       </x:c>
       <x:c r="V29" s="40" t="str">
         <x:v>—</x:v>
@@ -2965,7 +3085,7 @@
         <x:v>3問なし・子購入・おまかせ</x:v>
       </x:c>
       <x:c r="D30" s="40" t="str">
-        <x:v>おまかせする</x:v>
+        <x:v>家族におまかせする</x:v>
       </x:c>
       <x:c r="E30" s="40" t="n">
         <x:v>2</x:v>
@@ -3016,16 +3136,16 @@
         <x:v>不要</x:v>
       </x:c>
       <x:c r="U30" s="40" t="str">
-        <x:v>おまかせ確認・制作権限</x:v>
+        <x:v>進め方・おまかせ確認・制作権限</x:v>
       </x:c>
       <x:c r="V30" s="40" t="str">
-        <x:v>制作Supporterと共有</x:v>
+        <x:v>語りを見る権限のあるSupporterと共有</x:v>
       </x:c>
       <x:c r="W30" s="40" t="str">
-        <x:v>共有</x:v>
+        <x:v>進捗を見る権限に従う</x:v>
       </x:c>
       <x:c r="X30" s="40" t="str">
-        <x:v>support_mode＝おまかせ。本人Accountは任意</x:v>
+        <x:v>primary_mode＝家族中心。制作権限は個別Permission</x:v>
       </x:c>
       <x:c r="Y30" s="40" t="str">
         <x:v>確定</x:v>
@@ -3042,7 +3162,7 @@
         <x:v>3問なし・子購入・おまかせ</x:v>
       </x:c>
       <x:c r="D31" s="40" t="str">
-        <x:v>おまかせする</x:v>
+        <x:v>家族におまかせする</x:v>
       </x:c>
       <x:c r="E31" s="40" t="n">
         <x:v>3</x:v>
@@ -3119,7 +3239,7 @@
         <x:v>3問なし・子購入・おまかせ</x:v>
       </x:c>
       <x:c r="D32" s="40" t="str">
-        <x:v>おまかせする</x:v>
+        <x:v>家族におまかせする</x:v>
       </x:c>
       <x:c r="E32" s="40" t="n">
         <x:v>4</x:v>
@@ -3196,7 +3316,7 @@
         <x:v>3問なし・子購入</x:v>
       </x:c>
       <x:c r="D33" s="40" t="str">
-        <x:v>一緒に進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E33" s="40" t="n">
         <x:v>2</x:v>
@@ -3273,7 +3393,7 @@
         <x:v>3問なし・子購入</x:v>
       </x:c>
       <x:c r="D34" s="40" t="str">
-        <x:v>一緒に進める</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="E34" s="40" t="n">
         <x:v>3</x:v>
@@ -3360,6 +3480,12 @@
       <x:formula>$Y5="要確認"</x:formula>
     </x:cfRule>
     <x:cfRule type="expression" dxfId="12" priority="5">
+      <x:formula>$Y5="要確認"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="15" priority="6">
+      <x:formula>$Y5="要確認"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="18" priority="7">
       <x:formula>$Y5="要確認"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -3440,40 +3566,40 @@
       <x:c r="L3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="70" t="str">
+      <x:c r="A4" s="86" t="str">
         <x:v>Setting ID</x:v>
       </x:c>
-      <x:c r="B4" s="70" t="str">
+      <x:c r="B4" s="86" t="str">
         <x:v>設定・同意</x:v>
       </x:c>
-      <x:c r="C4" s="70" t="str">
+      <x:c r="C4" s="86" t="str">
         <x:v>Account登録</x:v>
       </x:c>
-      <x:c r="D4" s="70" t="str">
+      <x:c r="D4" s="86" t="str">
         <x:v>対象Person作成</x:v>
       </x:c>
-      <x:c r="E4" s="70" t="str">
+      <x:c r="E4" s="86" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="F4" s="70" t="str">
+      <x:c r="F4" s="86" t="str">
         <x:v>購入</x:v>
       </x:c>
-      <x:c r="G4" s="70" t="str">
+      <x:c r="G4" s="86" t="str">
         <x:v>本人接続</x:v>
       </x:c>
-      <x:c r="H4" s="70" t="str">
+      <x:c r="H4" s="86" t="str">
         <x:v>本編開始</x:v>
       </x:c>
-      <x:c r="I4" s="70" t="str">
+      <x:c r="I4" s="86" t="str">
         <x:v>制作中</x:v>
       </x:c>
-      <x:c r="J4" s="70" t="str">
+      <x:c r="J4" s="86" t="str">
         <x:v>仕上げ</x:v>
       </x:c>
-      <x:c r="K4" s="70" t="str">
+      <x:c r="K4" s="86" t="str">
         <x:v>完成後</x:v>
       </x:c>
-      <x:c r="L4" s="70" t="str">
+      <x:c r="L4" s="86" t="str">
         <x:v>備考</x:v>
       </x:c>
     </x:row>
@@ -3626,7 +3752,7 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="L8" s="40" t="str">
-        <x:v>自分で＝任意。一緒に・おまかせ＝制作Supporterへ共有</x:v>
+        <x:v>進捗を見るPermissionのあるSupporterへ共有。進め方とは独立</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="44" customHeight="1">
@@ -3664,7 +3790,7 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="L9" s="40" t="str">
-        <x:v>自分で＝本人のみ。一緒に・おまかせ＝制作Supporterと共有。語り単位で変更可</x:v>
+        <x:v>語りを見るPermissionのあるSupporterへ共有。語り単位で変更可</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="44" customHeight="1">
@@ -3816,7 +3942,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="L13" s="40" t="str">
-        <x:v>本人、または意向を確認したおまかせSupporterが明示操作</x:v>
+        <x:v>本人、または意向を確認した家族中心のSupporterが明示操作</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="44" customHeight="1">
@@ -3862,7 +3988,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="B15" s="40" t="str">
-        <x:v>支援スタイル・おまかせ確認</x:v>
+        <x:v>進め方・家族中心の了承確認</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
         <x:v>—</x:v>
@@ -3892,7 +4018,83 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="L15" s="40" t="str">
-        <x:v>本人の了承を確認。本人Accountは任意。途中変更可</x:v>
+        <x:v>本人が進める／家族におまかせする。途中変更可</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="44" customHeight="1">
+      <x:c r="A16" s="40" t="str">
+        <x:v>S12</x:v>
+      </x:c>
+      <x:c r="B16" s="40" t="str">
+        <x:v>Supporter権限</x:v>
+      </x:c>
+      <x:c r="C16" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D16" s="40" t="str">
+        <x:v>●</x:v>
+      </x:c>
+      <x:c r="E16" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="F16" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="G16" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="H16" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="I16" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="J16" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="K16" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="L16" s="40" t="str">
+        <x:v>進め方の初期プリセット後もPermissionを個別変更可</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="44" customHeight="1">
+      <x:c r="A17" s="40" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+      <x:c r="B17" s="40" t="str">
+        <x:v>通知先</x:v>
+      </x:c>
+      <x:c r="C17" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D17" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="E17" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="F17" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="G17" s="40" t="str">
+        <x:v>●</x:v>
+      </x:c>
+      <x:c r="H17" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="I17" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="J17" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="K17" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="L17" s="40" t="str">
+        <x:v>本人／Supporter／双方を将来選択可能。現時点でUI追加不要</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3957,31 +4159,31 @@
       <x:c r="I3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="70" t="str">
+      <x:c r="A4" s="86" t="str">
         <x:v>Case</x:v>
       </x:c>
-      <x:c r="B4" s="70" t="str">
+      <x:c r="B4" s="86" t="str">
         <x:v>位置づけ</x:v>
       </x:c>
-      <x:c r="C4" s="70" t="str">
+      <x:c r="C4" s="86" t="str">
         <x:v>HPに来た人</x:v>
       </x:c>
-      <x:c r="D4" s="70" t="str">
+      <x:c r="D4" s="86" t="str">
         <x:v>語る人</x:v>
       </x:c>
-      <x:c r="E4" s="70" t="str">
+      <x:c r="E4" s="86" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="F4" s="70" t="str">
+      <x:c r="F4" s="86" t="str">
         <x:v>同席・遠隔</x:v>
       </x:c>
-      <x:c r="G4" s="70" t="str">
+      <x:c r="G4" s="86" t="str">
         <x:v>購入者候補</x:v>
       </x:c>
-      <x:c r="H4" s="70" t="str">
+      <x:c r="H4" s="86" t="str">
         <x:v>本人Accountが必要になる時</x:v>
       </x:c>
-      <x:c r="I4" s="70" t="str">
+      <x:c r="I4" s="86" t="str">
         <x:v>要点</x:v>
       </x:c>
     </x:row>
@@ -4037,10 +4239,10 @@
         <x:v>子または本人。別Subcaseで管理。</x:v>
       </x:c>
       <x:c r="H6" s="40" t="str">
-        <x:v>自分で・一緒にでは必要。おまかせでは任意で後から接続可。</x:v>
+        <x:v>本人中心では必要。家族中心では任意で後から接続可。</x:v>
       </x:c>
       <x:c r="I6" s="40" t="str">
-        <x:v>Person中心。自分で／一緒に／おまかせの3スタイル</x:v>
+        <x:v>2つの進め方と個別Permissionを分けて管理</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
@@ -4122,22 +4324,22 @@
       <x:c r="F3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="70" t="str">
+      <x:c r="A4" s="86" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B4" s="70" t="str">
+      <x:c r="B4" s="86" t="str">
         <x:v>論点</x:v>
       </x:c>
-      <x:c r="C4" s="70" t="str">
+      <x:c r="C4" s="86" t="str">
         <x:v>現状案</x:v>
       </x:c>
-      <x:c r="D4" s="70" t="str">
+      <x:c r="D4" s="86" t="str">
         <x:v>状態</x:v>
       </x:c>
-      <x:c r="E4" s="70" t="str">
+      <x:c r="E4" s="86" t="str">
         <x:v>決める理由</x:v>
       </x:c>
-      <x:c r="F4" s="70" t="str">
+      <x:c r="F4" s="86" t="str">
         <x:v>次アクション</x:v>
       </x:c>
     </x:row>
@@ -4149,16 +4351,16 @@
         <x:v>無料3問の語り共有初期値</x:v>
       </x:c>
       <x:c r="C5" s="40" t="str">
-        <x:v>自分で＝本人のみ。一緒に・おまかせ＝制作Supporterと共有。語り単位で本人のみへ変更可</x:v>
+        <x:v>本人のみを基準。語りを見るPermissionのある制作Supporterには共有し、語り単位で変更可</x:v>
       </x:c>
       <x:c r="D5" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
       <x:c r="E5" s="40" t="str">
-        <x:v>支援に必要な閲覧権限と本人の選択余地を両立</x:v>
+        <x:v>進め方と閲覧Permissionを混同せず、本人の選択余地を残す</x:v>
       </x:c>
       <x:c r="F5" s="40" t="str">
-        <x:v>B同席・子購入の実装へ反映</x:v>
+        <x:v>Supporter権限の実装へ反映</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
@@ -4169,16 +4371,16 @@
         <x:v>親支援時の進捗共有初期値</x:v>
       </x:c>
       <x:c r="C6" s="40" t="str">
-        <x:v>自分で＝任意。一緒に・おまかせ＝制作Supporterへ共有</x:v>
+        <x:v>進捗を見るPermissionのあるSupporterへ共有</x:v>
       </x:c>
       <x:c r="D6" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
       <x:c r="E6" s="40" t="str">
-        <x:v>娘の遠隔フォローと制作継続に必要</x:v>
+        <x:v>本人中心でも必要に応じて家族が見守れる</x:v>
       </x:c>
       <x:c r="F6" s="40" t="str">
-        <x:v>支援スタイル選択時の説明へ反映</x:v>
+        <x:v>Supporter権限の実装へ反映</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -4326,19 +4528,19 @@
         <x:v>Q10</x:v>
       </x:c>
       <x:c r="B14" s="40" t="str">
-        <x:v>おまかせ時の本人Account・代理操作</x:v>
+        <x:v>2つの進め方と代理操作</x:v>
       </x:c>
       <x:c r="C14" s="40" t="str">
-        <x:v>Person中心。本人Accountは任意。Supporterが制作・購入・本編開始・仕上げを代理操作</x:v>
+        <x:v>本人が進める／家族におまかせする。家族中心では本人Accountを任意とし、広い制作権限を初期付与</x:v>
       </x:c>
       <x:c r="D14" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
       <x:c r="E14" s="40" t="str">
-        <x:v>高齢の語り手本人にAccountや端末操作を必須にしない</x:v>
+        <x:v>主な操作主体と個別Permissionを分け、高齢者にも自立利用者にも対応</x:v>
       </x:c>
       <x:c r="F14" s="40" t="str">
-        <x:v>06_支援スタイル・権限とBおまかせフローへ反映</x:v>
+        <x:v>06_支援スタイル・権限とBフローへ反映</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
@@ -4346,19 +4548,39 @@
         <x:v>Q11</x:v>
       </x:c>
       <x:c r="B15" s="40" t="str">
-        <x:v>支援スタイル・本人了承確認の保存先</x:v>
+        <x:v>進め方・本人了承・Permissionの保存先</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
-        <x:v>support_mode、confirmed_by、confirmed_at等を記録する案</x:v>
+        <x:v>primary_mode、supporter_permissions、confirmed_by、confirmed_at等を分離して記録する案</x:v>
       </x:c>
       <x:c r="D15" s="40" t="str">
         <x:v>要確認</x:v>
       </x:c>
       <x:c r="E15" s="40" t="str">
-        <x:v>本人Accountなしで広い制作権限を付与する根拠と監査履歴が必要</x:v>
+        <x:v>本人Accountなしの代理操作と途中変更を安全に追跡する</x:v>
       </x:c>
       <x:c r="F15" s="40" t="str">
         <x:v>DB・RLS・監査ログ設計と照合</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="54" customHeight="1">
+      <x:c r="A16" s="40" t="str">
+        <x:v>Q12</x:v>
+      </x:c>
+      <x:c r="B16" s="40" t="str">
+        <x:v>通知先の初期値・保存先</x:v>
+      </x:c>
+      <x:c r="C16" s="40" t="str">
+        <x:v>本人Account有無とPermissionに応じ、本人／Supporter／双方を将来設定可能にする</x:v>
+      </x:c>
+      <x:c r="D16" s="40" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
+      <x:c r="E16" s="40" t="str">
+        <x:v>進め方と通知先を固定せず、参加者変更に追随させる</x:v>
+      </x:c>
+      <x:c r="F16" s="40" t="str">
+        <x:v>既存通知実装と設定保存先を照合</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4385,11 +4607,22 @@
       <x:formula>$D5="要確認"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:conditionalFormatting sqref="A5:F16">
+    <x:cfRule type="expression" dxfId="16" priority="6">
+      <x:formula>$D5="要確認"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="19" priority="7">
+      <x:formula>$D5="要確認"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="D5:D13">
       <x:formula1>"確定,要確認"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D5:D15">
+      <x:formula1>"確定,要確認"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D5:D16">
       <x:formula1>"確定,要確認"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -4454,34 +4687,34 @@
       <x:c r="J3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="70" t="str">
+      <x:c r="A4" s="86" t="str">
         <x:v>Setting ID</x:v>
       </x:c>
-      <x:c r="B4" s="70" t="str">
+      <x:c r="B4" s="86" t="str">
         <x:v>設定・同意名</x:v>
       </x:c>
-      <x:c r="C4" s="70" t="str">
+      <x:c r="C4" s="86" t="str">
         <x:v>利用者が設定する画面</x:v>
       </x:c>
-      <x:c r="D4" s="70" t="str">
+      <x:c r="D4" s="86" t="str">
         <x:v>初期値</x:v>
       </x:c>
-      <x:c r="E4" s="70" t="str">
+      <x:c r="E4" s="86" t="str">
         <x:v>設定できる人</x:v>
       </x:c>
-      <x:c r="F4" s="70" t="str">
+      <x:c r="F4" s="86" t="str">
         <x:v>変更できる時期</x:v>
       </x:c>
-      <x:c r="G4" s="70" t="str">
+      <x:c r="G4" s="86" t="str">
         <x:v>保存先</x:v>
       </x:c>
-      <x:c r="H4" s="70" t="str">
+      <x:c r="H4" s="86" t="str">
         <x:v>関連Flow ID</x:v>
       </x:c>
-      <x:c r="I4" s="70" t="str">
+      <x:c r="I4" s="86" t="str">
         <x:v>実装状態</x:v>
       </x:c>
-      <x:c r="J4" s="70" t="str">
+      <x:c r="J4" s="86" t="str">
         <x:v>根拠仕様</x:v>
       </x:c>
     </x:row>
@@ -4589,16 +4822,16 @@
         <x:v>進捗共有</x:v>
       </x:c>
       <x:c r="C8" s="40" t="str">
-        <x:v>支援スタイル選択／家族とのつながり設定</x:v>
+        <x:v>Supporter権限／家族とのつながり設定</x:v>
       </x:c>
       <x:c r="D8" s="40" t="str">
-        <x:v>自分で＝任意。一緒に・おまかせ＝制作Supporterへ共有</x:v>
+        <x:v>進捗を見るPermissionがある場合のみ共有</x:v>
       </x:c>
       <x:c r="E8" s="40" t="str">
         <x:v>本人または本人の了承を確認したSupporter</x:v>
       </x:c>
       <x:c r="F8" s="40" t="str">
-        <x:v>初回説明後・本人接続後・随時</x:v>
+        <x:v>初回設定・本人接続後・随時</x:v>
       </x:c>
       <x:c r="G8" s="40" t="str">
         <x:v>family_subject_bindings.progress_enabled</x:v>
@@ -4621,13 +4854,13 @@
         <x:v>語り共有 本人のみ／制作Supporter</x:v>
       </x:c>
       <x:c r="C9" s="40" t="str">
-        <x:v>録音保存時／語り設定</x:v>
+        <x:v>録音保存時／Supporter権限／語り設定</x:v>
       </x:c>
       <x:c r="D9" s="40" t="str">
-        <x:v>自分で＝本人のみ。一緒に・おまかせ＝制作Supporterと共有</x:v>
+        <x:v>本人のみ。語りを見るPermissionがある場合は制作Supporterにも共有</x:v>
       </x:c>
       <x:c r="E9" s="40" t="str">
-        <x:v>本人または本人の了承を確認したSupporter。語り単位で本人のみに変更可。</x:v>
+        <x:v>本人または本人の了承を確認したSupporter。語り単位で変更可。</x:v>
       </x:c>
       <x:c r="F9" s="40" t="str">
         <x:v>語り保存時・後から随時</x:v>
@@ -4656,10 +4889,10 @@
         <x:v>仕上げ／掲載する語りの選択</x:v>
       </x:c>
       <x:c r="D10" s="40" t="str">
-        <x:v>共有可能な語りを候補表示</x:v>
+        <x:v>収録設定Permissionがある人に候補表示</x:v>
       </x:c>
       <x:c r="E10" s="40" t="str">
-        <x:v>本人または許可された仕上げ権限者。おまかせではSupporterが代理確定可。</x:v>
+        <x:v>本人または収録設定PermissionのあるSupporter</x:v>
       </x:c>
       <x:c r="F10" s="40" t="str">
         <x:v>制作中・仕上げ・最終確定前</x:v>
@@ -4691,7 +4924,7 @@
         <x:v>非共有</x:v>
       </x:c>
       <x:c r="E11" s="40" t="str">
-        <x:v>本人またはおまかせ権限のSupporter</x:v>
+        <x:v>本人または共有設定PermissionのあるSupporter</x:v>
       </x:c>
       <x:c r="F11" s="40" t="str">
         <x:v>仕上げ時・完成後</x:v>
@@ -4723,7 +4956,7 @@
         <x:v>掲載しない・非公開を基準</x:v>
       </x:c>
       <x:c r="E12" s="40" t="str">
-        <x:v>本人またはおまかせ権限のSupporter</x:v>
+        <x:v>本人または共有設定PermissionのあるSupporter</x:v>
       </x:c>
       <x:c r="F12" s="40" t="str">
         <x:v>仕上げ時・完成後の閲覧方法変更</x:v>
@@ -4755,7 +4988,7 @@
         <x:v>未開始</x:v>
       </x:c>
       <x:c r="E13" s="40" t="str">
-        <x:v>Person本人Accountまたは本人の意向を確認したおまかせ権限のSupporter</x:v>
+        <x:v>Person本人Accountまたは家族中心で開始権限のあるSupporter</x:v>
       </x:c>
       <x:c r="F13" s="40" t="str">
         <x:v>一度だけ。開始後は戻さない。</x:v>
@@ -4810,22 +5043,22 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="B15" s="40" t="str">
-        <x:v>支援スタイル・おまかせ確認</x:v>
+        <x:v>進め方・家族中心の了承確認</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
-        <x:v>対象Person作成／大切な人の物語の設定</x:v>
+        <x:v>対象Person作成／本格利用開始</x:v>
       </x:c>
       <x:c r="D15" s="40" t="str">
         <x:v>未選択</x:v>
       </x:c>
       <x:c r="E15" s="40" t="str">
-        <x:v>Supporter。おまかせ時は語り手本人の了承を確認。</x:v>
+        <x:v>本人またはSupporter。家族中心では語り手本人の了承を確認。</x:v>
       </x:c>
       <x:c r="F15" s="40" t="str">
         <x:v>開始時・購入時・本人接続時・随時</x:v>
       </x:c>
       <x:c r="G15" s="40" t="str">
-        <x:v>要確認（support_mode、confirmed_by、confirmed_at等）</x:v>
+        <x:v>要確認（primary_mode、confirmed_by、confirmed_at等）</x:v>
       </x:c>
       <x:c r="H15" s="40" t="str">
         <x:v>B-CO-020、B-CO-DELEGATED-050、B-DIRECT-DELEGATED-020</x:v>
@@ -4835,6 +5068,70 @@
       </x:c>
       <x:c r="J15" s="40" t="str">
         <x:v>06_支援スタイル・権限／04_運営チェック Q10・Q11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="74" customHeight="1">
+      <x:c r="A16" s="40" t="str">
+        <x:v>S12</x:v>
+      </x:c>
+      <x:c r="B16" s="40" t="str">
+        <x:v>Supporter権限</x:v>
+      </x:c>
+      <x:c r="C16" s="40" t="str">
+        <x:v>Supporter追加／お手伝い範囲の設定</x:v>
+      </x:c>
+      <x:c r="D16" s="40" t="str">
+        <x:v>本人中心＝必要な範囲。家族中心＝広い制作権限プリセット</x:v>
+      </x:c>
+      <x:c r="E16" s="40" t="str">
+        <x:v>本人または本人の了承を確認したSupporter</x:v>
+      </x:c>
+      <x:c r="F16" s="40" t="str">
+        <x:v>Supporter追加時・開始後随時</x:v>
+      </x:c>
+      <x:c r="G16" s="40" t="str">
+        <x:v>要確認（project_supporter_permissions等）</x:v>
+      </x:c>
+      <x:c r="H16" s="40" t="str">
+        <x:v>B-CO-020、B-CO-DELEGATED-050、B-DIRECT-DELEGATED-020、B-CO-GIFT-050</x:v>
+      </x:c>
+      <x:c r="I16" s="40" t="str">
+        <x:v>未実装</x:v>
+      </x:c>
+      <x:c r="J16" s="40" t="str">
+        <x:v>06_支援スタイル・権限／04_運営チェック Q11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="74" customHeight="1">
+      <x:c r="A17" s="40" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+      <x:c r="B17" s="40" t="str">
+        <x:v>通知先</x:v>
+      </x:c>
+      <x:c r="C17" s="40" t="str">
+        <x:v>現時点では既存通知ロジック。将来は通知設定</x:v>
+      </x:c>
+      <x:c r="D17" s="40" t="str">
+        <x:v>本人Account有無とPermissionに応じた既定</x:v>
+      </x:c>
+      <x:c r="E17" s="40" t="str">
+        <x:v>本人または通知管理PermissionのあるSupporter</x:v>
+      </x:c>
+      <x:c r="F17" s="40" t="str">
+        <x:v>本人接続時・Supporter変更時・随時</x:v>
+      </x:c>
+      <x:c r="G17" s="40" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
+      <x:c r="H17" s="40" t="str">
+        <x:v>B-CO-GIFT-050、B-CO-DELEGATED-050、B-REMOTE-GIFT-040</x:v>
+      </x:c>
+      <x:c r="I17" s="40" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
+      <x:c r="J17" s="40" t="str">
+        <x:v>06_支援スタイル・権限／04_運営チェック Q12</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4861,11 +5158,22 @@
       <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:conditionalFormatting sqref="A5:J17">
+    <x:cfRule type="expression" dxfId="17" priority="6">
+      <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="20" priority="7">
+      <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="I5:I14">
       <x:formula1>"実装済み,一部実装,未実装,要確認"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I5:I15">
+      <x:formula1>"実装済み,一部実装,未実装,要確認"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I5:I17">
       <x:formula1>"実装済み,一部実装,未実装,要確認"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -4877,16 +5185,16 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="31" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="57" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="64" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="28" t="str">
-        <x:v>支援スタイル・権限</x:v>
+        <x:v>進め方とSupporter権限</x:v>
       </x:c>
       <x:c r="B1" s="28"/>
       <x:c r="C1" s="28"/>
@@ -4895,7 +5203,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="30" t="str">
-        <x:v>Personが作品の主体。本人Account、Supporter Account、または両方が、選んだ支援スタイルに応じて同じPersonの制作を担う。</x:v>
+        <x:v>進め方は主な操作主体だけを決める。Supporter権限、本人Account、通知先は独立して設定し、開始後も変更できる。</x:v>
       </x:c>
       <x:c r="B2" s="30"/>
       <x:c r="C2" s="30"/>
@@ -4910,258 +5218,323 @@
       <x:c r="E3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="70" t="str">
-        <x:v>操作・条件</x:v>
-      </x:c>
-      <x:c r="B4" s="70" t="str">
-        <x:v>自分で進める</x:v>
-      </x:c>
-      <x:c r="C4" s="70" t="str">
-        <x:v>一緒に進める</x:v>
-      </x:c>
-      <x:c r="D4" s="70" t="str">
-        <x:v>おまかせする</x:v>
-      </x:c>
-      <x:c r="E4" s="70" t="str">
-        <x:v>補足</x:v>
+      <x:c r="A4" s="86" t="str">
+        <x:v>進め方</x:v>
+      </x:c>
+      <x:c r="B4" s="86" t="str">
+        <x:v>中心となる端末・Account</x:v>
+      </x:c>
+      <x:c r="C4" s="86" t="str">
+        <x:v>Supporterの初期状態</x:v>
+      </x:c>
+      <x:c r="D4" s="86" t="str">
+        <x:v>本人Account</x:v>
+      </x:c>
+      <x:c r="E4" s="86" t="str">
+        <x:v>ユーザー向け説明候補</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="66" t="str">
-        <x:v>本人Account必須</x:v>
+        <x:v>本人が進める</x:v>
       </x:c>
       <x:c r="B5" s="40" t="str">
-        <x:v>○</x:v>
+        <x:v>本人のスマホ／本人Account</x:v>
       </x:c>
       <x:c r="C5" s="40" t="str">
-        <x:v>○</x:v>
-      </x:c>
-      <x:c r="D5" s="74" t="str">
-        <x:v>×</x:v>
+        <x:v>なし、または必要な範囲を選択</x:v>
+      </x:c>
+      <x:c r="D5" s="40" t="str">
+        <x:v>必須</x:v>
       </x:c>
       <x:c r="E5" s="40" t="str">
-        <x:v>おまかせでは本人Accountを後から任意で接続できる</x:v>
+        <x:v>本人のスマホを中心に進めます。ご家族にも、必要な範囲でお手伝いしてもらえます。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="66" t="str">
-        <x:v>Supporter Account</x:v>
+        <x:v>家族におまかせする</x:v>
       </x:c>
       <x:c r="B6" s="40" t="str">
-        <x:v>任意</x:v>
+        <x:v>家族の端末／Supporter Account</x:v>
       </x:c>
       <x:c r="C6" s="40" t="str">
-        <x:v>○</x:v>
-      </x:c>
-      <x:c r="D6" s="74" t="str">
-        <x:v>○</x:v>
+        <x:v>制作に必要な権限を広く付与</x:v>
+      </x:c>
+      <x:c r="D6" s="40" t="str">
+        <x:v>任意・後から接続可</x:v>
       </x:c>
       <x:c r="E6" s="40" t="str">
-        <x:v>支援する家族・信頼できる人のAccount</x:v>
+        <x:v>家族の端末を中心に進めます。語りの収録から写真、本への仕上げまでおまかせできます。ご本人のスマホからも参加できます。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="66" t="str">
-        <x:v>録音操作</x:v>
+        <x:v>変更</x:v>
       </x:c>
       <x:c r="B7" s="40" t="str">
-        <x:v>本人</x:v>
+        <x:v>開始後も変更可</x:v>
       </x:c>
       <x:c r="C7" s="40" t="str">
-        <x:v>本人／Supporter</x:v>
-      </x:c>
-      <x:c r="D7" s="74" t="str">
-        <x:v>Supporter</x:v>
+        <x:v>権限は個別に変更可</x:v>
+      </x:c>
+      <x:c r="D7" s="40" t="str">
+        <x:v>既存Personへ後付け</x:v>
       </x:c>
       <x:c r="E7" s="40" t="str">
-        <x:v>語る人は常にPerson本人。端末操作は別の人でもよい</x:v>
+        <x:v>進め方やお手伝いの範囲は、あとからいつでも変更できます。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
-      <x:c r="A8" s="66" t="str">
-        <x:v>全語りの閲覧</x:v>
-      </x:c>
-      <x:c r="B8" s="40" t="str">
-        <x:v>本人</x:v>
-      </x:c>
-      <x:c r="C8" s="40" t="str">
-        <x:v>本人＋制作Supporter</x:v>
-      </x:c>
-      <x:c r="D8" s="74" t="str">
-        <x:v>制作Supporter</x:v>
-      </x:c>
-      <x:c r="E8" s="40" t="str">
-        <x:v>語り単位で本人のみへ変更できる</x:v>
-      </x:c>
+      <x:c r="A8" s="41"/>
+      <x:c r="B8" s="41"/>
+      <x:c r="C8" s="41"/>
+      <x:c r="D8" s="41"/>
+      <x:c r="E8" s="41"/>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
-      <x:c r="A9" s="66" t="str">
-        <x:v>文章編集・語り直し</x:v>
-      </x:c>
-      <x:c r="B9" s="40" t="str">
-        <x:v>本人</x:v>
-      </x:c>
-      <x:c r="C9" s="40" t="str">
-        <x:v>双方</x:v>
-      </x:c>
-      <x:c r="D9" s="74" t="str">
-        <x:v>Supporter代理可</x:v>
-      </x:c>
-      <x:c r="E9" s="40" t="str">
-        <x:v>本人の意向を確認しながら行う</x:v>
+      <x:c r="A9" s="86" t="str">
+        <x:v>Supporter権限</x:v>
+      </x:c>
+      <x:c r="B9" s="86" t="str">
+        <x:v>本人が進める 初期状態</x:v>
+      </x:c>
+      <x:c r="C9" s="86" t="str">
+        <x:v>家族におまかせ 初期状態</x:v>
+      </x:c>
+      <x:c r="D9" s="86" t="str">
+        <x:v>開始後の変更</x:v>
+      </x:c>
+      <x:c r="E9" s="86" t="str">
+        <x:v>権限の意味</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" s="66" t="str">
-        <x:v>写真追加</x:v>
-      </x:c>
-      <x:c r="B10" s="40" t="str">
-        <x:v>本人</x:v>
-      </x:c>
-      <x:c r="C10" s="40" t="str">
-        <x:v>双方</x:v>
-      </x:c>
-      <x:c r="D10" s="74" t="str">
-        <x:v>Supporter代理可</x:v>
+        <x:v>進捗を見る</x:v>
+      </x:c>
+      <x:c r="B10" s="90" t="str">
+        <x:v>OFF／追加時に選択</x:v>
+      </x:c>
+      <x:c r="C10" s="90" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="D10" s="40" t="str">
+        <x:v>個別にON／OFF</x:v>
       </x:c>
       <x:c r="E10" s="40" t="str">
-        <x:v>家族が離れた場所から追加できる</x:v>
+        <x:v>テーマや制作の進み具合を確認する</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
       <x:c r="A11" s="66" t="str">
-        <x:v>共有範囲の設定</x:v>
-      </x:c>
-      <x:c r="B11" s="40" t="str">
-        <x:v>本人</x:v>
-      </x:c>
-      <x:c r="C11" s="40" t="str">
-        <x:v>双方</x:v>
-      </x:c>
-      <x:c r="D11" s="74" t="str">
-        <x:v>Supporter代理可</x:v>
+        <x:v>語りを見る</x:v>
+      </x:c>
+      <x:c r="B11" s="90" t="str">
+        <x:v>OFF／追加時に選択</x:v>
+      </x:c>
+      <x:c r="C11" s="90" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="D11" s="40" t="str">
+        <x:v>個別にON／OFF</x:v>
       </x:c>
       <x:c r="E11" s="40" t="str">
-        <x:v>本人の意向を確認。既定は制作Supporterと共有</x:v>
+        <x:v>語りの内容を閲覧する。語り単位の非共有設定を優先</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" s="66" t="str">
-        <x:v>ブック収録選択</x:v>
-      </x:c>
-      <x:c r="B12" s="40" t="str">
-        <x:v>本人</x:v>
-      </x:c>
-      <x:c r="C12" s="40" t="str">
-        <x:v>双方</x:v>
-      </x:c>
-      <x:c r="D12" s="74" t="str">
-        <x:v>Supporter代理可</x:v>
+        <x:v>録音・語りを追加する</x:v>
+      </x:c>
+      <x:c r="B12" s="90" t="str">
+        <x:v>OFF／追加時に選択</x:v>
+      </x:c>
+      <x:c r="C12" s="90" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="D12" s="40" t="str">
+        <x:v>個別にON／OFF</x:v>
       </x:c>
       <x:c r="E12" s="40" t="str">
-        <x:v>本人に確認しながら掲載・除外を決める</x:v>
+        <x:v>本人と同席して録音操作を行い、Personへ語りを追加する</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="66" t="str">
-        <x:v>ブック編集</x:v>
-      </x:c>
-      <x:c r="B13" s="40" t="str">
-        <x:v>本人</x:v>
-      </x:c>
-      <x:c r="C13" s="40" t="str">
-        <x:v>双方</x:v>
-      </x:c>
-      <x:c r="D13" s="74" t="str">
-        <x:v>Supporter代理可</x:v>
+        <x:v>写真を追加・整理する</x:v>
+      </x:c>
+      <x:c r="B13" s="90" t="str">
+        <x:v>OFF／追加時に選択</x:v>
+      </x:c>
+      <x:c r="C13" s="90" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="D13" s="40" t="str">
+        <x:v>個別にON／OFF</x:v>
       </x:c>
       <x:c r="E13" s="40" t="str">
-        <x:v>並び順、文章、写真、タイトル等</x:v>
+        <x:v>写真の追加、並び替え、説明の編集を行う</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="66" t="str">
-        <x:v>Webブック・QR設定</x:v>
-      </x:c>
-      <x:c r="B14" s="40" t="str">
-        <x:v>本人</x:v>
-      </x:c>
-      <x:c r="C14" s="40" t="str">
-        <x:v>双方</x:v>
-      </x:c>
-      <x:c r="D14" s="74" t="str">
-        <x:v>Supporter代理可</x:v>
+        <x:v>文章を編集する</x:v>
+      </x:c>
+      <x:c r="B14" s="90" t="str">
+        <x:v>OFF／追加時に選択</x:v>
+      </x:c>
+      <x:c r="C14" s="90" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="D14" s="40" t="str">
+        <x:v>個別にON／OFF</x:v>
       </x:c>
       <x:c r="E14" s="40" t="str">
-        <x:v>公開範囲は作品単位。初期値は非公開側</x:v>
+        <x:v>文章の修正や語り直しの反映を行う</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="66" t="str">
-        <x:v>最終確定・製本注文・増刷</x:v>
-      </x:c>
-      <x:c r="B15" s="40" t="str">
-        <x:v>本人</x:v>
-      </x:c>
-      <x:c r="C15" s="40" t="str">
-        <x:v>本人中心／共同</x:v>
-      </x:c>
-      <x:c r="D15" s="74" t="str">
-        <x:v>Supporter代理可</x:v>
+        <x:v>語りの共有範囲を設定する</x:v>
+      </x:c>
+      <x:c r="B15" s="90" t="str">
+        <x:v>OFF／追加時に選択</x:v>
+      </x:c>
+      <x:c r="C15" s="90" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="D15" s="40" t="str">
+        <x:v>個別にON／OFF</x:v>
       </x:c>
       <x:c r="E15" s="40" t="str">
-        <x:v>操作主体と確定日時を記録する</x:v>
+        <x:v>本人の意向を確認し、閲覧できる範囲を設定する</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="66" t="str">
-        <x:v>本編開始</x:v>
-      </x:c>
-      <x:c r="B16" s="40" t="str">
-        <x:v>本人</x:v>
-      </x:c>
-      <x:c r="C16" s="40" t="str">
-        <x:v>本人／共同</x:v>
-      </x:c>
-      <x:c r="D16" s="74" t="str">
-        <x:v>Supporter代理可</x:v>
+        <x:v>本への収録を設定する</x:v>
+      </x:c>
+      <x:c r="B16" s="90" t="str">
+        <x:v>OFF／追加時に選択</x:v>
+      </x:c>
+      <x:c r="C16" s="90" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="D16" s="40" t="str">
+        <x:v>個別にON／OFF</x:v>
       </x:c>
       <x:c r="E16" s="40" t="str">
-        <x:v>本人の続行意思を確認。開始時に返金保証終了</x:v>
+        <x:v>本へ入れる語り・写真を選択する</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" s="66" t="str">
-        <x:v>支払い</x:v>
-      </x:c>
-      <x:c r="B17" s="40" t="str">
-        <x:v>本人等</x:v>
-      </x:c>
-      <x:c r="C17" s="40" t="str">
-        <x:v>どちらでも</x:v>
-      </x:c>
-      <x:c r="D17" s="74" t="str">
-        <x:v>Supporter想定</x:v>
+        <x:v>ブックを編集する</x:v>
+      </x:c>
+      <x:c r="B17" s="90" t="str">
+        <x:v>OFF／追加時に選択</x:v>
+      </x:c>
+      <x:c r="C17" s="90" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="D17" s="40" t="str">
+        <x:v>個別にON／OFF</x:v>
       </x:c>
       <x:c r="E17" s="40" t="str">
-        <x:v>PayerはPerson・操作者と独立して記録する</x:v>
+        <x:v>タイトル、文章、写真、並び順などを編集する</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="48" customHeight="1">
       <x:c r="A18" s="66" t="str">
-        <x:v>本人Accountの後付け</x:v>
-      </x:c>
-      <x:c r="B18" s="40" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C18" s="40" t="str">
-        <x:v>接続済み</x:v>
-      </x:c>
-      <x:c r="D18" s="74" t="str">
-        <x:v>任意</x:v>
+        <x:v>仕上げる</x:v>
+      </x:c>
+      <x:c r="B18" s="90" t="str">
+        <x:v>OFF／追加時に選択</x:v>
+      </x:c>
+      <x:c r="C18" s="90" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="D18" s="40" t="str">
+        <x:v>個別にON／OFF</x:v>
       </x:c>
       <x:c r="E18" s="40" t="str">
-        <x:v>接続しても既存Person・Projectを新規作成しない</x:v>
+        <x:v>Webブック、QR、共有範囲、最終版を設定する</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="48" customHeight="1">
+      <x:c r="A19" s="66" t="str">
+        <x:v>製本・注文する</x:v>
+      </x:c>
+      <x:c r="B19" s="90" t="str">
+        <x:v>OFF／追加時に選択</x:v>
+      </x:c>
+      <x:c r="C19" s="90" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="D19" s="40" t="str">
+        <x:v>個別にON／OFF</x:v>
+      </x:c>
+      <x:c r="E19" s="40" t="str">
+        <x:v>製本注文、追加注文、増刷を行う</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="48" customHeight="1">
+      <x:c r="A20" s="41"/>
+      <x:c r="B20" s="41"/>
+      <x:c r="C20" s="41"/>
+      <x:c r="D20" s="41"/>
+      <x:c r="E20" s="41"/>
+    </x:row>
+    <x:row r="21" ht="48" customHeight="1">
+      <x:c r="A21" s="86" t="str">
+        <x:v>独立して管理する項目</x:v>
+      </x:c>
+      <x:c r="B21" s="86" t="str">
+        <x:v>値・選択肢</x:v>
+      </x:c>
+      <x:c r="C21" s="86" t="str">
+        <x:v>進め方との関係</x:v>
+      </x:c>
+      <x:c r="D21" s="86" t="str">
+        <x:v>変更</x:v>
+      </x:c>
+      <x:c r="E21" s="86" t="str">
+        <x:v>補足</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="48" customHeight="1">
+      <x:c r="A22" s="66" t="str">
+        <x:v>本人Account</x:v>
+      </x:c>
+      <x:c r="B22" s="40" t="str">
+        <x:v>あり／なし</x:v>
+      </x:c>
+      <x:c r="C22" s="40" t="str">
+        <x:v>家族中心ではなしでも完結</x:v>
+      </x:c>
+      <x:c r="D22" s="40" t="str">
+        <x:v>後から追加可</x:v>
+      </x:c>
+      <x:c r="E22" s="40" t="str">
+        <x:v>接続時に既存Person・Projectを新規作成しない</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="48" customHeight="1">
+      <x:c r="A23" s="66" t="str">
+        <x:v>通知先</x:v>
+      </x:c>
+      <x:c r="B23" s="40" t="str">
+        <x:v>本人／Supporter／双方</x:v>
+      </x:c>
+      <x:c r="C23" s="40" t="str">
+        <x:v>進め方には固定しない</x:v>
+      </x:c>
+      <x:c r="D23" s="40" t="str">
+        <x:v>将来変更可</x:v>
+      </x:c>
+      <x:c r="E23" s="40" t="str">
+        <x:v>現時点ではUIを増やさず、将来設定可能な構造を前提とする</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: define supporter and family sharing
</commit_message>
<xml_diff>
--- a/docs/product/user-flow/user-flow-master.xlsx
+++ b/docs/product/user-flow/user-flow-master.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="Re93806d8928241dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_利用動線" sheetId="2" r:id="R682eaac39b764301"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定同意" sheetId="3" r:id="Re3a45a3e111f4fd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ケース一覧" sheetId="4" r:id="R8b404681be904d5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_運営チェック" sheetId="5" r:id="R09ef5931515a4d2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_実装対応" sheetId="6" r:id="R97853221312a4b2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_支援スタイル・権限" sheetId="7" r:id="R28f5b3081d014bbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="R30f2e29ecc134bf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_利用動線" sheetId="2" r:id="R86dfb88b1cce4af9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定同意" sheetId="3" r:id="Rf0116c1801ee473f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ケース一覧" sheetId="4" r:id="Rb01a26c3dc954996"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_運営チェック" sheetId="5" r:id="R2c0050a225a540b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_実装対応" sheetId="6" r:id="Rd53634f0194948e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_支援スタイル・権限" sheetId="7" r:id="R3545b792b82f4141"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -89,7 +89,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="20">
+  <x:fills count="22">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -186,6 +186,16 @@
         <x:fgColor rgb="FFEEF4F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF315B5B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF4F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -208,7 +218,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="91">
+  <x:cellXfs count="99">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -416,11 +426,61 @@
     <x:xf numFmtId="0" fontId="7" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="21">
+  <x:dxfs count="24">
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:color rgb="FF8A5A00"/>
@@ -855,13 +915,13 @@
       <x:c r="C3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="86" t="str">
+      <x:c r="A4" s="94" t="str">
         <x:v>シート</x:v>
       </x:c>
-      <x:c r="B4" s="86" t="str">
+      <x:c r="B4" s="94" t="str">
         <x:v>役割</x:v>
       </x:c>
-      <x:c r="C4" s="86" t="str">
+      <x:c r="C4" s="94" t="str">
         <x:v>ポイント</x:v>
       </x:c>
     </x:row>
@@ -925,10 +985,10 @@
         <x:v>06_支援スタイル・権限</x:v>
       </x:c>
       <x:c r="B10" s="40" t="str">
-        <x:v>進め方と権限の基準</x:v>
+        <x:v>進め方と関係者の基準</x:v>
       </x:c>
       <x:c r="C10" s="40" t="str">
-        <x:v>2つの進め方、個別のSupporter権限、本人Account、通知先を分けて定義する。</x:v>
+        <x:v>2つの進め方、Supporter、家族・Viewer、本人Account、通知先を分けて定義する。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
@@ -937,13 +997,13 @@
       <x:c r="C11" s="41"/>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
-      <x:c r="A12" s="89" t="str">
+      <x:c r="A12" s="97" t="str">
         <x:v>更新ルール</x:v>
       </x:c>
-      <x:c r="B12" s="89" t="str">
+      <x:c r="B12" s="97" t="str">
         <x:v>同名ファイルを更新</x:v>
       </x:c>
-      <x:c r="C12" s="89" t="str">
+      <x:c r="C12" s="97" t="str">
         <x:v>別バージョンのExcelを増やさず、変更理由と履歴はGitで管理する。</x:v>
       </x:c>
     </x:row>
@@ -1018,7 +1078,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="30" t="str">
-        <x:v>進め方は主な操作主体だけを表す。Supporter権限、本人Account、通知先は別に管理し、途中で変更できる。</x:v>
+        <x:v>進め方は主な操作主体だけを表す。Supporterは制作内部へ原則フルアクセスし、家族・Viewerへの共有とは分けて管理する。</x:v>
       </x:c>
       <x:c r="B2" s="30"/>
       <x:c r="C2" s="30"/>
@@ -1073,79 +1133,79 @@
       <x:c r="Y3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="86" t="str">
+      <x:c r="A4" s="94" t="str">
         <x:v>Flow ID</x:v>
       </x:c>
-      <x:c r="B4" s="86" t="str">
+      <x:c r="B4" s="94" t="str">
         <x:v>Case</x:v>
       </x:c>
-      <x:c r="C4" s="86" t="str">
+      <x:c r="C4" s="94" t="str">
         <x:v>Subcase</x:v>
       </x:c>
-      <x:c r="D4" s="86" t="str">
+      <x:c r="D4" s="94" t="str">
         <x:v>進め方</x:v>
       </x:c>
-      <x:c r="E4" s="86" t="str">
+      <x:c r="E4" s="94" t="str">
         <x:v>Step</x:v>
       </x:c>
-      <x:c r="F4" s="86" t="str">
+      <x:c r="F4" s="94" t="str">
         <x:v>ユーザー行動</x:v>
       </x:c>
-      <x:c r="G4" s="86" t="str">
+      <x:c r="G4" s="94" t="str">
         <x:v>ユーザーへの説明</x:v>
       </x:c>
-      <x:c r="H4" s="86" t="str">
+      <x:c r="H4" s="94" t="str">
         <x:v>利用中Account</x:v>
       </x:c>
-      <x:c r="I4" s="86" t="str">
+      <x:c r="I4" s="94" t="str">
         <x:v>このStepの操作者</x:v>
       </x:c>
-      <x:c r="J4" s="86" t="str">
+      <x:c r="J4" s="94" t="str">
         <x:v>このStepで語る人</x:v>
       </x:c>
-      <x:c r="K4" s="86" t="str">
+      <x:c r="K4" s="94" t="str">
         <x:v>Person</x:v>
       </x:c>
-      <x:c r="L4" s="86" t="str">
+      <x:c r="L4" s="94" t="str">
         <x:v>Payer</x:v>
       </x:c>
-      <x:c r="M4" s="86" t="str">
+      <x:c r="M4" s="94" t="str">
         <x:v>Supporter</x:v>
       </x:c>
-      <x:c r="N4" s="86" t="str">
+      <x:c r="N4" s="94" t="str">
         <x:v>Device</x:v>
       </x:c>
-      <x:c r="O4" s="86" t="str">
+      <x:c r="O4" s="94" t="str">
         <x:v>現在状態</x:v>
       </x:c>
-      <x:c r="P4" s="86" t="str">
+      <x:c r="P4" s="94" t="str">
         <x:v>分岐条件</x:v>
       </x:c>
-      <x:c r="Q4" s="86" t="str">
+      <x:c r="Q4" s="94" t="str">
         <x:v>次の状態</x:v>
       </x:c>
-      <x:c r="R4" s="86" t="str">
+      <x:c r="R4" s="94" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="S4" s="86" t="str">
+      <x:c r="S4" s="94" t="str">
         <x:v>購入</x:v>
       </x:c>
-      <x:c r="T4" s="86" t="str">
+      <x:c r="T4" s="94" t="str">
         <x:v>本人認証</x:v>
       </x:c>
-      <x:c r="U4" s="86" t="str">
+      <x:c r="U4" s="94" t="str">
         <x:v>設定・同意</x:v>
       </x:c>
-      <x:c r="V4" s="86" t="str">
+      <x:c r="V4" s="94" t="str">
         <x:v>内容共有</x:v>
       </x:c>
-      <x:c r="W4" s="86" t="str">
+      <x:c r="W4" s="94" t="str">
         <x:v>進捗共有</x:v>
       </x:c>
-      <x:c r="X4" s="86" t="str">
+      <x:c r="X4" s="94" t="str">
         <x:v>内部メモ</x:v>
       </x:c>
-      <x:c r="Y4" s="86" t="str">
+      <x:c r="Y4" s="94" t="str">
         <x:v>確定度</x:v>
       </x:c>
     </x:row>
@@ -1288,10 +1348,10 @@
         <x:v>済</x:v>
       </x:c>
       <x:c r="U6" s="40" t="str">
-        <x:v>語り共有初期値</x:v>
+        <x:v>家族共有初期値</x:v>
       </x:c>
       <x:c r="V6" s="40" t="str">
-        <x:v>本人のみ</x:v>
+        <x:v>家族に共有しない</x:v>
       </x:c>
       <x:c r="W6" s="40" t="str">
         <x:v>—</x:v>
@@ -1631,7 +1691,7 @@
         <x:v>HP→大切な人の物語→一緒に試す</x:v>
       </x:c>
       <x:c r="G11" s="40" t="str">
-        <x:v>このスマホで一緒に3問試せます。続ける場合は、本人のスマホをつなぐか、ご家族がおまかせで進められます。</x:v>
+        <x:v>このスマホで一緒に3問試せます。続ける場合は、本人のスマホをつなぐか、家族・信頼する方におまかせできます。</x:v>
       </x:c>
       <x:c r="H11" s="40" t="str">
         <x:v>なし</x:v>
@@ -1750,13 +1810,13 @@
         <x:v>親なし</x:v>
       </x:c>
       <x:c r="U12" s="40" t="str">
-        <x:v>対象Person・進め方・Supporter権限</x:v>
+        <x:v>対象Person・進め方・Supporter参加・制作アクセス</x:v>
       </x:c>
       <x:c r="V12" s="40" t="str">
-        <x:v>未設定</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W12" s="40" t="str">
-        <x:v>設定候補</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X12" s="40" t="str">
         <x:v>actor Accountとsubject Personを分離</x:v>
@@ -1776,7 +1836,7 @@
         <x:v>同席3問</x:v>
       </x:c>
       <x:c r="D13" s="40" t="str">
-        <x:v>未選択（家族端末で体験）</x:v>
+        <x:v>未選択（Supporter端末で体験）</x:v>
       </x:c>
       <x:c r="E13" s="40" t="n">
         <x:v>3</x:v>
@@ -1827,13 +1887,13 @@
         <x:v>母なし</x:v>
       </x:c>
       <x:c r="U13" s="40" t="str">
-        <x:v>進め方・Supporter権限・共有設定</x:v>
+        <x:v>進め方・Supporter参加・制作アクセス・共有設定</x:v>
       </x:c>
       <x:c r="V13" s="40" t="str">
-        <x:v>語りを見る権限のあるSupporterと共有</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W13" s="40" t="str">
-        <x:v>進捗を見る権限に従う</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X13" s="40" t="str">
         <x:v>Account＝子、語る人＝母、Person＝母</x:v>
@@ -1853,7 +1913,7 @@
         <x:v>同席3問・子購入</x:v>
       </x:c>
       <x:c r="D14" s="40" t="str">
-        <x:v>未選択→本人が進める／家族におまかせする</x:v>
+        <x:v>未選択→本人が進める／サポーターにおまかせする</x:v>
       </x:c>
       <x:c r="E14" s="40" t="n">
         <x:v>4</x:v>
@@ -1862,7 +1922,7 @@
         <x:v>子が購入して贈る</x:v>
       </x:c>
       <x:c r="G14" s="40" t="str">
-        <x:v>購入後、本人のスマホで続けるか、ご家族がおまかせで進めるか選べます。</x:v>
+        <x:v>購入後、本人のスマホで続けるか、家族・信頼する方におまかせするか選べます。</x:v>
       </x:c>
       <x:c r="H14" s="40" t="str">
         <x:v>子</x:v>
@@ -1907,10 +1967,10 @@
         <x:v>購入条件・45日保証</x:v>
       </x:c>
       <x:c r="V14" s="40" t="str">
-        <x:v>維持</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W14" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X14" s="40" t="str">
         <x:v>購入だけで本編開始しない</x:v>
@@ -1930,7 +1990,7 @@
         <x:v>同席3問・子購入・おまかせ</x:v>
       </x:c>
       <x:c r="D15" s="40" t="str">
-        <x:v>家族におまかせする</x:v>
+        <x:v>サポーターにおまかせする</x:v>
       </x:c>
       <x:c r="E15" s="40" t="n">
         <x:v>5</x:v>
@@ -1981,16 +2041,16 @@
         <x:v>不要</x:v>
       </x:c>
       <x:c r="U15" s="40" t="str">
-        <x:v>進め方・おまかせ確認・制作権限</x:v>
+        <x:v>進め方・おまかせ確認・Supporter制作アクセス</x:v>
       </x:c>
       <x:c r="V15" s="40" t="str">
-        <x:v>語りを見る権限のあるSupporterと共有</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W15" s="40" t="str">
-        <x:v>進捗を見る権限に従う</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X15" s="40" t="str">
-        <x:v>primary_mode＝家族中心。制作権限は個別Permission</x:v>
+        <x:v>primary_mode＝supporter。Supporterは制作内部へ原則フルアクセス</x:v>
       </x:c>
       <x:c r="Y15" s="40" t="str">
         <x:v>確定</x:v>
@@ -2007,7 +2067,7 @@
         <x:v>同席3問・子購入・おまかせ</x:v>
       </x:c>
       <x:c r="D16" s="40" t="str">
-        <x:v>家族におまかせする</x:v>
+        <x:v>サポーターにおまかせする</x:v>
       </x:c>
       <x:c r="E16" s="40" t="n">
         <x:v>6</x:v>
@@ -2061,10 +2121,10 @@
         <x:v>本編開始確認</x:v>
       </x:c>
       <x:c r="V16" s="40" t="str">
-        <x:v>制作Supporterと共有</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W16" s="40" t="str">
-        <x:v>共有</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X16" s="40" t="str">
         <x:v>actor＝娘、subject＝母として開始を記録</x:v>
@@ -2084,7 +2144,7 @@
         <x:v>同席3問・子購入・おまかせ</x:v>
       </x:c>
       <x:c r="D17" s="40" t="str">
-        <x:v>家族におまかせする</x:v>
+        <x:v>サポーターにおまかせする</x:v>
       </x:c>
       <x:c r="E17" s="40" t="n">
         <x:v>7</x:v>
@@ -2138,10 +2198,10 @@
         <x:v>共有・収録・Web・QR・最終確定</x:v>
       </x:c>
       <x:c r="V17" s="40" t="str">
-        <x:v>制作Supporterと共有（変更可）</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W17" s="40" t="str">
-        <x:v>共有</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X17" s="40" t="str">
         <x:v>本人Accountは後から任意で接続可能</x:v>
@@ -2215,10 +2275,10 @@
         <x:v>本人接続・進捗共有</x:v>
       </x:c>
       <x:c r="V18" s="40" t="str">
-        <x:v>本人権限</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W18" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X18" s="40" t="str">
         <x:v>新しいPerson・Projectを作らない</x:v>
@@ -2292,10 +2352,10 @@
         <x:v>本編開始確認</x:v>
       </x:c>
       <x:c r="V19" s="40" t="str">
-        <x:v>語りごと</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W19" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X19" s="40" t="str">
         <x:v>娘はSupporterのまま</x:v>
@@ -2446,10 +2506,10 @@
         <x:v>招待・進捗説明</x:v>
       </x:c>
       <x:c r="V21" s="40" t="str">
-        <x:v>未設定</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W21" s="40" t="str">
-        <x:v>設定候補</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X21" s="40" t="str">
         <x:v>送信成功を推定しない</x:v>
@@ -2523,10 +2583,10 @@
         <x:v>体験同意</x:v>
       </x:c>
       <x:c r="V22" s="40" t="str">
-        <x:v>本人のみ</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W22" s="40" t="str">
-        <x:v>完了≠続行</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X22" s="40" t="str">
         <x:v>Account登録を必須にしない</x:v>
@@ -2600,10 +2660,10 @@
         <x:v>続行意思・通知先説明</x:v>
       </x:c>
       <x:c r="V23" s="40" t="str">
-        <x:v>維持</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W23" s="40" t="str">
-        <x:v>完了≠続行</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X23" s="40" t="str">
         <x:v>Cは独立契約フローではない</x:v>
@@ -2677,10 +2737,10 @@
         <x:v>購入条件・45日保証</x:v>
       </x:c>
       <x:c r="V24" s="40" t="str">
-        <x:v>維持</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W24" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X24" s="40" t="str">
         <x:v>二重購入を防止</x:v>
@@ -2754,10 +2814,10 @@
         <x:v>本人接続・進捗共有</x:v>
       </x:c>
       <x:c r="V25" s="40" t="str">
-        <x:v>本人権限</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W25" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X25" s="40" t="str">
         <x:v>45日保証は本編開始前まで</x:v>
@@ -2831,10 +2891,10 @@
         <x:v>通知先・購入案内</x:v>
       </x:c>
       <x:c r="V26" s="40" t="str">
-        <x:v>維持</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W26" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X26" s="40" t="str">
         <x:v>購入義務や代理課金ではない</x:v>
@@ -2908,10 +2968,10 @@
         <x:v>本人接続・購入条件・30日保証</x:v>
       </x:c>
       <x:c r="V27" s="40" t="str">
-        <x:v>本人権限</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W27" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X27" s="40" t="str">
         <x:v>購入とAccount接続の厳密な順序は要確認</x:v>
@@ -2985,10 +3045,10 @@
         <x:v>本編開始確認</x:v>
       </x:c>
       <x:c r="V28" s="40" t="str">
-        <x:v>語りごと</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W28" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X28" s="40" t="str">
         <x:v>同じPersonを継続</x:v>
@@ -3008,7 +3068,7 @@
         <x:v>3問なし・子購入</x:v>
       </x:c>
       <x:c r="D29" s="40" t="str">
-        <x:v>未選択→本人が進める／家族におまかせする</x:v>
+        <x:v>未選択→本人が進める／サポーターにおまかせする</x:v>
       </x:c>
       <x:c r="E29" s="40" t="n">
         <x:v>1</x:v>
@@ -3017,7 +3077,7 @@
         <x:v>HP→親に贈る→子が購入</x:v>
       </x:c>
       <x:c r="G29" s="40" t="str">
-        <x:v>無料体験をせずに購入し、本人接続か、ご家族のおまかせかを選べます。</x:v>
+        <x:v>無料体験をせずに購入し、本人が進めるか、家族・信頼する方におまかせするか選べます。</x:v>
       </x:c>
       <x:c r="H29" s="40" t="str">
         <x:v>子</x:v>
@@ -3062,10 +3122,10 @@
         <x:v>購入条件・45日保証・進め方</x:v>
       </x:c>
       <x:c r="V29" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W29" s="40" t="str">
-        <x:v>設定候補</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X29" s="40" t="str">
         <x:v>購入だけで本編開始しない</x:v>
@@ -3085,7 +3145,7 @@
         <x:v>3問なし・子購入・おまかせ</x:v>
       </x:c>
       <x:c r="D30" s="40" t="str">
-        <x:v>家族におまかせする</x:v>
+        <x:v>サポーターにおまかせする</x:v>
       </x:c>
       <x:c r="E30" s="40" t="n">
         <x:v>2</x:v>
@@ -3094,7 +3154,7 @@
         <x:v>子が本人の了承を確認し、おまかせで進める</x:v>
       </x:c>
       <x:c r="G30" s="40" t="str">
-        <x:v>ご本人の意向を確認し、ご家族が制作を引き受けます。本人のAccountは必要ありません。</x:v>
+        <x:v>ご本人の意向を確認し、信頼するサポーターが制作を引き受けます。本人のAccountは必要ありません。</x:v>
       </x:c>
       <x:c r="H30" s="40" t="str">
         <x:v>子</x:v>
@@ -3136,16 +3196,16 @@
         <x:v>不要</x:v>
       </x:c>
       <x:c r="U30" s="40" t="str">
-        <x:v>進め方・おまかせ確認・制作権限</x:v>
+        <x:v>進め方・おまかせ確認・Supporter制作アクセス</x:v>
       </x:c>
       <x:c r="V30" s="40" t="str">
-        <x:v>語りを見る権限のあるSupporterと共有</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W30" s="40" t="str">
-        <x:v>進捗を見る権限に従う</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X30" s="40" t="str">
-        <x:v>primary_mode＝家族中心。制作権限は個別Permission</x:v>
+        <x:v>primary_mode＝supporter。Supporterは制作内部へ原則フルアクセス</x:v>
       </x:c>
       <x:c r="Y30" s="40" t="str">
         <x:v>確定</x:v>
@@ -3162,7 +3222,7 @@
         <x:v>3問なし・子購入・おまかせ</x:v>
       </x:c>
       <x:c r="D31" s="40" t="str">
-        <x:v>家族におまかせする</x:v>
+        <x:v>サポーターにおまかせする</x:v>
       </x:c>
       <x:c r="E31" s="40" t="n">
         <x:v>3</x:v>
@@ -3216,10 +3276,10 @@
         <x:v>本編開始確認</x:v>
       </x:c>
       <x:c r="V31" s="40" t="str">
-        <x:v>制作Supporterと共有</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W31" s="40" t="str">
-        <x:v>共有</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X31" s="40" t="str">
         <x:v>actor＝子、subject＝親として開始を記録</x:v>
@@ -3239,7 +3299,7 @@
         <x:v>3問なし・子購入・おまかせ</x:v>
       </x:c>
       <x:c r="D32" s="40" t="str">
-        <x:v>家族におまかせする</x:v>
+        <x:v>サポーターにおまかせする</x:v>
       </x:c>
       <x:c r="E32" s="40" t="n">
         <x:v>4</x:v>
@@ -3293,10 +3353,10 @@
         <x:v>共有・収録・Web・QR・最終確定</x:v>
       </x:c>
       <x:c r="V32" s="40" t="str">
-        <x:v>制作Supporterと共有（変更可）</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W32" s="40" t="str">
-        <x:v>共有</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X32" s="40" t="str">
         <x:v>本人Accountは後から任意で接続可能</x:v>
@@ -3370,10 +3430,10 @@
         <x:v>本人接続・進捗共有</x:v>
       </x:c>
       <x:c r="V33" s="40" t="str">
-        <x:v>本人権限</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W33" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X33" s="40" t="str">
         <x:v>同じPerson・Projectへ接続</x:v>
@@ -3447,10 +3507,10 @@
         <x:v>本編開始確認</x:v>
       </x:c>
       <x:c r="V34" s="40" t="str">
-        <x:v>語りごと</x:v>
+        <x:v>Supporterは制作素材を閲覧。家族・Viewerは共有指定のみ</x:v>
       </x:c>
       <x:c r="W34" s="40" t="str">
-        <x:v>設定通り</x:v>
+        <x:v>Supporterは全進捗を確認</x:v>
       </x:c>
       <x:c r="X34" s="40" t="str">
         <x:v>娘はSupporterのまま</x:v>
@@ -3486,6 +3546,9 @@
       <x:formula>$Y5="要確認"</x:formula>
     </x:cfRule>
     <x:cfRule type="expression" dxfId="18" priority="7">
+      <x:formula>$Y5="要確認"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="21" priority="8">
       <x:formula>$Y5="要確認"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -3566,40 +3629,40 @@
       <x:c r="L3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="86" t="str">
+      <x:c r="A4" s="94" t="str">
         <x:v>Setting ID</x:v>
       </x:c>
-      <x:c r="B4" s="86" t="str">
+      <x:c r="B4" s="94" t="str">
         <x:v>設定・同意</x:v>
       </x:c>
-      <x:c r="C4" s="86" t="str">
+      <x:c r="C4" s="94" t="str">
         <x:v>Account登録</x:v>
       </x:c>
-      <x:c r="D4" s="86" t="str">
+      <x:c r="D4" s="94" t="str">
         <x:v>対象Person作成</x:v>
       </x:c>
-      <x:c r="E4" s="86" t="str">
+      <x:c r="E4" s="94" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="F4" s="86" t="str">
+      <x:c r="F4" s="94" t="str">
         <x:v>購入</x:v>
       </x:c>
-      <x:c r="G4" s="86" t="str">
+      <x:c r="G4" s="94" t="str">
         <x:v>本人接続</x:v>
       </x:c>
-      <x:c r="H4" s="86" t="str">
+      <x:c r="H4" s="94" t="str">
         <x:v>本編開始</x:v>
       </x:c>
-      <x:c r="I4" s="86" t="str">
+      <x:c r="I4" s="94" t="str">
         <x:v>制作中</x:v>
       </x:c>
-      <x:c r="J4" s="86" t="str">
+      <x:c r="J4" s="94" t="str">
         <x:v>仕上げ</x:v>
       </x:c>
-      <x:c r="K4" s="86" t="str">
+      <x:c r="K4" s="94" t="str">
         <x:v>完成後</x:v>
       </x:c>
-      <x:c r="L4" s="86" t="str">
+      <x:c r="L4" s="94" t="str">
         <x:v>備考</x:v>
       </x:c>
     </x:row>
@@ -3722,7 +3785,7 @@
         <x:v>S04</x:v>
       </x:c>
       <x:c r="B8" s="40" t="str">
-        <x:v>進捗共有</x:v>
+        <x:v>Supporter制作アクセス</x:v>
       </x:c>
       <x:c r="C8" s="40" t="str">
         <x:v>—</x:v>
@@ -3734,13 +3797,13 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="F8" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>△</x:v>
       </x:c>
       <x:c r="G8" s="40" t="str">
         <x:v>●</x:v>
       </x:c>
       <x:c r="H8" s="40" t="str">
-        <x:v>—</x:v>
+        <x:v>△</x:v>
       </x:c>
       <x:c r="I8" s="40" t="str">
         <x:v>△</x:v>
@@ -3752,7 +3815,7 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="L8" s="40" t="str">
-        <x:v>進捗を見るPermissionのあるSupporterへ共有。進め方とは独立</x:v>
+        <x:v>明示的に参加したSupporterは、制作のため全語り・進捗・素材へアクセス</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="44" customHeight="1">
@@ -3760,7 +3823,7 @@
         <x:v>S05</x:v>
       </x:c>
       <x:c r="B9" s="40" t="str">
-        <x:v>語り共有 本人のみ／制作Supporter</x:v>
+        <x:v>家族共有 共有する／共有しない</x:v>
       </x:c>
       <x:c r="C9" s="40" t="str">
         <x:v>—</x:v>
@@ -3790,7 +3853,7 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="L9" s="40" t="str">
-        <x:v>語りを見るPermissionのあるSupporterへ共有。語り単位で変更可</x:v>
+        <x:v>初期値は共有しない。Supporterの制作アクセスとは別</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="44" customHeight="1">
@@ -3942,7 +4005,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="L13" s="40" t="str">
-        <x:v>本人、または意向を確認した家族中心のSupporterが明示操作</x:v>
+        <x:v>本人、または本人の意向を確認したSupporterが明示操作</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="44" customHeight="1">
@@ -3988,7 +4051,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="B15" s="40" t="str">
-        <x:v>進め方・家族中心の了承確認</x:v>
+        <x:v>進め方・Supporter中心の了承確認</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
         <x:v>—</x:v>
@@ -4018,7 +4081,7 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="L15" s="40" t="str">
-        <x:v>本人が進める／家族におまかせする。途中変更可</x:v>
+        <x:v>本人が進める／サポーターにおまかせする。UI候補は『家族・信頼する方におまかせする』</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="44" customHeight="1">
@@ -4026,7 +4089,7 @@
         <x:v>S12</x:v>
       </x:c>
       <x:c r="B16" s="40" t="str">
-        <x:v>Supporter権限</x:v>
+        <x:v>Supporter種別</x:v>
       </x:c>
       <x:c r="C16" s="40" t="str">
         <x:v>—</x:v>
@@ -4056,7 +4119,7 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="L16" s="40" t="str">
-        <x:v>進め方の初期プリセット後もPermissionを個別変更可</x:v>
+        <x:v>personal／professional。professionalは将来の施設・有料制作支援向け</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="44" customHeight="1">
@@ -4159,31 +4222,31 @@
       <x:c r="I3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="86" t="str">
+      <x:c r="A4" s="94" t="str">
         <x:v>Case</x:v>
       </x:c>
-      <x:c r="B4" s="86" t="str">
+      <x:c r="B4" s="94" t="str">
         <x:v>位置づけ</x:v>
       </x:c>
-      <x:c r="C4" s="86" t="str">
+      <x:c r="C4" s="94" t="str">
         <x:v>HPに来た人</x:v>
       </x:c>
-      <x:c r="D4" s="86" t="str">
+      <x:c r="D4" s="94" t="str">
         <x:v>語る人</x:v>
       </x:c>
-      <x:c r="E4" s="86" t="str">
+      <x:c r="E4" s="94" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="F4" s="86" t="str">
+      <x:c r="F4" s="94" t="str">
         <x:v>同席・遠隔</x:v>
       </x:c>
-      <x:c r="G4" s="86" t="str">
+      <x:c r="G4" s="94" t="str">
         <x:v>購入者候補</x:v>
       </x:c>
-      <x:c r="H4" s="86" t="str">
+      <x:c r="H4" s="94" t="str">
         <x:v>本人Accountが必要になる時</x:v>
       </x:c>
-      <x:c r="I4" s="86" t="str">
+      <x:c r="I4" s="94" t="str">
         <x:v>要点</x:v>
       </x:c>
     </x:row>
@@ -4221,10 +4284,10 @@
         <x:v>B 大切な人に語ってもらう</x:v>
       </x:c>
       <x:c r="B6" s="40" t="str">
-        <x:v>家族起点</x:v>
+        <x:v>家族・信頼する方起点</x:v>
       </x:c>
       <x:c r="C6" s="40" t="str">
-        <x:v>子・家族</x:v>
+        <x:v>家族・友人等</x:v>
       </x:c>
       <x:c r="D6" s="40" t="str">
         <x:v>親等</x:v>
@@ -4236,13 +4299,13 @@
         <x:v>同席／遠隔</x:v>
       </x:c>
       <x:c r="G6" s="40" t="str">
-        <x:v>子または本人。別Subcaseで管理。</x:v>
+        <x:v>Supporterまたは本人。別Subcaseで管理。</x:v>
       </x:c>
       <x:c r="H6" s="40" t="str">
-        <x:v>本人中心では必要。家族中心では任意で後から接続可。</x:v>
+        <x:v>本人中心では必要。Supporter中心では任意で後から接続可。</x:v>
       </x:c>
       <x:c r="I6" s="40" t="str">
-        <x:v>2つの進め方と個別Permissionを分けて管理</x:v>
+        <x:v>Supporterは家族に限定せず、制作内部へ原則フルアクセス</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
@@ -4324,22 +4387,22 @@
       <x:c r="F3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="86" t="str">
+      <x:c r="A4" s="94" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B4" s="86" t="str">
+      <x:c r="B4" s="94" t="str">
         <x:v>論点</x:v>
       </x:c>
-      <x:c r="C4" s="86" t="str">
+      <x:c r="C4" s="94" t="str">
         <x:v>現状案</x:v>
       </x:c>
-      <x:c r="D4" s="86" t="str">
+      <x:c r="D4" s="94" t="str">
         <x:v>状態</x:v>
       </x:c>
-      <x:c r="E4" s="86" t="str">
+      <x:c r="E4" s="94" t="str">
         <x:v>決める理由</x:v>
       </x:c>
-      <x:c r="F4" s="86" t="str">
+      <x:c r="F4" s="94" t="str">
         <x:v>次アクション</x:v>
       </x:c>
     </x:row>
@@ -4351,16 +4414,16 @@
         <x:v>無料3問の語り共有初期値</x:v>
       </x:c>
       <x:c r="C5" s="40" t="str">
-        <x:v>本人のみを基準。語りを見るPermissionのある制作Supporterには共有し、語り単位で変更可</x:v>
+        <x:v>Supporterには制作目的で全語り・素材を共有。家族・Viewerには共有指定した内容だけ</x:v>
       </x:c>
       <x:c r="D5" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
       <x:c r="E5" s="40" t="str">
-        <x:v>進め方と閲覧Permissionを混同せず、本人の選択余地を残す</x:v>
+        <x:v>制作支援と家族閲覧を混同せず、現実的な共同制作を成立させる</x:v>
       </x:c>
       <x:c r="F5" s="40" t="str">
-        <x:v>Supporter権限の実装へ反映</x:v>
+        <x:v>Supporterロールと家族共有へ反映</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
@@ -4371,16 +4434,16 @@
         <x:v>親支援時の進捗共有初期値</x:v>
       </x:c>
       <x:c r="C6" s="40" t="str">
-        <x:v>進捗を見るPermissionのあるSupporterへ共有</x:v>
+        <x:v>Supporterは全進捗を確認可能</x:v>
       </x:c>
       <x:c r="D6" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
       <x:c r="E6" s="40" t="str">
-        <x:v>本人中心でも必要に応じて家族が見守れる</x:v>
+        <x:v>制作を担う人が遠隔でも状況を把握できるようにする</x:v>
       </x:c>
       <x:c r="F6" s="40" t="str">
-        <x:v>Supporter権限の実装へ反映</x:v>
+        <x:v>Supporterロールへ反映</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -4531,13 +4594,13 @@
         <x:v>2つの進め方と代理操作</x:v>
       </x:c>
       <x:c r="C14" s="40" t="str">
-        <x:v>本人が進める／家族におまかせする。家族中心では本人Accountを任意とし、広い制作権限を初期付与</x:v>
+        <x:v>本人が進める／サポーターにおまかせする。権限差ではなく主なAccount・端末の違い</x:v>
       </x:c>
       <x:c r="D14" s="40" t="str">
         <x:v>確定</x:v>
       </x:c>
       <x:c r="E14" s="40" t="str">
-        <x:v>主な操作主体と個別Permissionを分け、高齢者にも自立利用者にも対応</x:v>
+        <x:v>本人主体でもSupporterは制作内部へ原則フルアクセスできる</x:v>
       </x:c>
       <x:c r="F14" s="40" t="str">
         <x:v>06_支援スタイル・権限とBフローへ反映</x:v>
@@ -4548,10 +4611,10 @@
         <x:v>Q11</x:v>
       </x:c>
       <x:c r="B15" s="40" t="str">
-        <x:v>進め方・本人了承・Permissionの保存先</x:v>
+        <x:v>進め方・本人了承・Supporter関係の保存先</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
-        <x:v>primary_mode、supporter_permissions、confirmed_by、confirmed_at等を分離して記録する案</x:v>
+        <x:v>primary_mode、supporter_type、confirmed_by、confirmed_at等を分離して記録する案</x:v>
       </x:c>
       <x:c r="D15" s="40" t="str">
         <x:v>要確認</x:v>
@@ -4571,7 +4634,7 @@
         <x:v>通知先の初期値・保存先</x:v>
       </x:c>
       <x:c r="C16" s="40" t="str">
-        <x:v>本人Account有無とPermissionに応じ、本人／Supporter／双方を将来設定可能にする</x:v>
+        <x:v>本人Account有無に応じ、本人／Supporter／双方を将来設定可能にする</x:v>
       </x:c>
       <x:c r="D16" s="40" t="str">
         <x:v>要確認</x:v>
@@ -4581,6 +4644,26 @@
       </x:c>
       <x:c r="F16" s="40" t="str">
         <x:v>既存通知実装と設定保存先を照合</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="54" customHeight="1">
+      <x:c r="A17" s="40" t="str">
+        <x:v>Q13</x:v>
+      </x:c>
+      <x:c r="B17" s="40" t="str">
+        <x:v>professional Supporterの業務管理</x:v>
+      </x:c>
+      <x:c r="C17" s="40" t="str">
+        <x:v>担当期間、操作・閲覧ログ、担当終了時のアクセス停止を管理する</x:v>
+      </x:c>
+      <x:c r="D17" s="40" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
+      <x:c r="E17" s="40" t="str">
+        <x:v>施設スタッフや当社スタッフが扱う場合のプライバシーと運営責任を明確にする</x:v>
+      </x:c>
+      <x:c r="F17" s="40" t="str">
+        <x:v>有料制作支援の実装前にDB・管理画面・監査要件を確定</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4615,7 +4698,12 @@
       <x:formula>$D5="要確認"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="3">
+  <x:conditionalFormatting sqref="A5:F17">
+    <x:cfRule type="expression" dxfId="22" priority="8">
+      <x:formula>$D5="要確認"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="D5:D13">
       <x:formula1>"確定,要確認"</x:formula1>
     </x:dataValidation>
@@ -4623,6 +4711,9 @@
       <x:formula1>"確定,要確認"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D5:D16">
+      <x:formula1>"確定,要確認"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D5:D17">
       <x:formula1>"確定,要確認"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -4687,34 +4778,34 @@
       <x:c r="J3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="86" t="str">
+      <x:c r="A4" s="94" t="str">
         <x:v>Setting ID</x:v>
       </x:c>
-      <x:c r="B4" s="86" t="str">
+      <x:c r="B4" s="94" t="str">
         <x:v>設定・同意名</x:v>
       </x:c>
-      <x:c r="C4" s="86" t="str">
+      <x:c r="C4" s="94" t="str">
         <x:v>利用者が設定する画面</x:v>
       </x:c>
-      <x:c r="D4" s="86" t="str">
+      <x:c r="D4" s="94" t="str">
         <x:v>初期値</x:v>
       </x:c>
-      <x:c r="E4" s="86" t="str">
+      <x:c r="E4" s="94" t="str">
         <x:v>設定できる人</x:v>
       </x:c>
-      <x:c r="F4" s="86" t="str">
+      <x:c r="F4" s="94" t="str">
         <x:v>変更できる時期</x:v>
       </x:c>
-      <x:c r="G4" s="86" t="str">
+      <x:c r="G4" s="94" t="str">
         <x:v>保存先</x:v>
       </x:c>
-      <x:c r="H4" s="86" t="str">
+      <x:c r="H4" s="94" t="str">
         <x:v>関連Flow ID</x:v>
       </x:c>
-      <x:c r="I4" s="86" t="str">
+      <x:c r="I4" s="94" t="str">
         <x:v>実装状態</x:v>
       </x:c>
-      <x:c r="J4" s="86" t="str">
+      <x:c r="J4" s="94" t="str">
         <x:v>根拠仕様</x:v>
       </x:c>
     </x:row>
@@ -4790,19 +4881,19 @@
         <x:v>Supporter参加</x:v>
       </x:c>
       <x:c r="C7" s="40" t="str">
-        <x:v>大切な人の物語の開始／家族とのつながり</x:v>
+        <x:v>大切な人の物語の開始／Supporter招待</x:v>
       </x:c>
       <x:c r="D7" s="40" t="str">
         <x:v>未参加</x:v>
       </x:c>
       <x:c r="E7" s="40" t="str">
-        <x:v>本人と支援を開始するAccount</x:v>
+        <x:v>本人、または本人の了承を確認した開始Account</x:v>
       </x:c>
       <x:c r="F7" s="40" t="str">
         <x:v>開始時・本人接続後・停止時</x:v>
       </x:c>
       <x:c r="G7" s="40" t="str">
-        <x:v>project_supporters／family_subject_bindings.initiated_by</x:v>
+        <x:v>project_supporters／family_subject_bindings.initiated_by。supporter_typeは要確認</x:v>
       </x:c>
       <x:c r="H7" s="40" t="str">
         <x:v>B-CO-020、B-REMOTE-020、B-DIRECT-GIFT-010</x:v>
@@ -4819,22 +4910,22 @@
         <x:v>S04</x:v>
       </x:c>
       <x:c r="B8" s="40" t="str">
-        <x:v>進捗共有</x:v>
+        <x:v>Supporter制作アクセス</x:v>
       </x:c>
       <x:c r="C8" s="40" t="str">
-        <x:v>Supporter権限／家族とのつながり設定</x:v>
+        <x:v>Supporter参加の説明・確認</x:v>
       </x:c>
       <x:c r="D8" s="40" t="str">
-        <x:v>進捗を見るPermissionがある場合のみ共有</x:v>
+        <x:v>参加したSupporterは制作内部へ原則フルアクセス</x:v>
       </x:c>
       <x:c r="E8" s="40" t="str">
-        <x:v>本人または本人の了承を確認したSupporter</x:v>
+        <x:v>本人、または本人の了承を確認したSupporter</x:v>
       </x:c>
       <x:c r="F8" s="40" t="str">
-        <x:v>初回設定・本人接続後・随時</x:v>
+        <x:v>Supporter参加時・停止時</x:v>
       </x:c>
       <x:c r="G8" s="40" t="str">
-        <x:v>family_subject_bindings.progress_enabled</x:v>
+        <x:v>project_supporters／family_subject_bindings／RLS。全制作範囲の正は要確認</x:v>
       </x:c>
       <x:c r="H8" s="40" t="str">
         <x:v>B-CO-020、B-CO-030、B-REMOTE-020、B-CO-DELEGATED-050</x:v>
@@ -4843,7 +4934,7 @@
         <x:v>一部実装</x:v>
       </x:c>
       <x:c r="J8" s="40" t="str">
-        <x:v>docs/family-assisted-early-release-spec-20260917.md §5／202609170002_family_subject_connection.sql</x:v>
+        <x:v>06_支援スタイル・権限／202609170002_family_subject_connection.sql</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="74" customHeight="1">
@@ -4851,16 +4942,16 @@
         <x:v>S05</x:v>
       </x:c>
       <x:c r="B9" s="40" t="str">
-        <x:v>語り共有 本人のみ／制作Supporter</x:v>
+        <x:v>家族共有 共有する／共有しない</x:v>
       </x:c>
       <x:c r="C9" s="40" t="str">
-        <x:v>録音保存時／Supporter権限／語り設定</x:v>
+        <x:v>録音保存時／語り設定</x:v>
       </x:c>
       <x:c r="D9" s="40" t="str">
-        <x:v>本人のみ。語りを見るPermissionがある場合は制作Supporterにも共有</x:v>
+        <x:v>共有しない。制作Supporterには常に表示</x:v>
       </x:c>
       <x:c r="E9" s="40" t="str">
-        <x:v>本人または本人の了承を確認したSupporter。語り単位で変更可。</x:v>
+        <x:v>本人または本人の了承を確認したSupporter</x:v>
       </x:c>
       <x:c r="F9" s="40" t="str">
         <x:v>語り保存時・後から随時</x:v>
@@ -4889,10 +4980,10 @@
         <x:v>仕上げ／掲載する語りの選択</x:v>
       </x:c>
       <x:c r="D10" s="40" t="str">
-        <x:v>収録設定Permissionがある人に候補表示</x:v>
+        <x:v>制作対象を候補表示</x:v>
       </x:c>
       <x:c r="E10" s="40" t="str">
-        <x:v>本人または収録設定PermissionのあるSupporter</x:v>
+        <x:v>本人またはSupporter</x:v>
       </x:c>
       <x:c r="F10" s="40" t="str">
         <x:v>制作中・仕上げ・最終確定前</x:v>
@@ -4924,7 +5015,7 @@
         <x:v>非共有</x:v>
       </x:c>
       <x:c r="E11" s="40" t="str">
-        <x:v>本人または共有設定PermissionのあるSupporter</x:v>
+        <x:v>本人またはSupporter</x:v>
       </x:c>
       <x:c r="F11" s="40" t="str">
         <x:v>仕上げ時・完成後</x:v>
@@ -4956,7 +5047,7 @@
         <x:v>掲載しない・非公開を基準</x:v>
       </x:c>
       <x:c r="E12" s="40" t="str">
-        <x:v>本人または共有設定PermissionのあるSupporter</x:v>
+        <x:v>本人またはSupporter</x:v>
       </x:c>
       <x:c r="F12" s="40" t="str">
         <x:v>仕上げ時・完成後の閲覧方法変更</x:v>
@@ -4988,7 +5079,7 @@
         <x:v>未開始</x:v>
       </x:c>
       <x:c r="E13" s="40" t="str">
-        <x:v>Person本人Accountまたは家族中心で開始権限のあるSupporter</x:v>
+        <x:v>Person本人Accountまたは本人の意向を確認したSupporter</x:v>
       </x:c>
       <x:c r="F13" s="40" t="str">
         <x:v>一度だけ。開始後は戻さない。</x:v>
@@ -5043,7 +5134,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="B15" s="40" t="str">
-        <x:v>進め方・家族中心の了承確認</x:v>
+        <x:v>進め方・Supporter中心の了承確認</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
         <x:v>対象Person作成／本格利用開始</x:v>
@@ -5052,7 +5143,7 @@
         <x:v>未選択</x:v>
       </x:c>
       <x:c r="E15" s="40" t="str">
-        <x:v>本人またはSupporter。家族中心では語り手本人の了承を確認。</x:v>
+        <x:v>本人またはSupporter。Supporter中心では語り手本人の了承を確認。</x:v>
       </x:c>
       <x:c r="F15" s="40" t="str">
         <x:v>開始時・購入時・本人接続時・随時</x:v>
@@ -5075,22 +5166,22 @@
         <x:v>S12</x:v>
       </x:c>
       <x:c r="B16" s="40" t="str">
-        <x:v>Supporter権限</x:v>
+        <x:v>Supporter種別</x:v>
       </x:c>
       <x:c r="C16" s="40" t="str">
-        <x:v>Supporter追加／お手伝い範囲の設定</x:v>
+        <x:v>Supporter追加／運営管理</x:v>
       </x:c>
       <x:c r="D16" s="40" t="str">
-        <x:v>本人中心＝必要な範囲。家族中心＝広い制作権限プリセット</x:v>
+        <x:v>personal。professionalは将来拡張</x:v>
       </x:c>
       <x:c r="E16" s="40" t="str">
-        <x:v>本人または本人の了承を確認したSupporter</x:v>
+        <x:v>本人、本人の了承を確認したSupporter、professionalは運営</x:v>
       </x:c>
       <x:c r="F16" s="40" t="str">
-        <x:v>Supporter追加時・開始後随時</x:v>
+        <x:v>Supporter追加時・業務担当変更時</x:v>
       </x:c>
       <x:c r="G16" s="40" t="str">
-        <x:v>要確認（project_supporter_permissions等）</x:v>
+        <x:v>要確認（supporter_type、assignment期間等）</x:v>
       </x:c>
       <x:c r="H16" s="40" t="str">
         <x:v>B-CO-020、B-CO-DELEGATED-050、B-DIRECT-DELEGATED-020、B-CO-GIFT-050</x:v>
@@ -5099,7 +5190,7 @@
         <x:v>未実装</x:v>
       </x:c>
       <x:c r="J16" s="40" t="str">
-        <x:v>06_支援スタイル・権限／04_運営チェック Q11</x:v>
+        <x:v>06_支援スタイル・権限／04_運営チェック Q11・Q13</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="74" customHeight="1">
@@ -5113,10 +5204,10 @@
         <x:v>現時点では既存通知ロジック。将来は通知設定</x:v>
       </x:c>
       <x:c r="D17" s="40" t="str">
-        <x:v>本人Account有無とPermissionに応じた既定</x:v>
+        <x:v>本人Account有無に応じた既定</x:v>
       </x:c>
       <x:c r="E17" s="40" t="str">
-        <x:v>本人または通知管理PermissionのあるSupporter</x:v>
+        <x:v>本人またはSupporter</x:v>
       </x:c>
       <x:c r="F17" s="40" t="str">
         <x:v>本人接続時・Supporter変更時・随時</x:v>
@@ -5132,6 +5223,38 @@
       </x:c>
       <x:c r="J17" s="40" t="str">
         <x:v>06_支援スタイル・権限／04_運営チェック Q12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="74" customHeight="1">
+      <x:c r="A18" s="40" t="str">
+        <x:v>S14</x:v>
+      </x:c>
+      <x:c r="B18" s="40" t="str">
+        <x:v>業務Supporterアクセス管理</x:v>
+      </x:c>
+      <x:c r="C18" s="40" t="str">
+        <x:v>運営管理画面（将来）</x:v>
+      </x:c>
+      <x:c r="D18" s="40" t="str">
+        <x:v>アクセスなし</x:v>
+      </x:c>
+      <x:c r="E18" s="40" t="str">
+        <x:v>権限ある運営者</x:v>
+      </x:c>
+      <x:c r="F18" s="40" t="str">
+        <x:v>担当開始・変更・終了時</x:v>
+      </x:c>
+      <x:c r="G18" s="40" t="str">
+        <x:v>要確認（assignment期間、アクセスログ、失効）</x:v>
+      </x:c>
+      <x:c r="H18" s="40" t="str">
+        <x:v>将来の施設・制作支援ケース</x:v>
+      </x:c>
+      <x:c r="I18" s="40" t="str">
+        <x:v>未実装</x:v>
+      </x:c>
+      <x:c r="J18" s="40" t="str">
+        <x:v>04_運営チェック Q13／06_支援スタイル・権限</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5166,7 +5289,12 @@
       <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="3">
+  <x:conditionalFormatting sqref="A5:J18">
+    <x:cfRule type="expression" dxfId="23" priority="8">
+      <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="I5:I14">
       <x:formula1>"実装済み,一部実装,未実装,要確認"</x:formula1>
     </x:dataValidation>
@@ -5174,6 +5302,9 @@
       <x:formula1>"実装済み,一部実装,未実装,要確認"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I5:I17">
+      <x:formula1>"実装済み,一部実装,未実装,要確認"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I5:I18">
       <x:formula1>"実装済み,一部実装,未実装,要確認"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -5185,16 +5316,16 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="64" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="39" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="49" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="43" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="60" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="28" t="str">
-        <x:v>進め方とSupporter権限</x:v>
+        <x:v>進め方とSupporter</x:v>
       </x:c>
       <x:c r="B1" s="28"/>
       <x:c r="C1" s="28"/>
@@ -5203,7 +5334,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="30" t="str">
-        <x:v>進め方は主な操作主体だけを決める。Supporter権限、本人Account、通知先は独立して設定し、開始後も変更できる。</x:v>
+        <x:v>Supporterは、本人が信頼して物語づくりを任せる制作メンバー。家族・Viewerへの共有とは別に、制作内部へ原則フルアクセスする。</x:v>
       </x:c>
       <x:c r="B2" s="30"/>
       <x:c r="C2" s="30"/>
@@ -5218,23 +5349,23 @@
       <x:c r="E3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="86" t="str">
-        <x:v>進め方</x:v>
-      </x:c>
-      <x:c r="B4" s="86" t="str">
+      <x:c r="A4" s="94" t="str">
+        <x:v>進め方（内部名）</x:v>
+      </x:c>
+      <x:c r="B4" s="94" t="str">
         <x:v>中心となる端末・Account</x:v>
       </x:c>
-      <x:c r="C4" s="86" t="str">
-        <x:v>Supporterの初期状態</x:v>
-      </x:c>
-      <x:c r="D4" s="86" t="str">
+      <x:c r="C4" s="94" t="str">
+        <x:v>Supporter</x:v>
+      </x:c>
+      <x:c r="D4" s="94" t="str">
         <x:v>本人Account</x:v>
       </x:c>
-      <x:c r="E4" s="86" t="str">
-        <x:v>ユーザー向け説明候補</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="48" customHeight="1">
+      <x:c r="E4" s="94" t="str">
+        <x:v>ユーザー向け表現・説明候補</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="54" customHeight="1">
       <x:c r="A5" s="66" t="str">
         <x:v>本人が進める</x:v>
       </x:c>
@@ -5242,33 +5373,33 @@
         <x:v>本人のスマホ／本人Account</x:v>
       </x:c>
       <x:c r="C5" s="40" t="str">
-        <x:v>なし、または必要な範囲を選択</x:v>
+        <x:v>任意。追加した場合は制作内部へフルアクセス</x:v>
       </x:c>
       <x:c r="D5" s="40" t="str">
         <x:v>必須</x:v>
       </x:c>
       <x:c r="E5" s="40" t="str">
-        <x:v>本人のスマホを中心に進めます。ご家族にも、必要な範囲でお手伝いしてもらえます。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="48" customHeight="1">
+        <x:v>本人が進める｜本人のスマホを中心に進めます。必要に応じて、家族や信頼する方にもお手伝いしてもらえます。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="54" customHeight="1">
       <x:c r="A6" s="66" t="str">
-        <x:v>家族におまかせする</x:v>
+        <x:v>サポーターにおまかせする</x:v>
       </x:c>
       <x:c r="B6" s="40" t="str">
-        <x:v>家族の端末／Supporter Account</x:v>
+        <x:v>Supporterの端末／Account</x:v>
       </x:c>
       <x:c r="C6" s="40" t="str">
-        <x:v>制作に必要な権限を広く付与</x:v>
+        <x:v>必須。制作内部へフルアクセス</x:v>
       </x:c>
       <x:c r="D6" s="40" t="str">
         <x:v>任意・後から接続可</x:v>
       </x:c>
       <x:c r="E6" s="40" t="str">
-        <x:v>家族の端末を中心に進めます。語りの収録から写真、本への仕上げまでおまかせできます。ご本人のスマホからも参加できます。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="48" customHeight="1">
+        <x:v>家族・信頼する方におまかせする｜信頼する方の端末を中心に進めます。語りの収録から写真、本への仕上げまでお手伝いしてもらえます。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="54" customHeight="1">
       <x:c r="A7" s="66" t="str">
         <x:v>変更</x:v>
       </x:c>
@@ -5276,266 +5407,236 @@
         <x:v>開始後も変更可</x:v>
       </x:c>
       <x:c r="C7" s="40" t="str">
-        <x:v>権限は個別に変更可</x:v>
+        <x:v>追加・停止可</x:v>
       </x:c>
       <x:c r="D7" s="40" t="str">
         <x:v>既存Personへ後付け</x:v>
       </x:c>
       <x:c r="E7" s="40" t="str">
-        <x:v>進め方やお手伝いの範囲は、あとからいつでも変更できます。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="48" customHeight="1">
+        <x:v>進め方はあとから変更できます。本人のスマホからも参加できます。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="54" customHeight="1">
       <x:c r="A8" s="41"/>
       <x:c r="B8" s="41"/>
       <x:c r="C8" s="41"/>
       <x:c r="D8" s="41"/>
       <x:c r="E8" s="41"/>
     </x:row>
-    <x:row r="9" ht="48" customHeight="1">
-      <x:c r="A9" s="86" t="str">
-        <x:v>Supporter権限</x:v>
-      </x:c>
-      <x:c r="B9" s="86" t="str">
-        <x:v>本人が進める 初期状態</x:v>
-      </x:c>
-      <x:c r="C9" s="86" t="str">
-        <x:v>家族におまかせ 初期状態</x:v>
-      </x:c>
-      <x:c r="D9" s="86" t="str">
-        <x:v>開始後の変更</x:v>
-      </x:c>
-      <x:c r="E9" s="86" t="str">
-        <x:v>権限の意味</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="48" customHeight="1">
+    <x:row r="9" ht="54" customHeight="1">
+      <x:c r="A9" s="94" t="str">
+        <x:v>関係</x:v>
+      </x:c>
+      <x:c r="B9" s="94" t="str">
+        <x:v>定義</x:v>
+      </x:c>
+      <x:c r="C9" s="94" t="str">
+        <x:v>アクセス範囲</x:v>
+      </x:c>
+      <x:c r="D9" s="94" t="str">
+        <x:v>主な役割</x:v>
+      </x:c>
+      <x:c r="E9" s="94" t="str">
+        <x:v>対象例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="54" customHeight="1">
       <x:c r="A10" s="66" t="str">
-        <x:v>進捗を見る</x:v>
-      </x:c>
-      <x:c r="B10" s="90" t="str">
-        <x:v>OFF／追加時に選択</x:v>
-      </x:c>
-      <x:c r="C10" s="90" t="str">
-        <x:v>ON</x:v>
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="B10" s="40" t="str">
+        <x:v>人生・作品の主人公であり、本人Accountから参加できる人</x:v>
+      </x:c>
+      <x:c r="C10" s="98" t="str">
+        <x:v>自分のPerson・Project</x:v>
       </x:c>
       <x:c r="D10" s="40" t="str">
-        <x:v>個別にON／OFF</x:v>
+        <x:v>語る、確認する、制作する</x:v>
       </x:c>
       <x:c r="E10" s="40" t="str">
-        <x:v>テーマや制作の進み具合を確認する</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="48" customHeight="1">
+        <x:v>語り手本人</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="54" customHeight="1">
       <x:c r="A11" s="66" t="str">
-        <x:v>語りを見る</x:v>
-      </x:c>
-      <x:c r="B11" s="90" t="str">
-        <x:v>OFF／追加時に選択</x:v>
-      </x:c>
-      <x:c r="C11" s="90" t="str">
-        <x:v>ON</x:v>
+        <x:v>Supporter</x:v>
+      </x:c>
+      <x:c r="B11" s="40" t="str">
+        <x:v>本人が信頼し、語り・作品づくりを手伝ってもらう制作メンバー</x:v>
+      </x:c>
+      <x:c r="C11" s="98" t="str">
+        <x:v>全語り、音声、写真、下書き、進捗、ブック制作など制作内部全体</x:v>
       </x:c>
       <x:c r="D11" s="40" t="str">
-        <x:v>個別にON／OFF</x:v>
+        <x:v>録音、写真、文章編集、収録・共有設定、仕上げ、注文</x:v>
       </x:c>
       <x:c r="E11" s="40" t="str">
-        <x:v>語りの内容を閲覧する。語り単位の非共有設定を優先</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="48" customHeight="1">
+        <x:v>家族、友人、仕事仲間、施設スタッフ、当社スタッフ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="54" customHeight="1">
       <x:c r="A12" s="66" t="str">
-        <x:v>録音・語りを追加する</x:v>
-      </x:c>
-      <x:c r="B12" s="90" t="str">
-        <x:v>OFF／追加時に選択</x:v>
-      </x:c>
-      <x:c r="C12" s="90" t="str">
-        <x:v>ON</x:v>
+        <x:v>Family / Viewer</x:v>
+      </x:c>
+      <x:c r="B12" s="40" t="str">
+        <x:v>本人またはSupporterが共有した内容を見る閲覧者</x:v>
+      </x:c>
+      <x:c r="C12" s="98" t="str">
+        <x:v>家族共有した語り、共有されたWebブック・完成作品のみ</x:v>
       </x:c>
       <x:c r="D12" s="40" t="str">
-        <x:v>個別にON／OFF</x:v>
+        <x:v>閲覧、受け取り</x:v>
       </x:c>
       <x:c r="E12" s="40" t="str">
-        <x:v>本人と同席して録音操作を行い、Personへ語りを追加する</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="48" customHeight="1">
+        <x:v>家族、親族、招待された閲覧者</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="54" customHeight="1">
       <x:c r="A13" s="66" t="str">
-        <x:v>写真を追加・整理する</x:v>
-      </x:c>
-      <x:c r="B13" s="90" t="str">
-        <x:v>OFF／追加時に選択</x:v>
-      </x:c>
-      <x:c r="C13" s="90" t="str">
-        <x:v>ON</x:v>
+        <x:v>Payer</x:v>
+      </x:c>
+      <x:c r="B13" s="40" t="str">
+        <x:v>料金を支払う人。制作・閲覧の権限とは独立</x:v>
+      </x:c>
+      <x:c r="C13" s="98" t="str">
+        <x:v>支払い・契約情報</x:v>
       </x:c>
       <x:c r="D13" s="40" t="str">
-        <x:v>個別にON／OFF</x:v>
+        <x:v>購入、領収情報の受け取り</x:v>
       </x:c>
       <x:c r="E13" s="40" t="str">
-        <x:v>写真の追加、並び替え、説明の編集を行う</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="48" customHeight="1">
-      <x:c r="A14" s="66" t="str">
-        <x:v>文章を編集する</x:v>
-      </x:c>
-      <x:c r="B14" s="90" t="str">
-        <x:v>OFF／追加時に選択</x:v>
-      </x:c>
-      <x:c r="C14" s="90" t="str">
-        <x:v>ON</x:v>
-      </x:c>
-      <x:c r="D14" s="40" t="str">
-        <x:v>個別にON／OFF</x:v>
-      </x:c>
-      <x:c r="E14" s="40" t="str">
-        <x:v>文章の修正や語り直しの反映を行う</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="48" customHeight="1">
-      <x:c r="A15" s="66" t="str">
-        <x:v>語りの共有範囲を設定する</x:v>
-      </x:c>
-      <x:c r="B15" s="90" t="str">
-        <x:v>OFF／追加時に選択</x:v>
-      </x:c>
-      <x:c r="C15" s="90" t="str">
-        <x:v>ON</x:v>
-      </x:c>
-      <x:c r="D15" s="40" t="str">
-        <x:v>個別にON／OFF</x:v>
-      </x:c>
-      <x:c r="E15" s="40" t="str">
-        <x:v>本人の意向を確認し、閲覧できる範囲を設定する</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="48" customHeight="1">
+        <x:v>本人、家族、法人等</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="54" customHeight="1">
+      <x:c r="A14" s="41"/>
+      <x:c r="B14" s="41"/>
+      <x:c r="C14" s="41"/>
+      <x:c r="D14" s="41"/>
+      <x:c r="E14" s="41"/>
+    </x:row>
+    <x:row r="15" ht="54" customHeight="1">
+      <x:c r="A15" s="94" t="str">
+        <x:v>Supporter種別</x:v>
+      </x:c>
+      <x:c r="B15" s="94" t="str">
+        <x:v>定義</x:v>
+      </x:c>
+      <x:c r="C15" s="94" t="str">
+        <x:v>アクセス</x:v>
+      </x:c>
+      <x:c r="D15" s="94" t="str">
+        <x:v>運営管理</x:v>
+      </x:c>
+      <x:c r="E15" s="94" t="str">
+        <x:v>対象例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="54" customHeight="1">
       <x:c r="A16" s="66" t="str">
-        <x:v>本への収録を設定する</x:v>
-      </x:c>
-      <x:c r="B16" s="90" t="str">
-        <x:v>OFF／追加時に選択</x:v>
-      </x:c>
-      <x:c r="C16" s="90" t="str">
-        <x:v>ON</x:v>
-      </x:c>
-      <x:c r="D16" s="40" t="str">
-        <x:v>個別にON／OFF</x:v>
+        <x:v>personal</x:v>
+      </x:c>
+      <x:c r="B16" s="40" t="str">
+        <x:v>本人が招待した個人Supporter</x:v>
+      </x:c>
+      <x:c r="C16" s="98" t="str">
+        <x:v>制作内部へフルアクセス</x:v>
+      </x:c>
+      <x:c r="D16" s="98" t="str">
+        <x:v>本人の了承、参加・停止を記録</x:v>
       </x:c>
       <x:c r="E16" s="40" t="str">
-        <x:v>本へ入れる語り・写真を選択する</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="48" customHeight="1">
+        <x:v>家族、友人、信頼する知人</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="54" customHeight="1">
       <x:c r="A17" s="66" t="str">
-        <x:v>ブックを編集する</x:v>
-      </x:c>
-      <x:c r="B17" s="90" t="str">
-        <x:v>OFF／追加時に選択</x:v>
-      </x:c>
-      <x:c r="C17" s="90" t="str">
-        <x:v>ON</x:v>
-      </x:c>
-      <x:c r="D17" s="40" t="str">
-        <x:v>個別にON／OFF</x:v>
+        <x:v>professional</x:v>
+      </x:c>
+      <x:c r="B17" s="40" t="str">
+        <x:v>業務として制作を支援するSupporter（将来拡張）</x:v>
+      </x:c>
+      <x:c r="C17" s="98" t="str">
+        <x:v>制作内部へフルアクセス</x:v>
+      </x:c>
+      <x:c r="D17" s="98" t="str">
+        <x:v>担当期間、操作・閲覧ログ、終了時のアクセス停止が必要</x:v>
       </x:c>
       <x:c r="E17" s="40" t="str">
-        <x:v>タイトル、文章、写真、並び順などを編集する</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="48" customHeight="1">
-      <x:c r="A18" s="66" t="str">
-        <x:v>仕上げる</x:v>
-      </x:c>
-      <x:c r="B18" s="90" t="str">
-        <x:v>OFF／追加時に選択</x:v>
-      </x:c>
-      <x:c r="C18" s="90" t="str">
-        <x:v>ON</x:v>
-      </x:c>
-      <x:c r="D18" s="40" t="str">
-        <x:v>個別にON／OFF</x:v>
-      </x:c>
-      <x:c r="E18" s="40" t="str">
-        <x:v>Webブック、QR、共有範囲、最終版を設定する</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="48" customHeight="1">
-      <x:c r="A19" s="66" t="str">
-        <x:v>製本・注文する</x:v>
-      </x:c>
-      <x:c r="B19" s="90" t="str">
-        <x:v>OFF／追加時に選択</x:v>
-      </x:c>
-      <x:c r="C19" s="90" t="str">
-        <x:v>ON</x:v>
-      </x:c>
-      <x:c r="D19" s="40" t="str">
-        <x:v>個別にON／OFF</x:v>
-      </x:c>
-      <x:c r="E19" s="40" t="str">
-        <x:v>製本注文、追加注文、増刷を行う</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="48" customHeight="1">
-      <x:c r="A20" s="41"/>
-      <x:c r="B20" s="41"/>
-      <x:c r="C20" s="41"/>
-      <x:c r="D20" s="41"/>
-      <x:c r="E20" s="41"/>
-    </x:row>
-    <x:row r="21" ht="48" customHeight="1">
-      <x:c r="A21" s="86" t="str">
+        <x:v>施設スタッフ、縦糸横糸スタッフ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="54" customHeight="1">
+      <x:c r="A18" s="41"/>
+      <x:c r="B18" s="41"/>
+      <x:c r="C18" s="41"/>
+      <x:c r="D18" s="41"/>
+      <x:c r="E18" s="41"/>
+    </x:row>
+    <x:row r="19" ht="54" customHeight="1">
+      <x:c r="A19" s="94" t="str">
         <x:v>独立して管理する項目</x:v>
       </x:c>
-      <x:c r="B21" s="86" t="str">
+      <x:c r="B19" s="94" t="str">
         <x:v>値・選択肢</x:v>
       </x:c>
-      <x:c r="C21" s="86" t="str">
+      <x:c r="C19" s="94" t="str">
         <x:v>進め方との関係</x:v>
       </x:c>
-      <x:c r="D21" s="86" t="str">
+      <x:c r="D19" s="94" t="str">
         <x:v>変更</x:v>
       </x:c>
-      <x:c r="E21" s="86" t="str">
+      <x:c r="E19" s="94" t="str">
         <x:v>補足</x:v>
       </x:c>
     </x:row>
+    <x:row r="20" ht="54" customHeight="1">
+      <x:c r="A20" s="66" t="str">
+        <x:v>本人Account</x:v>
+      </x:c>
+      <x:c r="B20" s="40" t="str">
+        <x:v>あり／なし</x:v>
+      </x:c>
+      <x:c r="C20" s="40" t="str">
+        <x:v>Supporter中心ではなしでも完結</x:v>
+      </x:c>
+      <x:c r="D20" s="40" t="str">
+        <x:v>後から追加可</x:v>
+      </x:c>
+      <x:c r="E20" s="40" t="str">
+        <x:v>接続時に既存Person・Projectを新規作成しない</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="54" customHeight="1">
+      <x:c r="A21" s="66" t="str">
+        <x:v>通知先</x:v>
+      </x:c>
+      <x:c r="B21" s="40" t="str">
+        <x:v>本人／Supporter／双方</x:v>
+      </x:c>
+      <x:c r="C21" s="40" t="str">
+        <x:v>進め方には固定しない</x:v>
+      </x:c>
+      <x:c r="D21" s="40" t="str">
+        <x:v>将来変更可</x:v>
+      </x:c>
+      <x:c r="E21" s="40" t="str">
+        <x:v>現時点ではUIを増やさず、将来設定可能な構造を前提とする</x:v>
+      </x:c>
+    </x:row>
     <x:row r="22" ht="48" customHeight="1">
-      <x:c r="A22" s="66" t="str">
-        <x:v>本人Account</x:v>
-      </x:c>
-      <x:c r="B22" s="40" t="str">
-        <x:v>あり／なし</x:v>
-      </x:c>
-      <x:c r="C22" s="40" t="str">
-        <x:v>家族中心ではなしでも完結</x:v>
-      </x:c>
-      <x:c r="D22" s="40" t="str">
-        <x:v>後から追加可</x:v>
-      </x:c>
-      <x:c r="E22" s="40" t="str">
-        <x:v>接続時に既存Person・Projectを新規作成しない</x:v>
-      </x:c>
+      <x:c r="A22"/>
+      <x:c r="B22"/>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+      <x:c r="E22"/>
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
-      <x:c r="A23" s="66" t="str">
-        <x:v>通知先</x:v>
-      </x:c>
-      <x:c r="B23" s="40" t="str">
-        <x:v>本人／Supporter／双方</x:v>
-      </x:c>
-      <x:c r="C23" s="40" t="str">
-        <x:v>進め方には固定しない</x:v>
-      </x:c>
-      <x:c r="D23" s="40" t="str">
-        <x:v>将来変更可</x:v>
-      </x:c>
-      <x:c r="E23" s="40" t="str">
-        <x:v>現時点ではUIを増やさず、将来設定可能な構造を前提とする</x:v>
-      </x:c>
+      <x:c r="A23"/>
+      <x:c r="B23"/>
+      <x:c r="C23"/>
+      <x:c r="D23"/>
+      <x:c r="E23"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
docs: add trial production support model
</commit_message>
<xml_diff>
--- a/docs/product/user-flow/user-flow-master.xlsx
+++ b/docs/product/user-flow/user-flow-master.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="R30f2e29ecc134bf8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_利用動線" sheetId="2" r:id="R86dfb88b1cce4af9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定同意" sheetId="3" r:id="Rf0116c1801ee473f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ケース一覧" sheetId="4" r:id="Rb01a26c3dc954996"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_運営チェック" sheetId="5" r:id="R2c0050a225a540b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_実装対応" sheetId="6" r:id="Rd53634f0194948e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_支援スタイル・権限" sheetId="7" r:id="R3545b792b82f4141"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使い方" sheetId="1" r:id="R8db73844b28e4710"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_利用動線" sheetId="2" r:id="R77e6eb0167f44f3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定同意" sheetId="3" r:id="Re762f938a3cd444e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ケース一覧" sheetId="4" r:id="R9452f4ad9f4d4bf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_運営チェック" sheetId="5" r:id="R27153271789949ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_実装対応" sheetId="6" r:id="R53bad281ed904874"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_支援スタイル・権限" sheetId="7" r:id="R4639201667bf433a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -89,7 +89,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="22">
+  <x:fills count="24">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -196,6 +196,16 @@
         <x:fgColor rgb="FFEEF4F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF315B5B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF4F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -218,7 +228,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="99">
+  <x:cellXfs count="107">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -446,11 +456,61 @@
     <x:xf numFmtId="0" fontId="7" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="23" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="24">
+  <x:dxfs count="27">
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:color rgb="FF8A5A00"/>
@@ -915,13 +975,13 @@
       <x:c r="C3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="94" t="str">
+      <x:c r="A4" s="102" t="str">
         <x:v>シート</x:v>
       </x:c>
-      <x:c r="B4" s="94" t="str">
+      <x:c r="B4" s="102" t="str">
         <x:v>役割</x:v>
       </x:c>
-      <x:c r="C4" s="94" t="str">
+      <x:c r="C4" s="102" t="str">
         <x:v>ポイント</x:v>
       </x:c>
     </x:row>
@@ -997,13 +1057,13 @@
       <x:c r="C11" s="41"/>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
-      <x:c r="A12" s="97" t="str">
+      <x:c r="A12" s="105" t="str">
         <x:v>更新ルール</x:v>
       </x:c>
-      <x:c r="B12" s="97" t="str">
+      <x:c r="B12" s="105" t="str">
         <x:v>同名ファイルを更新</x:v>
       </x:c>
-      <x:c r="C12" s="97" t="str">
+      <x:c r="C12" s="105" t="str">
         <x:v>別バージョンのExcelを増やさず、変更理由と履歴はGitで管理する。</x:v>
       </x:c>
     </x:row>
@@ -1133,79 +1193,79 @@
       <x:c r="Y3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="94" t="str">
+      <x:c r="A4" s="102" t="str">
         <x:v>Flow ID</x:v>
       </x:c>
-      <x:c r="B4" s="94" t="str">
+      <x:c r="B4" s="102" t="str">
         <x:v>Case</x:v>
       </x:c>
-      <x:c r="C4" s="94" t="str">
+      <x:c r="C4" s="102" t="str">
         <x:v>Subcase</x:v>
       </x:c>
-      <x:c r="D4" s="94" t="str">
+      <x:c r="D4" s="102" t="str">
         <x:v>進め方</x:v>
       </x:c>
-      <x:c r="E4" s="94" t="str">
+      <x:c r="E4" s="102" t="str">
         <x:v>Step</x:v>
       </x:c>
-      <x:c r="F4" s="94" t="str">
+      <x:c r="F4" s="102" t="str">
         <x:v>ユーザー行動</x:v>
       </x:c>
-      <x:c r="G4" s="94" t="str">
+      <x:c r="G4" s="102" t="str">
         <x:v>ユーザーへの説明</x:v>
       </x:c>
-      <x:c r="H4" s="94" t="str">
+      <x:c r="H4" s="102" t="str">
         <x:v>利用中Account</x:v>
       </x:c>
-      <x:c r="I4" s="94" t="str">
+      <x:c r="I4" s="102" t="str">
         <x:v>このStepの操作者</x:v>
       </x:c>
-      <x:c r="J4" s="94" t="str">
+      <x:c r="J4" s="102" t="str">
         <x:v>このStepで語る人</x:v>
       </x:c>
-      <x:c r="K4" s="94" t="str">
+      <x:c r="K4" s="102" t="str">
         <x:v>Person</x:v>
       </x:c>
-      <x:c r="L4" s="94" t="str">
+      <x:c r="L4" s="102" t="str">
         <x:v>Payer</x:v>
       </x:c>
-      <x:c r="M4" s="94" t="str">
+      <x:c r="M4" s="102" t="str">
         <x:v>Supporter</x:v>
       </x:c>
-      <x:c r="N4" s="94" t="str">
+      <x:c r="N4" s="102" t="str">
         <x:v>Device</x:v>
       </x:c>
-      <x:c r="O4" s="94" t="str">
+      <x:c r="O4" s="102" t="str">
         <x:v>現在状態</x:v>
       </x:c>
-      <x:c r="P4" s="94" t="str">
+      <x:c r="P4" s="102" t="str">
         <x:v>分岐条件</x:v>
       </x:c>
-      <x:c r="Q4" s="94" t="str">
+      <x:c r="Q4" s="102" t="str">
         <x:v>次の状態</x:v>
       </x:c>
-      <x:c r="R4" s="94" t="str">
+      <x:c r="R4" s="102" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="S4" s="94" t="str">
+      <x:c r="S4" s="102" t="str">
         <x:v>購入</x:v>
       </x:c>
-      <x:c r="T4" s="94" t="str">
+      <x:c r="T4" s="102" t="str">
         <x:v>本人認証</x:v>
       </x:c>
-      <x:c r="U4" s="94" t="str">
+      <x:c r="U4" s="102" t="str">
         <x:v>設定・同意</x:v>
       </x:c>
-      <x:c r="V4" s="94" t="str">
+      <x:c r="V4" s="102" t="str">
         <x:v>内容共有</x:v>
       </x:c>
-      <x:c r="W4" s="94" t="str">
+      <x:c r="W4" s="102" t="str">
         <x:v>進捗共有</x:v>
       </x:c>
-      <x:c r="X4" s="94" t="str">
+      <x:c r="X4" s="102" t="str">
         <x:v>内部メモ</x:v>
       </x:c>
-      <x:c r="Y4" s="94" t="str">
+      <x:c r="Y4" s="102" t="str">
         <x:v>確定度</x:v>
       </x:c>
     </x:row>
@@ -3549,6 +3609,9 @@
       <x:formula>$Y5="要確認"</x:formula>
     </x:cfRule>
     <x:cfRule type="expression" dxfId="21" priority="8">
+      <x:formula>$Y5="要確認"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="24" priority="9">
       <x:formula>$Y5="要確認"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -3629,40 +3692,40 @@
       <x:c r="L3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="94" t="str">
+      <x:c r="A4" s="102" t="str">
         <x:v>Setting ID</x:v>
       </x:c>
-      <x:c r="B4" s="94" t="str">
+      <x:c r="B4" s="102" t="str">
         <x:v>設定・同意</x:v>
       </x:c>
-      <x:c r="C4" s="94" t="str">
+      <x:c r="C4" s="102" t="str">
         <x:v>Account登録</x:v>
       </x:c>
-      <x:c r="D4" s="94" t="str">
+      <x:c r="D4" s="102" t="str">
         <x:v>対象Person作成</x:v>
       </x:c>
-      <x:c r="E4" s="94" t="str">
+      <x:c r="E4" s="102" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="F4" s="94" t="str">
+      <x:c r="F4" s="102" t="str">
         <x:v>購入</x:v>
       </x:c>
-      <x:c r="G4" s="94" t="str">
+      <x:c r="G4" s="102" t="str">
         <x:v>本人接続</x:v>
       </x:c>
-      <x:c r="H4" s="94" t="str">
+      <x:c r="H4" s="102" t="str">
         <x:v>本編開始</x:v>
       </x:c>
-      <x:c r="I4" s="94" t="str">
+      <x:c r="I4" s="102" t="str">
         <x:v>制作中</x:v>
       </x:c>
-      <x:c r="J4" s="94" t="str">
+      <x:c r="J4" s="102" t="str">
         <x:v>仕上げ</x:v>
       </x:c>
-      <x:c r="K4" s="94" t="str">
+      <x:c r="K4" s="102" t="str">
         <x:v>完成後</x:v>
       </x:c>
-      <x:c r="L4" s="94" t="str">
+      <x:c r="L4" s="102" t="str">
         <x:v>備考</x:v>
       </x:c>
     </x:row>
@@ -4119,7 +4182,7 @@
         <x:v>△</x:v>
       </x:c>
       <x:c r="L16" s="40" t="str">
-        <x:v>personal／professional。professionalは将来の施設・有料制作支援向け</x:v>
+        <x:v>personal／staff。staffは縦糸横糸スタッフによる制作サポート向け</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="44" customHeight="1">
@@ -4158,6 +4221,44 @@
       </x:c>
       <x:c r="L17" s="40" t="str">
         <x:v>本人／Supporter／双方を将来選択可能。現時点でUI追加不要</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="44" customHeight="1">
+      <x:c r="A18" s="40" t="str">
+        <x:v>S14</x:v>
+      </x:c>
+      <x:c r="B18" s="40" t="str">
+        <x:v>制作サポート希望受付</x:v>
+      </x:c>
+      <x:c r="C18" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D18" s="40" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E18" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="F18" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="G18" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="H18" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="I18" s="40" t="str">
+        <x:v>●</x:v>
+      </x:c>
+      <x:c r="J18" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="K18" s="40" t="str">
+        <x:v>△</x:v>
+      </x:c>
+      <x:c r="L18" s="40" t="str">
+        <x:v>希望受付のみ。運営が状況確認後に対応可否を判断し、申込時点では利用確定しない</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4222,31 +4323,31 @@
       <x:c r="I3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="94" t="str">
+      <x:c r="A4" s="102" t="str">
         <x:v>Case</x:v>
       </x:c>
-      <x:c r="B4" s="94" t="str">
+      <x:c r="B4" s="102" t="str">
         <x:v>位置づけ</x:v>
       </x:c>
-      <x:c r="C4" s="94" t="str">
+      <x:c r="C4" s="102" t="str">
         <x:v>HPに来た人</x:v>
       </x:c>
-      <x:c r="D4" s="94" t="str">
+      <x:c r="D4" s="102" t="str">
         <x:v>語る人</x:v>
       </x:c>
-      <x:c r="E4" s="94" t="str">
+      <x:c r="E4" s="102" t="str">
         <x:v>無料3問</x:v>
       </x:c>
-      <x:c r="F4" s="94" t="str">
+      <x:c r="F4" s="102" t="str">
         <x:v>同席・遠隔</x:v>
       </x:c>
-      <x:c r="G4" s="94" t="str">
+      <x:c r="G4" s="102" t="str">
         <x:v>購入者候補</x:v>
       </x:c>
-      <x:c r="H4" s="94" t="str">
+      <x:c r="H4" s="102" t="str">
         <x:v>本人Accountが必要になる時</x:v>
       </x:c>
-      <x:c r="I4" s="94" t="str">
+      <x:c r="I4" s="102" t="str">
         <x:v>要点</x:v>
       </x:c>
     </x:row>
@@ -4387,22 +4488,22 @@
       <x:c r="F3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="94" t="str">
+      <x:c r="A4" s="102" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B4" s="94" t="str">
+      <x:c r="B4" s="102" t="str">
         <x:v>論点</x:v>
       </x:c>
-      <x:c r="C4" s="94" t="str">
+      <x:c r="C4" s="102" t="str">
         <x:v>現状案</x:v>
       </x:c>
-      <x:c r="D4" s="94" t="str">
+      <x:c r="D4" s="102" t="str">
         <x:v>状態</x:v>
       </x:c>
-      <x:c r="E4" s="94" t="str">
+      <x:c r="E4" s="102" t="str">
         <x:v>決める理由</x:v>
       </x:c>
-      <x:c r="F4" s="94" t="str">
+      <x:c r="F4" s="102" t="str">
         <x:v>次アクション</x:v>
       </x:c>
     </x:row>
@@ -4651,7 +4752,7 @@
         <x:v>Q13</x:v>
       </x:c>
       <x:c r="B17" s="40" t="str">
-        <x:v>professional Supporterの業務管理</x:v>
+        <x:v>staff Supporterの業務管理</x:v>
       </x:c>
       <x:c r="C17" s="40" t="str">
         <x:v>担当期間、操作・閲覧ログ、担当終了時のアクセス停止を管理する</x:v>
@@ -4660,10 +4761,30 @@
         <x:v>要確認</x:v>
       </x:c>
       <x:c r="E17" s="40" t="str">
-        <x:v>施設スタッフや当社スタッフが扱う場合のプライバシーと運営責任を明確にする</x:v>
+        <x:v>当社スタッフが扱う場合のプライバシーと運営責任を明確にする</x:v>
       </x:c>
       <x:c r="F17" s="40" t="str">
-        <x:v>有料制作支援の実装前にDB・管理画面・監査要件を確定</x:v>
+        <x:v>試験提供前にDB・管理画面・監査要件を確定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="54" customHeight="1">
+      <x:c r="A18" s="40" t="str">
+        <x:v>Q14</x:v>
+      </x:c>
+      <x:c r="B18" s="40" t="str">
+        <x:v>制作サポートの試験提供</x:v>
+      </x:c>
+      <x:c r="C18" s="40" t="str">
+        <x:v>希望受付→状況確認→対応可否判断→staff Supporter設定。価格・回数・SLAは未確定</x:v>
+      </x:c>
+      <x:c r="D18" s="40" t="str">
+        <x:v>確定</x:v>
+      </x:c>
+      <x:c r="E18" s="40" t="str">
+        <x:v>提供保証を負わず少人数で工数と利用上のつまずきを観察する</x:v>
+      </x:c>
+      <x:c r="F18" s="40" t="str">
+        <x:v>希望受付、調整中、対応中、終了を記録し、必要時は受付停止</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4703,7 +4824,12 @@
       <x:formula>$D5="要確認"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="4">
+  <x:conditionalFormatting sqref="A5:F18">
+    <x:cfRule type="expression" dxfId="25" priority="9">
+      <x:formula>$D5="要確認"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="D5:D13">
       <x:formula1>"確定,要確認"</x:formula1>
     </x:dataValidation>
@@ -4714,6 +4840,9 @@
       <x:formula1>"確定,要確認"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D5:D17">
+      <x:formula1>"確定,要確認"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D5:D18">
       <x:formula1>"確定,要確認"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -4778,34 +4907,34 @@
       <x:c r="J3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="94" t="str">
+      <x:c r="A4" s="102" t="str">
         <x:v>Setting ID</x:v>
       </x:c>
-      <x:c r="B4" s="94" t="str">
+      <x:c r="B4" s="102" t="str">
         <x:v>設定・同意名</x:v>
       </x:c>
-      <x:c r="C4" s="94" t="str">
+      <x:c r="C4" s="102" t="str">
         <x:v>利用者が設定する画面</x:v>
       </x:c>
-      <x:c r="D4" s="94" t="str">
+      <x:c r="D4" s="102" t="str">
         <x:v>初期値</x:v>
       </x:c>
-      <x:c r="E4" s="94" t="str">
+      <x:c r="E4" s="102" t="str">
         <x:v>設定できる人</x:v>
       </x:c>
-      <x:c r="F4" s="94" t="str">
+      <x:c r="F4" s="102" t="str">
         <x:v>変更できる時期</x:v>
       </x:c>
-      <x:c r="G4" s="94" t="str">
+      <x:c r="G4" s="102" t="str">
         <x:v>保存先</x:v>
       </x:c>
-      <x:c r="H4" s="94" t="str">
+      <x:c r="H4" s="102" t="str">
         <x:v>関連Flow ID</x:v>
       </x:c>
-      <x:c r="I4" s="94" t="str">
+      <x:c r="I4" s="102" t="str">
         <x:v>実装状態</x:v>
       </x:c>
-      <x:c r="J4" s="94" t="str">
+      <x:c r="J4" s="102" t="str">
         <x:v>根拠仕様</x:v>
       </x:c>
     </x:row>
@@ -5172,10 +5301,10 @@
         <x:v>Supporter追加／運営管理</x:v>
       </x:c>
       <x:c r="D16" s="40" t="str">
-        <x:v>personal。professionalは将来拡張</x:v>
+        <x:v>personal。staffは試験提供時に運営が設定</x:v>
       </x:c>
       <x:c r="E16" s="40" t="str">
-        <x:v>本人、本人の了承を確認したSupporter、professionalは運営</x:v>
+        <x:v>本人、本人の了承を確認したSupporter、staffは運営</x:v>
       </x:c>
       <x:c r="F16" s="40" t="str">
         <x:v>Supporter追加時・業務担当変更時</x:v>
@@ -5230,31 +5359,63 @@
         <x:v>S14</x:v>
       </x:c>
       <x:c r="B18" s="40" t="str">
-        <x:v>業務Supporterアクセス管理</x:v>
+        <x:v>制作サポート希望受付</x:v>
       </x:c>
       <x:c r="C18" s="40" t="str">
-        <x:v>運営管理画面（将来）</x:v>
+        <x:v>制作サポート案内／希望送信</x:v>
       </x:c>
       <x:c r="D18" s="40" t="str">
-        <x:v>アクセスなし</x:v>
+        <x:v>未希望</x:v>
       </x:c>
       <x:c r="E18" s="40" t="str">
-        <x:v>権限ある運営者</x:v>
+        <x:v>本人または既存Supporter</x:v>
       </x:c>
       <x:c r="F18" s="40" t="str">
-        <x:v>担当開始・変更・終了時</x:v>
+        <x:v>無料体験後・購入後・制作中・仕上げ時</x:v>
       </x:c>
       <x:c r="G18" s="40" t="str">
-        <x:v>要確認（assignment期間、アクセスログ、失効）</x:v>
+        <x:v>要確認（support_request、status、requested_at等）</x:v>
       </x:c>
       <x:c r="H18" s="40" t="str">
-        <x:v>将来の施設・制作支援ケース</x:v>
+        <x:v>制作サポート試験提供</x:v>
       </x:c>
       <x:c r="I18" s="40" t="str">
         <x:v>未実装</x:v>
       </x:c>
       <x:c r="J18" s="40" t="str">
-        <x:v>04_運営チェック Q13／06_支援スタイル・権限</x:v>
+        <x:v>04_運営チェック Q14／06_支援スタイル・権限</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="74" customHeight="1">
+      <x:c r="A19" s="40" t="str">
+        <x:v>S15</x:v>
+      </x:c>
+      <x:c r="B19" s="40" t="str">
+        <x:v>staff Supporterアクセス管理</x:v>
+      </x:c>
+      <x:c r="C19" s="40" t="str">
+        <x:v>運営管理画面（試験提供）</x:v>
+      </x:c>
+      <x:c r="D19" s="40" t="str">
+        <x:v>アクセスなし</x:v>
+      </x:c>
+      <x:c r="E19" s="40" t="str">
+        <x:v>権限ある運営者</x:v>
+      </x:c>
+      <x:c r="F19" s="40" t="str">
+        <x:v>担当開始・変更・終了時</x:v>
+      </x:c>
+      <x:c r="G19" s="40" t="str">
+        <x:v>要確認（assignment期間、アクセスログ、失効）</x:v>
+      </x:c>
+      <x:c r="H19" s="40" t="str">
+        <x:v>制作サポート試験提供</x:v>
+      </x:c>
+      <x:c r="I19" s="40" t="str">
+        <x:v>未実装</x:v>
+      </x:c>
+      <x:c r="J19" s="40" t="str">
+        <x:v>04_運営チェック Q13・Q14／06_支援スタイル・権限</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5294,7 +5455,12 @@
       <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="4">
+  <x:conditionalFormatting sqref="A5:J19">
+    <x:cfRule type="expression" dxfId="26" priority="9">
+      <x:formula>OR($G5="要確認",$I5="要確認")</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="I5:I14">
       <x:formula1>"実装済み,一部実装,未実装,要確認"</x:formula1>
     </x:dataValidation>
@@ -5305,6 +5471,9 @@
       <x:formula1>"実装済み,一部実装,未実装,要確認"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I5:I18">
+      <x:formula1>"実装済み,一部実装,未実装,要確認"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I5:I19">
       <x:formula1>"実装済み,一部実装,未実装,要確認"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -5349,19 +5518,19 @@
       <x:c r="E3"/>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="94" t="str">
+      <x:c r="A4" s="102" t="str">
         <x:v>進め方（内部名）</x:v>
       </x:c>
-      <x:c r="B4" s="94" t="str">
+      <x:c r="B4" s="102" t="str">
         <x:v>中心となる端末・Account</x:v>
       </x:c>
-      <x:c r="C4" s="94" t="str">
+      <x:c r="C4" s="102" t="str">
         <x:v>Supporter</x:v>
       </x:c>
-      <x:c r="D4" s="94" t="str">
+      <x:c r="D4" s="102" t="str">
         <x:v>本人Account</x:v>
       </x:c>
-      <x:c r="E4" s="94" t="str">
+      <x:c r="E4" s="102" t="str">
         <x:v>ユーザー向け表現・説明候補</x:v>
       </x:c>
     </x:row>
@@ -5424,19 +5593,19 @@
       <x:c r="E8" s="41"/>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
-      <x:c r="A9" s="94" t="str">
+      <x:c r="A9" s="102" t="str">
         <x:v>関係</x:v>
       </x:c>
-      <x:c r="B9" s="94" t="str">
+      <x:c r="B9" s="102" t="str">
         <x:v>定義</x:v>
       </x:c>
-      <x:c r="C9" s="94" t="str">
+      <x:c r="C9" s="102" t="str">
         <x:v>アクセス範囲</x:v>
       </x:c>
-      <x:c r="D9" s="94" t="str">
+      <x:c r="D9" s="102" t="str">
         <x:v>主な役割</x:v>
       </x:c>
-      <x:c r="E9" s="94" t="str">
+      <x:c r="E9" s="102" t="str">
         <x:v>対象例</x:v>
       </x:c>
     </x:row>
@@ -5447,7 +5616,7 @@
       <x:c r="B10" s="40" t="str">
         <x:v>人生・作品の主人公であり、本人Accountから参加できる人</x:v>
       </x:c>
-      <x:c r="C10" s="98" t="str">
+      <x:c r="C10" s="106" t="str">
         <x:v>自分のPerson・Project</x:v>
       </x:c>
       <x:c r="D10" s="40" t="str">
@@ -5464,7 +5633,7 @@
       <x:c r="B11" s="40" t="str">
         <x:v>本人が信頼し、語り・作品づくりを手伝ってもらう制作メンバー</x:v>
       </x:c>
-      <x:c r="C11" s="98" t="str">
+      <x:c r="C11" s="106" t="str">
         <x:v>全語り、音声、写真、下書き、進捗、ブック制作など制作内部全体</x:v>
       </x:c>
       <x:c r="D11" s="40" t="str">
@@ -5481,7 +5650,7 @@
       <x:c r="B12" s="40" t="str">
         <x:v>本人またはSupporterが共有した内容を見る閲覧者</x:v>
       </x:c>
-      <x:c r="C12" s="98" t="str">
+      <x:c r="C12" s="106" t="str">
         <x:v>家族共有した語り、共有されたWebブック・完成作品のみ</x:v>
       </x:c>
       <x:c r="D12" s="40" t="str">
@@ -5498,7 +5667,7 @@
       <x:c r="B13" s="40" t="str">
         <x:v>料金を支払う人。制作・閲覧の権限とは独立</x:v>
       </x:c>
-      <x:c r="C13" s="98" t="str">
+      <x:c r="C13" s="106" t="str">
         <x:v>支払い・契約情報</x:v>
       </x:c>
       <x:c r="D13" s="40" t="str">
@@ -5516,19 +5685,19 @@
       <x:c r="E14" s="41"/>
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
-      <x:c r="A15" s="94" t="str">
+      <x:c r="A15" s="102" t="str">
         <x:v>Supporter種別</x:v>
       </x:c>
-      <x:c r="B15" s="94" t="str">
+      <x:c r="B15" s="102" t="str">
         <x:v>定義</x:v>
       </x:c>
-      <x:c r="C15" s="94" t="str">
+      <x:c r="C15" s="102" t="str">
         <x:v>アクセス</x:v>
       </x:c>
-      <x:c r="D15" s="94" t="str">
+      <x:c r="D15" s="102" t="str">
         <x:v>運営管理</x:v>
       </x:c>
-      <x:c r="E15" s="94" t="str">
+      <x:c r="E15" s="102" t="str">
         <x:v>対象例</x:v>
       </x:c>
     </x:row>
@@ -5539,10 +5708,10 @@
       <x:c r="B16" s="40" t="str">
         <x:v>本人が招待した個人Supporter</x:v>
       </x:c>
-      <x:c r="C16" s="98" t="str">
+      <x:c r="C16" s="106" t="str">
         <x:v>制作内部へフルアクセス</x:v>
       </x:c>
-      <x:c r="D16" s="98" t="str">
+      <x:c r="D16" s="106" t="str">
         <x:v>本人の了承、参加・停止を記録</x:v>
       </x:c>
       <x:c r="E16" s="40" t="str">
@@ -5551,19 +5720,19 @@
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
       <x:c r="A17" s="66" t="str">
-        <x:v>professional</x:v>
+        <x:v>staff</x:v>
       </x:c>
       <x:c r="B17" s="40" t="str">
-        <x:v>業務として制作を支援するSupporter（将来拡張）</x:v>
-      </x:c>
-      <x:c r="C17" s="98" t="str">
+        <x:v>縦糸横糸スタッフとして制作を支援するSupporter</x:v>
+      </x:c>
+      <x:c r="C17" s="106" t="str">
         <x:v>制作内部へフルアクセス</x:v>
       </x:c>
-      <x:c r="D17" s="98" t="str">
+      <x:c r="D17" s="106" t="str">
         <x:v>担当期間、操作・閲覧ログ、終了時のアクセス停止が必要</x:v>
       </x:c>
       <x:c r="E17" s="40" t="str">
-        <x:v>施設スタッフ、縦糸横糸スタッフ</x:v>
+        <x:v>縦糸横糸の制作サポート担当者</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
@@ -5574,69 +5743,113 @@
       <x:c r="E18" s="41"/>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
-      <x:c r="A19" s="94" t="str">
-        <x:v>独立して管理する項目</x:v>
-      </x:c>
-      <x:c r="B19" s="94" t="str">
-        <x:v>値・選択肢</x:v>
-      </x:c>
-      <x:c r="C19" s="94" t="str">
-        <x:v>進め方との関係</x:v>
-      </x:c>
-      <x:c r="D19" s="94" t="str">
-        <x:v>変更</x:v>
-      </x:c>
-      <x:c r="E19" s="94" t="str">
-        <x:v>補足</x:v>
+      <x:c r="A19" s="102" t="str">
+        <x:v>制作サポート試験提供</x:v>
+      </x:c>
+      <x:c r="B19" s="102" t="str">
+        <x:v>受付</x:v>
+      </x:c>
+      <x:c r="C19" s="102" t="str">
+        <x:v>提供判断</x:v>
+      </x:c>
+      <x:c r="D19" s="102" t="str">
+        <x:v>条件</x:v>
+      </x:c>
+      <x:c r="E19" s="102" t="str">
+        <x:v>検証</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
       <x:c r="A20" s="66" t="str">
-        <x:v>本人Account</x:v>
+        <x:v>位置づけ</x:v>
       </x:c>
       <x:c r="B20" s="40" t="str">
-        <x:v>あり／なし</x:v>
+        <x:v>『サポートを希望する』による希望受付</x:v>
       </x:c>
       <x:c r="C20" s="40" t="str">
-        <x:v>Supporter中心ではなしでも完結</x:v>
+        <x:v>運営が状況確認後に対応可否を判断。申込時点では利用確定しない</x:v>
       </x:c>
       <x:c r="D20" s="40" t="str">
-        <x:v>後から追加可</x:v>
+        <x:v>価格・回数・SLAは未確定。必要時は受付停止可</x:v>
       </x:c>
       <x:c r="E20" s="40" t="str">
-        <x:v>接続時に既存Person・Projectを新規作成しない</x:v>
+        <x:v>操作のつまずき、支援内容、工数を記録</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
       <x:c r="A21" s="66" t="str">
+        <x:v>状態</x:v>
+      </x:c>
+      <x:c r="B21" s="40" t="str">
+        <x:v>希望受付</x:v>
+      </x:c>
+      <x:c r="C21" s="40" t="str">
+        <x:v>調整中</x:v>
+      </x:c>
+      <x:c r="D21" s="40" t="str">
+        <x:v>対応中</x:v>
+      </x:c>
+      <x:c r="E21" s="40" t="str">
+        <x:v>終了</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="54" customHeight="1">
+      <x:c r="A22" s="41"/>
+      <x:c r="B22" s="41"/>
+      <x:c r="C22" s="41"/>
+      <x:c r="D22" s="41"/>
+      <x:c r="E22" s="41"/>
+    </x:row>
+    <x:row r="23" ht="54" customHeight="1">
+      <x:c r="A23" s="102" t="str">
+        <x:v>独立して管理する項目</x:v>
+      </x:c>
+      <x:c r="B23" s="102" t="str">
+        <x:v>値・選択肢</x:v>
+      </x:c>
+      <x:c r="C23" s="102" t="str">
+        <x:v>進め方との関係</x:v>
+      </x:c>
+      <x:c r="D23" s="102" t="str">
+        <x:v>変更</x:v>
+      </x:c>
+      <x:c r="E23" s="102" t="str">
+        <x:v>補足</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="54" customHeight="1">
+      <x:c r="A24" s="66" t="str">
+        <x:v>本人Account</x:v>
+      </x:c>
+      <x:c r="B24" s="40" t="str">
+        <x:v>あり／なし</x:v>
+      </x:c>
+      <x:c r="C24" s="40" t="str">
+        <x:v>Supporter中心ではなしでも完結</x:v>
+      </x:c>
+      <x:c r="D24" s="40" t="str">
+        <x:v>後から追加可</x:v>
+      </x:c>
+      <x:c r="E24" s="40" t="str">
+        <x:v>接続時に既存Person・Projectを新規作成しない</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="54" customHeight="1">
+      <x:c r="A25" s="66" t="str">
         <x:v>通知先</x:v>
       </x:c>
-      <x:c r="B21" s="40" t="str">
+      <x:c r="B25" s="40" t="str">
         <x:v>本人／Supporter／双方</x:v>
       </x:c>
-      <x:c r="C21" s="40" t="str">
+      <x:c r="C25" s="40" t="str">
         <x:v>進め方には固定しない</x:v>
       </x:c>
-      <x:c r="D21" s="40" t="str">
+      <x:c r="D25" s="40" t="str">
         <x:v>将来変更可</x:v>
       </x:c>
-      <x:c r="E21" s="40" t="str">
+      <x:c r="E25" s="40" t="str">
         <x:v>現時点ではUIを増やさず、将来設定可能な構造を前提とする</x:v>
       </x:c>
-    </x:row>
-    <x:row r="22" ht="48" customHeight="1">
-      <x:c r="A22"/>
-      <x:c r="B22"/>
-      <x:c r="C22"/>
-      <x:c r="D22"/>
-      <x:c r="E22"/>
-    </x:row>
-    <x:row r="23" ht="48" customHeight="1">
-      <x:c r="A23"/>
-      <x:c r="B23"/>
-      <x:c r="C23"/>
-      <x:c r="D23"/>
-      <x:c r="E23"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>